<commit_message>
Add a caspex rule from umut-PC
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -5211,7 +5211,7 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O62" t="inlineStr">
@@ -5293,7 +5293,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O63" t="inlineStr">
@@ -5375,7 +5375,7 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
@@ -5457,7 +5457,7 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
@@ -5539,7 +5539,7 @@
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O66" t="inlineStr">
@@ -5621,7 +5621,7 @@
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
@@ -11555,7 +11555,7 @@
       </c>
       <c r="N139" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O139" t="inlineStr">
@@ -11637,7 +11637,7 @@
       </c>
       <c r="N140" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O140" t="inlineStr">
@@ -11719,7 +11719,7 @@
       </c>
       <c r="N141" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O141" t="inlineStr">
@@ -11801,7 +11801,7 @@
       </c>
       <c r="N142" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O142" t="inlineStr">
@@ -16868,7 +16868,7 @@
       </c>
       <c r="N203" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O203" t="inlineStr">
@@ -16950,7 +16950,7 @@
       </c>
       <c r="N204" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O204" t="inlineStr">

</xml_diff>

<commit_message>
Mark a date Unknown from umut-PC
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -23252,9 +23252,9 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="J281" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">

</xml_diff>

<commit_message>
Edit Du145 from umut-PC
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -19577,9 +19577,9 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="J236" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
@@ -19654,9 +19654,9 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="J237" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -20059,9 +20059,9 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="J242" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
@@ -26793,9 +26793,9 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="J324" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
         </is>
       </c>
       <c r="K324" t="inlineStr">

</xml_diff>

<commit_message>
Handoff: received boxes from CAA
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -28393,14 +28393,34 @@
       </c>
     </row>
     <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t xml:space="preserve">From CAA</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t xml:space="preserve">From CAA</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CLAUDE BOX 1</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A1</t>
+        </is>
+      </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">hek caspex g8</t>
         </is>
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t xml:space="preserve">p23</t>
+          <t xml:space="preserve">P6</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
@@ -28410,12 +28430,12 @@
       </c>
       <c r="H344" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-07-31</t>
+          <t xml:space="preserve">2025-07-28</t>
         </is>
       </c>
       <c r="I344" t="inlineStr">
         <is>
-          <t xml:space="preserve">31-07-26</t>
+          <t xml:space="preserve">28-07-25</t>
         </is>
       </c>
       <c r="K344" t="inlineStr">
@@ -28425,193 +28445,253 @@
       </c>
       <c r="L344" t="inlineStr">
         <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="M344" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N344" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="O344" t="inlineStr">
+        <is>
+          <t xml:space="preserve">g8</t>
+        </is>
+      </c>
+      <c r="R344" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S344" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-emcm6az9</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">From CAA</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">From CAA</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CLAUDE BOX 1</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A2</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hek tox4 KO g8</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P5</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-07-28</t>
+        </is>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">28-07-25</t>
+        </is>
+      </c>
+      <c r="K345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="L345" t="inlineStr">
+        <is>
           <t xml:space="preserve">KO</t>
         </is>
       </c>
-      <c r="M344" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="N344" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="O344" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="R344" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S344" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-243</t>
-        </is>
-      </c>
-    </row>
-    <row r="345">
-      <c r="E345" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK gNT</t>
-        </is>
-      </c>
-      <c r="F345" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p18</t>
-        </is>
-      </c>
-      <c r="G345" t="inlineStr">
+      <c r="M345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">g8</t>
+        </is>
+      </c>
+      <c r="R345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-x8hm3iw7</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t xml:space="preserve">From CAA</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t xml:space="preserve">From CAA</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fff</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A1</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LNCAP</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p5</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H345" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-10</t>
-        </is>
-      </c>
-      <c r="I345" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10/8/2026</t>
-        </is>
-      </c>
-      <c r="K345" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="L345" t="inlineStr">
+      <c r="H346" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-07-28</t>
+        </is>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t xml:space="preserve">28-07-25</t>
+        </is>
+      </c>
+      <c r="K346" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="L346" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M345" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="N345" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="O345" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gNT</t>
-        </is>
-      </c>
-      <c r="R345" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S345" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-329</t>
-        </is>
-      </c>
-    </row>
-    <row r="346">
-      <c r="E346" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK ATF3 OX rep 3</t>
-        </is>
-      </c>
-      <c r="F346" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p26</t>
-        </is>
-      </c>
-      <c r="G346" t="inlineStr">
+      <c r="M346" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N346" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O346" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R346" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S346" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-zde7yyzi</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t xml:space="preserve">From CAA</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t xml:space="preserve">From CAA</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fff</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A2</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t xml:space="preserve">lncap caspex</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P6</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H346" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-10</t>
-        </is>
-      </c>
-      <c r="I346" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10/8/2026</t>
-        </is>
-      </c>
-      <c r="K346" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="L346" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OX</t>
-        </is>
-      </c>
-      <c r="M346" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="N346" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="O346" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="R346" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S346" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-330</t>
-        </is>
-      </c>
-    </row>
-    <row r="347">
-      <c r="E347" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
-        </is>
-      </c>
-      <c r="F347" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p18</t>
-        </is>
-      </c>
-      <c r="G347" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-10</t>
+          <t xml:space="preserve">2025-07-28</t>
         </is>
       </c>
       <c r="I347" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/8/2026</t>
+          <t xml:space="preserve">28-07-25</t>
         </is>
       </c>
       <c r="K347" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L347" t="inlineStr">
         <is>
-          <t xml:space="preserve">3xFLAG</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M347" t="inlineStr">
@@ -28621,7 +28701,7 @@
       </c>
       <c r="N347" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O347" t="inlineStr">
@@ -28631,24 +28711,24 @@
       </c>
       <c r="R347" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">stored</t>
         </is>
       </c>
       <c r="S347" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-331</t>
+          <t xml:space="preserve">v-rb9gprqv</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="E348" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F348" t="inlineStr">
         <is>
-          <t xml:space="preserve">p15</t>
+          <t xml:space="preserve">p23</t>
         </is>
       </c>
       <c r="G348" t="inlineStr">
@@ -28658,22 +28738,22 @@
       </c>
       <c r="H348" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-10</t>
+          <t xml:space="preserve">2026-07-31</t>
         </is>
       </c>
       <c r="I348" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/8/2026</t>
+          <t xml:space="preserve">31-07-26</t>
         </is>
       </c>
       <c r="K348" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L348" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M348" t="inlineStr">
@@ -28688,7 +28768,7 @@
       </c>
       <c r="O348" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R348" t="inlineStr">
@@ -28698,19 +28778,19 @@
       </c>
       <c r="S348" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-355</t>
+          <t xml:space="preserve">v-243</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="E349" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 KO rep 3</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F349" t="inlineStr">
         <is>
-          <t xml:space="preserve">p16</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G349" t="inlineStr">
@@ -28730,12 +28810,12 @@
       </c>
       <c r="K349" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L349" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M349" t="inlineStr">
@@ -28750,7 +28830,7 @@
       </c>
       <c r="O349" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R349" t="inlineStr">
@@ -28760,19 +28840,19 @@
       </c>
       <c r="S349" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-356</t>
+          <t xml:space="preserve">v-329</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="E350" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 OX rep 3</t>
+          <t xml:space="preserve">HEK ATF3 OX rep 3</t>
         </is>
       </c>
       <c r="F350" t="inlineStr">
         <is>
-          <t xml:space="preserve">p16</t>
+          <t xml:space="preserve">p26</t>
         </is>
       </c>
       <c r="G350" t="inlineStr">
@@ -28792,7 +28872,7 @@
       </c>
       <c r="K350" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L350" t="inlineStr">
@@ -28822,67 +28902,315 @@
       </c>
       <c r="S350" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-357</t>
+          <t xml:space="preserve">v-330</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="E351" t="inlineStr">
         <is>
+          <t xml:space="preserve">HEK 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-10</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/8/2026</t>
+        </is>
+      </c>
+      <c r="K351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="L351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3xFLAG</t>
+        </is>
+      </c>
+      <c r="M351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-331</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="E352" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 gNT</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p15</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-10</t>
+        </is>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/8/2026</t>
+        </is>
+      </c>
+      <c r="K352" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L352" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M352" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N352" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O352" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gNT</t>
+        </is>
+      </c>
+      <c r="R352" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S352" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-355</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="E353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 KO rep 3</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p16</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-10</t>
+        </is>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/8/2026</t>
+        </is>
+      </c>
+      <c r="K353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KO</t>
+        </is>
+      </c>
+      <c r="M353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-356</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="E354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 OX rep 3</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p16</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-10</t>
+        </is>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/8/2026</t>
+        </is>
+      </c>
+      <c r="K354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OX</t>
+        </is>
+      </c>
+      <c r="M354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-357</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="E355" t="inlineStr">
+        <is>
           <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
-      <c r="F351" t="inlineStr">
+      <c r="F355" t="inlineStr">
         <is>
           <t xml:space="preserve">p15</t>
         </is>
       </c>
-      <c r="G351" t="inlineStr">
+      <c r="G355" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H351" t="inlineStr">
+      <c r="H355" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-08-10</t>
         </is>
       </c>
-      <c r="I351" t="inlineStr">
+      <c r="I355" t="inlineStr">
         <is>
           <t xml:space="preserve">10/8/2026</t>
         </is>
       </c>
-      <c r="K351" t="inlineStr">
+      <c r="K355" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L351" t="inlineStr">
+      <c r="L355" t="inlineStr">
         <is>
           <t xml:space="preserve">3xFLAG</t>
         </is>
       </c>
-      <c r="M351" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="N351" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="O351" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="R351" t="inlineStr">
+      <c r="M355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R355" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
-      <c r="S351" t="inlineStr">
+      <c r="S355" t="inlineStr">
         <is>
           <t xml:space="preserve">v-358</t>
         </is>
@@ -32724,22 +33052,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCAP BMK</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">LNCAP</t>
         </is>
       </c>
       <c r="E126">
@@ -32755,7 +33068,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap (m3) no sort</t>
+          <t xml:space="preserve">LNCAP BMK</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -32786,7 +33099,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G2</t>
+          <t xml:space="preserve">LnCap (m3) no sort</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -32817,7 +33130,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G3</t>
+          <t xml:space="preserve">LnCap Canada V1G2</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -32848,7 +33161,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G4</t>
+          <t xml:space="preserve">LnCap Canada V1G3</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -32879,7 +33192,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap ER</t>
+          <t xml:space="preserve">LnCap Canada V1G4</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -32910,7 +33223,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap V1G1</t>
+          <t xml:space="preserve">LnCap ER</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -32941,7 +33254,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap478 #2 98%</t>
+          <t xml:space="preserve">LnCap V1G1</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -32972,7 +33285,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select</t>
+          <t xml:space="preserve">LnCap478 #2 98%</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -32982,7 +33295,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -33003,7 +33316,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select C</t>
+          <t xml:space="preserve">LnCapCASPEX no select</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -33034,17 +33347,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap (m1) no sort</t>
+          <t xml:space="preserve">LnCapCASPEX no select C</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -33065,12 +33378,12 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDA-MB g1.1 p10</t>
+          <t xml:space="preserve">LuCap (m1) no sort</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDA-MB-231</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -33080,7 +33393,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E137">
@@ -33096,7 +33409,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDA-MB gNT</t>
+          <t xml:space="preserve">MDA-MB g1.1 p10</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -33111,7 +33424,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g1.1</t>
         </is>
       </c>
       <c r="E138">
@@ -33127,124 +33440,203 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">MDA-MB gNT</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">MDA-MB-231</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E139">
+        <v>1</v>
+      </c>
+      <c r="F139">
         <v>0</v>
       </c>
-      <c r="F139">
+      <c r="G139">
         <v>1</v>
-      </c>
-      <c r="G139">
-        <v>0</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep 3</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OX</t>
-        </is>
-      </c>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">hek caspex g8</t>
         </is>
       </c>
       <c r="E140">
+        <v>1</v>
+      </c>
+      <c r="F140">
         <v>0</v>
       </c>
-      <c r="F140">
+      <c r="G140">
         <v>1</v>
-      </c>
-      <c r="G140">
-        <v>0</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 KO rep 3</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t xml:space="preserve">KO</t>
-        </is>
-      </c>
-      <c r="D141" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">hek tox4 KO g8</t>
         </is>
       </c>
       <c r="E141">
+        <v>1</v>
+      </c>
+      <c r="F141">
         <v>0</v>
       </c>
-      <c r="F141">
+      <c r="G141">
         <v>1</v>
-      </c>
-      <c r="G141">
-        <v>0</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
+          <t xml:space="preserve">lncap caspex</t>
+        </is>
+      </c>
+      <c r="E142">
+        <v>1</v>
+      </c>
+      <c r="F142">
+        <v>0</v>
+      </c>
+      <c r="G142">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KO</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="E143">
+        <v>0</v>
+      </c>
+      <c r="F143">
+        <v>1</v>
+      </c>
+      <c r="G143">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK ATF3 OX rep 3</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OX</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="E144">
+        <v>0</v>
+      </c>
+      <c r="F144">
+        <v>1</v>
+      </c>
+      <c r="G144">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 KO rep 3</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KO</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="E145">
+        <v>0</v>
+      </c>
+      <c r="F145">
+        <v>1</v>
+      </c>
+      <c r="G145">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
           <t xml:space="preserve">Huh7 OX rep 3</t>
         </is>
       </c>
-      <c r="B142" t="inlineStr">
+      <c r="B146" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="C142" t="inlineStr">
+      <c r="C146" t="inlineStr">
         <is>
           <t xml:space="preserve">OX</t>
         </is>
       </c>
-      <c r="D142" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="E142">
+      <c r="D146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="E146">
         <v>0</v>
       </c>
-      <c r="F142">
+      <c r="F146">
         <v>1</v>
       </c>
-      <c r="G142">
+      <c r="G146">
         <v>0</v>
       </c>
     </row>
@@ -34078,6 +34470,90 @@
         <v>81</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">From CAA</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">freezer</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">From CAA</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CLAUDE BOX 1</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">grid</t>
+        </is>
+      </c>
+      <c r="F10">
+        <v>9</v>
+      </c>
+      <c r="G10">
+        <v>9</v>
+      </c>
+      <c r="H10">
+        <v>81</v>
+      </c>
+      <c r="I10">
+        <v>2</v>
+      </c>
+      <c r="J10">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">From CAA</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">freezer</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">From CAA</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fff</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">grid</t>
+        </is>
+      </c>
+      <c r="F11">
+        <v>9</v>
+      </c>
+      <c r="G11">
+        <v>9</v>
+      </c>
+      <c r="H11">
+        <v>81</v>
+      </c>
+      <c r="I11">
+        <v>2</v>
+      </c>
+      <c r="J11">
+        <v>79</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add a resistance rule from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -5124,7 +5124,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -11140,7 +11140,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N134" t="inlineStr">
@@ -11304,7 +11304,7 @@
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N136" t="inlineStr">
@@ -11386,7 +11386,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N137" t="inlineStr">
@@ -11468,7 +11468,7 @@
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N138" t="inlineStr">
@@ -13287,7 +13287,7 @@
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t xml:space="preserve">50CR</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N160" t="inlineStr">
@@ -13379,7 +13379,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t xml:space="preserve">50CR</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
@@ -13625,7 +13625,7 @@
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t xml:space="preserve">50CR</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N164" t="inlineStr">
@@ -13707,7 +13707,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t xml:space="preserve">50CR</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
@@ -13789,7 +13789,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t xml:space="preserve">50CR</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -13871,7 +13871,7 @@
       </c>
       <c r="M167" t="inlineStr">
         <is>
-          <t xml:space="preserve">50CR</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N167" t="inlineStr">
@@ -13953,7 +13953,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t xml:space="preserve">50CR</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -14035,7 +14035,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t xml:space="preserve">50CR</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -15633,7 +15633,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t xml:space="preserve">50CR</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -15715,7 +15715,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t xml:space="preserve">50CR</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -15797,7 +15797,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t xml:space="preserve">50CR</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">
@@ -15879,7 +15879,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t xml:space="preserve">50CR</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
@@ -15961,7 +15961,7 @@
       </c>
       <c r="M192" t="inlineStr">
         <is>
-          <t xml:space="preserve">50CR</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N192" t="inlineStr">
@@ -16043,7 +16043,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t xml:space="preserve">50CR</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
@@ -16125,7 +16125,7 @@
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t xml:space="preserve">50CR</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N194" t="inlineStr">
@@ -16371,7 +16371,7 @@
       </c>
       <c r="M197" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N197" t="inlineStr">
@@ -16453,7 +16453,7 @@
       </c>
       <c r="M198" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N198" t="inlineStr">
@@ -16535,7 +16535,7 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
@@ -16617,7 +16617,7 @@
       </c>
       <c r="M200" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N200" t="inlineStr">
@@ -16699,7 +16699,7 @@
       </c>
       <c r="M201" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N201" t="inlineStr">
@@ -16781,7 +16781,7 @@
       </c>
       <c r="M202" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N202" t="inlineStr">
@@ -17027,7 +17027,7 @@
       </c>
       <c r="M205" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N205" t="inlineStr">
@@ -28286,7 +28286,7 @@
       </c>
       <c r="M342" t="inlineStr">
         <is>
-          <t xml:space="preserve">50CR</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N342" t="inlineStr">
@@ -28393,34 +28393,14 @@
       </c>
     </row>
     <row r="344">
-      <c r="A344" t="inlineStr">
-        <is>
-          <t xml:space="preserve">From CAA</t>
-        </is>
-      </c>
-      <c r="B344" t="inlineStr">
-        <is>
-          <t xml:space="preserve">From CAA</t>
-        </is>
-      </c>
-      <c r="C344" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CLAUDE BOX 1</t>
-        </is>
-      </c>
-      <c r="D344" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A1</t>
-        </is>
-      </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t xml:space="preserve">hek caspex g8</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t xml:space="preserve">P6</t>
+          <t xml:space="preserve">p23</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
@@ -28430,12 +28410,12 @@
       </c>
       <c r="H344" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-07-28</t>
+          <t xml:space="preserve">2026-07-31</t>
         </is>
       </c>
       <c r="I344" t="inlineStr">
         <is>
-          <t xml:space="preserve">28-07-25</t>
+          <t xml:space="preserve">31-07-26</t>
         </is>
       </c>
       <c r="K344" t="inlineStr">
@@ -28445,7 +28425,7 @@
       </c>
       <c r="L344" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M344" t="inlineStr">
@@ -28455,54 +28435,34 @@
       </c>
       <c r="N344" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O344" t="inlineStr">
         <is>
-          <t xml:space="preserve">g8</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R344" t="inlineStr">
         <is>
-          <t xml:space="preserve">stored</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="S344" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-emcm6az9</t>
+          <t xml:space="preserve">v-243</t>
         </is>
       </c>
     </row>
     <row r="345">
-      <c r="A345" t="inlineStr">
-        <is>
-          <t xml:space="preserve">From CAA</t>
-        </is>
-      </c>
-      <c r="B345" t="inlineStr">
-        <is>
-          <t xml:space="preserve">From CAA</t>
-        </is>
-      </c>
-      <c r="C345" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CLAUDE BOX 1</t>
-        </is>
-      </c>
-      <c r="D345" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A2</t>
-        </is>
-      </c>
       <c r="E345" t="inlineStr">
         <is>
-          <t xml:space="preserve">hek tox4 KO g8</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F345" t="inlineStr">
         <is>
-          <t xml:space="preserve">P5</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G345" t="inlineStr">
@@ -28512,12 +28472,12 @@
       </c>
       <c r="H345" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-07-28</t>
+          <t xml:space="preserve">2026-08-10</t>
         </is>
       </c>
       <c r="I345" t="inlineStr">
         <is>
-          <t xml:space="preserve">28-07-25</t>
+          <t xml:space="preserve">10/8/2026</t>
         </is>
       </c>
       <c r="K345" t="inlineStr">
@@ -28527,7 +28487,7 @@
       </c>
       <c r="L345" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M345" t="inlineStr">
@@ -28542,49 +28502,29 @@
       </c>
       <c r="O345" t="inlineStr">
         <is>
-          <t xml:space="preserve">g8</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R345" t="inlineStr">
         <is>
-          <t xml:space="preserve">stored</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="S345" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-x8hm3iw7</t>
+          <t xml:space="preserve">v-329</t>
         </is>
       </c>
     </row>
     <row r="346">
-      <c r="A346" t="inlineStr">
-        <is>
-          <t xml:space="preserve">From CAA</t>
-        </is>
-      </c>
-      <c r="B346" t="inlineStr">
-        <is>
-          <t xml:space="preserve">From CAA</t>
-        </is>
-      </c>
-      <c r="C346" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fff</t>
-        </is>
-      </c>
-      <c r="D346" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A1</t>
-        </is>
-      </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCAP</t>
+          <t xml:space="preserve">HEK ATF3 OX rep 3</t>
         </is>
       </c>
       <c r="F346" t="inlineStr">
         <is>
-          <t xml:space="preserve">p5</t>
+          <t xml:space="preserve">p26</t>
         </is>
       </c>
       <c r="G346" t="inlineStr">
@@ -28594,22 +28534,22 @@
       </c>
       <c r="H346" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-07-28</t>
+          <t xml:space="preserve">2026-08-10</t>
         </is>
       </c>
       <c r="I346" t="inlineStr">
         <is>
-          <t xml:space="preserve">28-07-25</t>
+          <t xml:space="preserve">10/8/2026</t>
         </is>
       </c>
       <c r="K346" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L346" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M346" t="inlineStr">
@@ -28629,44 +28569,24 @@
       </c>
       <c r="R346" t="inlineStr">
         <is>
-          <t xml:space="preserve">stored</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="S346" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-zde7yyzi</t>
+          <t xml:space="preserve">v-330</t>
         </is>
       </c>
     </row>
     <row r="347">
-      <c r="A347" t="inlineStr">
-        <is>
-          <t xml:space="preserve">From CAA</t>
-        </is>
-      </c>
-      <c r="B347" t="inlineStr">
-        <is>
-          <t xml:space="preserve">From CAA</t>
-        </is>
-      </c>
-      <c r="C347" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fff</t>
-        </is>
-      </c>
-      <c r="D347" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A2</t>
-        </is>
-      </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t xml:space="preserve">lncap caspex</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t xml:space="preserve">P6</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
@@ -28676,22 +28596,22 @@
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-07-28</t>
+          <t xml:space="preserve">2026-08-10</t>
         </is>
       </c>
       <c r="I347" t="inlineStr">
         <is>
-          <t xml:space="preserve">28-07-25</t>
+          <t xml:space="preserve">10/8/2026</t>
         </is>
       </c>
       <c r="K347" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L347" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">3xFLAG</t>
         </is>
       </c>
       <c r="M347" t="inlineStr">
@@ -28701,7 +28621,7 @@
       </c>
       <c r="N347" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O347" t="inlineStr">
@@ -28711,24 +28631,24 @@
       </c>
       <c r="R347" t="inlineStr">
         <is>
-          <t xml:space="preserve">stored</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="S347" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-rb9gprqv</t>
+          <t xml:space="preserve">v-331</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="E348" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="F348" t="inlineStr">
         <is>
-          <t xml:space="preserve">p23</t>
+          <t xml:space="preserve">p15</t>
         </is>
       </c>
       <c r="G348" t="inlineStr">
@@ -28738,22 +28658,22 @@
       </c>
       <c r="H348" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-07-31</t>
+          <t xml:space="preserve">2026-08-10</t>
         </is>
       </c>
       <c r="I348" t="inlineStr">
         <is>
-          <t xml:space="preserve">31-07-26</t>
+          <t xml:space="preserve">10/8/2026</t>
         </is>
       </c>
       <c r="K348" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L348" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M348" t="inlineStr">
@@ -28768,7 +28688,7 @@
       </c>
       <c r="O348" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R348" t="inlineStr">
@@ -28778,19 +28698,19 @@
       </c>
       <c r="S348" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-243</t>
+          <t xml:space="preserve">v-355</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="E349" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">Huh7 KO rep 3</t>
         </is>
       </c>
       <c r="F349" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p16</t>
         </is>
       </c>
       <c r="G349" t="inlineStr">
@@ -28810,12 +28730,12 @@
       </c>
       <c r="K349" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L349" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M349" t="inlineStr">
@@ -28830,7 +28750,7 @@
       </c>
       <c r="O349" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R349" t="inlineStr">
@@ -28840,19 +28760,19 @@
       </c>
       <c r="S349" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-329</t>
+          <t xml:space="preserve">v-356</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="E350" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep 3</t>
+          <t xml:space="preserve">Huh7 OX rep 3</t>
         </is>
       </c>
       <c r="F350" t="inlineStr">
         <is>
-          <t xml:space="preserve">p26</t>
+          <t xml:space="preserve">p16</t>
         </is>
       </c>
       <c r="G350" t="inlineStr">
@@ -28872,7 +28792,7 @@
       </c>
       <c r="K350" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L350" t="inlineStr">
@@ -28902,19 +28822,19 @@
       </c>
       <c r="S350" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-330</t>
+          <t xml:space="preserve">v-357</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="E351" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="F351" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p15</t>
         </is>
       </c>
       <c r="G351" t="inlineStr">
@@ -28934,7 +28854,7 @@
       </c>
       <c r="K351" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L351" t="inlineStr">
@@ -28963,254 +28883,6 @@
         </is>
       </c>
       <c r="S351" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-331</t>
-        </is>
-      </c>
-    </row>
-    <row r="352">
-      <c r="E352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7 gNT</t>
-        </is>
-      </c>
-      <c r="F352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p15</t>
-        </is>
-      </c>
-      <c r="G352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-10</t>
-        </is>
-      </c>
-      <c r="I352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10/8/2026</t>
-        </is>
-      </c>
-      <c r="K352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
-        </is>
-      </c>
-      <c r="L352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="N352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="O352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gNT</t>
-        </is>
-      </c>
-      <c r="R352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-355</t>
-        </is>
-      </c>
-    </row>
-    <row r="353">
-      <c r="E353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7 KO rep 3</t>
-        </is>
-      </c>
-      <c r="F353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p16</t>
-        </is>
-      </c>
-      <c r="G353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-10</t>
-        </is>
-      </c>
-      <c r="I353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10/8/2026</t>
-        </is>
-      </c>
-      <c r="K353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
-        </is>
-      </c>
-      <c r="L353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">KO</t>
-        </is>
-      </c>
-      <c r="M353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="N353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="O353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="R353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-356</t>
-        </is>
-      </c>
-    </row>
-    <row r="354">
-      <c r="E354" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7 OX rep 3</t>
-        </is>
-      </c>
-      <c r="F354" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p16</t>
-        </is>
-      </c>
-      <c r="G354" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H354" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-10</t>
-        </is>
-      </c>
-      <c r="I354" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10/8/2026</t>
-        </is>
-      </c>
-      <c r="K354" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
-        </is>
-      </c>
-      <c r="L354" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OX</t>
-        </is>
-      </c>
-      <c r="M354" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="N354" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="O354" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="R354" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S354" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-357</t>
-        </is>
-      </c>
-    </row>
-    <row r="355">
-      <c r="E355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
-        </is>
-      </c>
-      <c r="F355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p15</t>
-        </is>
-      </c>
-      <c r="G355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-10</t>
-        </is>
-      </c>
-      <c r="I355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10/8/2026</t>
-        </is>
-      </c>
-      <c r="K355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
-        </is>
-      </c>
-      <c r="L355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3xFLAG</t>
-        </is>
-      </c>
-      <c r="M355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="N355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="O355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="R355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S355" t="inlineStr">
         <is>
           <t xml:space="preserve">v-358</t>
         </is>
@@ -33052,7 +32724,22 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCAP</t>
+          <t xml:space="preserve">LNCAP BMK</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E126">
@@ -33068,7 +32755,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCAP BMK</t>
+          <t xml:space="preserve">LnCap (m3) no sort</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -33099,7 +32786,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap (m3) no sort</t>
+          <t xml:space="preserve">LnCap Canada V1G2</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -33130,7 +32817,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G2</t>
+          <t xml:space="preserve">LnCap Canada V1G3</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -33161,7 +32848,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G3</t>
+          <t xml:space="preserve">LnCap Canada V1G4</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -33192,7 +32879,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G4</t>
+          <t xml:space="preserve">LnCap ER</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -33223,7 +32910,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap ER</t>
+          <t xml:space="preserve">LnCap V1G1</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -33254,7 +32941,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap V1G1</t>
+          <t xml:space="preserve">LnCap478 #2 98%</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -33285,7 +32972,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap478 #2 98%</t>
+          <t xml:space="preserve">LnCapCASPEX no select</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -33295,7 +32982,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -33316,7 +33003,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select</t>
+          <t xml:space="preserve">LnCapCASPEX no select C</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -33347,17 +33034,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select C</t>
+          <t xml:space="preserve">LuCap (m1) no sort</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -33378,12 +33065,12 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap (m1) no sort</t>
+          <t xml:space="preserve">MDA-MB g1.1 p10</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">MDA-MB-231</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -33393,7 +33080,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1.1</t>
         </is>
       </c>
       <c r="E137">
@@ -33409,7 +33096,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDA-MB g1.1 p10</t>
+          <t xml:space="preserve">MDA-MB gNT</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -33424,7 +33111,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.1</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E138">
@@ -33440,203 +33127,124 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDA-MB gNT</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDA-MB-231</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E139">
+        <v>0</v>
+      </c>
+      <c r="F139">
         <v>1</v>
       </c>
-      <c r="F139">
+      <c r="G139">
         <v>0</v>
-      </c>
-      <c r="G139">
-        <v>1</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">hek caspex g8</t>
+          <t xml:space="preserve">HEK ATF3 OX rep 3</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OX</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E140">
+        <v>0</v>
+      </c>
+      <c r="F140">
         <v>1</v>
       </c>
-      <c r="F140">
+      <c r="G140">
         <v>0</v>
-      </c>
-      <c r="G140">
-        <v>1</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">hek tox4 KO g8</t>
+          <t xml:space="preserve">Huh7 KO rep 3</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KO</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E141">
+        <v>0</v>
+      </c>
+      <c r="F141">
         <v>1</v>
       </c>
-      <c r="F141">
+      <c r="G141">
         <v>0</v>
-      </c>
-      <c r="G141">
-        <v>1</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">lncap caspex</t>
+          <t xml:space="preserve">Huh7 OX rep 3</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OX</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E142">
+        <v>0</v>
+      </c>
+      <c r="F142">
         <v>1</v>
       </c>
-      <c r="F142">
-        <v>0</v>
-      </c>
       <c r="G142">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t xml:space="preserve">KO</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="E143">
-        <v>0</v>
-      </c>
-      <c r="F143">
-        <v>1</v>
-      </c>
-      <c r="G143">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK ATF3 OX rep 3</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OX</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="E144">
-        <v>0</v>
-      </c>
-      <c r="F144">
-        <v>1</v>
-      </c>
-      <c r="G144">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7 KO rep 3</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t xml:space="preserve">KO</t>
-        </is>
-      </c>
-      <c r="D145" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="E145">
-        <v>0</v>
-      </c>
-      <c r="F145">
-        <v>1</v>
-      </c>
-      <c r="G145">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7 OX rep 3</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OX</t>
-        </is>
-      </c>
-      <c r="D146" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="E146">
-        <v>0</v>
-      </c>
-      <c r="F146">
-        <v>1</v>
-      </c>
-      <c r="G146">
         <v>0</v>
       </c>
     </row>
@@ -34470,90 +34078,6 @@
         <v>81</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">From CAA</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">freezer</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">From CAA</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CLAUDE BOX 1</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">grid</t>
-        </is>
-      </c>
-      <c r="F10">
-        <v>9</v>
-      </c>
-      <c r="G10">
-        <v>9</v>
-      </c>
-      <c r="H10">
-        <v>81</v>
-      </c>
-      <c r="I10">
-        <v>2</v>
-      </c>
-      <c r="J10">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">From CAA</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">freezer</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">From CAA</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fff</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">grid</t>
-        </is>
-      </c>
-      <c r="F11">
-        <v>9</v>
-      </c>
-      <c r="G11">
-        <v>9</v>
-      </c>
-      <c r="H11">
-        <v>81</v>
-      </c>
-      <c r="I11">
-        <v>2</v>
-      </c>
-      <c r="J11">
-        <v>79</v>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Confirm 128 dates from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -184,14 +184,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-05</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t xml:space="preserve">5/5/2025</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -266,14 +266,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-05</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t xml:space="preserve">5/5/2025</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -348,14 +348,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-05</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t xml:space="preserve">5/5/2025</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -430,14 +430,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-05</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t xml:space="preserve">5/5/2025</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -512,14 +512,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-04-09</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t xml:space="preserve">9/4/2026</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -594,14 +594,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-04-09</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t xml:space="preserve">9/4/2026</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -840,14 +840,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-10</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t xml:space="preserve">10/2/2026</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1578,14 +1578,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-08</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t xml:space="preserve">8/5/2025</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1660,14 +1660,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-08</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t xml:space="preserve">8/5/2025</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1742,14 +1742,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-08</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t xml:space="preserve">8/5/2025</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1824,14 +1824,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-08</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
           <t xml:space="preserve">8/5/2025</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1906,14 +1906,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-07</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t xml:space="preserve">7/5/2025</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1988,14 +1988,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-07</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t xml:space="preserve">7/5/2025</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2070,14 +2070,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-07</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t xml:space="preserve">7/5/2025</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -3176,14 +3176,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-02-03</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t xml:space="preserve">3/2/2023</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3340,14 +3340,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-02</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t xml:space="preserve">2/5/2025</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3750,14 +3750,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-06</t>
+        </is>
+      </c>
       <c r="I45" t="inlineStr">
         <is>
           <t xml:space="preserve">6/2/2026</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3914,14 +3914,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-05</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr">
         <is>
           <t xml:space="preserve">5/2/2026</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3996,14 +3996,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-02</t>
+        </is>
+      </c>
       <c r="I48" t="inlineStr">
         <is>
           <t xml:space="preserve">2/2/2026</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -4160,14 +4160,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-02</t>
+        </is>
+      </c>
       <c r="I50" t="inlineStr">
         <is>
           <t xml:space="preserve">2/2/2026</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -4324,14 +4324,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-03</t>
+        </is>
+      </c>
       <c r="I52" t="inlineStr">
         <is>
           <t xml:space="preserve">3/3/2026</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -4406,14 +4406,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-03</t>
+        </is>
+      </c>
       <c r="I53" t="inlineStr">
         <is>
           <t xml:space="preserve">3/3/2026</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -5686,14 +5686,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-02</t>
+        </is>
+      </c>
       <c r="I68" t="inlineStr">
         <is>
           <t xml:space="preserve">2/2/2026</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -5850,14 +5850,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-02</t>
+        </is>
+      </c>
       <c r="I70" t="inlineStr">
         <is>
           <t xml:space="preserve">2/2/2026</t>
-        </is>
-      </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -6096,14 +6096,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-04-10</t>
+        </is>
+      </c>
       <c r="I73" t="inlineStr">
         <is>
           <t xml:space="preserve">10/4/2026</t>
-        </is>
-      </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -6178,14 +6178,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-04-10</t>
+        </is>
+      </c>
       <c r="I74" t="inlineStr">
         <is>
           <t xml:space="preserve">10/4/2026</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -6752,14 +6752,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-10</t>
+        </is>
+      </c>
       <c r="I81" t="inlineStr">
         <is>
           <t xml:space="preserve">10/3/2026</t>
-        </is>
-      </c>
-      <c r="J81" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -6834,14 +6834,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-11</t>
+        </is>
+      </c>
       <c r="I82" t="inlineStr">
         <is>
           <t xml:space="preserve">11/3/2026</t>
-        </is>
-      </c>
-      <c r="J82" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -6916,14 +6916,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-11</t>
+        </is>
+      </c>
       <c r="I83" t="inlineStr">
         <is>
           <t xml:space="preserve">11/3/2026</t>
-        </is>
-      </c>
-      <c r="J83" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -6998,14 +6998,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-10</t>
+        </is>
+      </c>
       <c r="I84" t="inlineStr">
         <is>
           <t xml:space="preserve">10/3/2026</t>
-        </is>
-      </c>
-      <c r="J84" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -7162,14 +7162,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-07-07</t>
+        </is>
+      </c>
       <c r="I86" t="inlineStr">
         <is>
           <t xml:space="preserve">7/7/2025</t>
-        </is>
-      </c>
-      <c r="J86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -7254,14 +7254,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-09</t>
+        </is>
+      </c>
       <c r="I87" t="inlineStr">
         <is>
           <t xml:space="preserve">9/6/2026</t>
-        </is>
-      </c>
-      <c r="J87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -7418,14 +7418,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-09</t>
+        </is>
+      </c>
       <c r="I89" t="inlineStr">
         <is>
           <t xml:space="preserve">9/6/2026</t>
-        </is>
-      </c>
-      <c r="J89" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -7500,14 +7500,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-08</t>
+        </is>
+      </c>
       <c r="I90" t="inlineStr">
         <is>
           <t xml:space="preserve">8/5/2026</t>
-        </is>
-      </c>
-      <c r="J90" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -8320,14 +8320,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-11-10</t>
+        </is>
+      </c>
       <c r="I100" t="inlineStr">
         <is>
           <t xml:space="preserve">10/11/2025</t>
-        </is>
-      </c>
-      <c r="J100" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -8402,14 +8402,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-11-10</t>
+        </is>
+      </c>
       <c r="I101" t="inlineStr">
         <is>
           <t xml:space="preserve">10/11/2025</t>
-        </is>
-      </c>
-      <c r="J101" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -8484,14 +8484,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-06-02</t>
+        </is>
+      </c>
       <c r="I102" t="inlineStr">
         <is>
           <t xml:space="preserve">2/6/2025</t>
-        </is>
-      </c>
-      <c r="J102" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -8576,14 +8576,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-08</t>
+        </is>
+      </c>
       <c r="I103" t="inlineStr">
         <is>
           <t xml:space="preserve">8/5/2026</t>
-        </is>
-      </c>
-      <c r="J103" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -8740,14 +8740,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-10-09</t>
+        </is>
+      </c>
       <c r="I105" t="inlineStr">
         <is>
           <t xml:space="preserve">9/10/2025</t>
-        </is>
-      </c>
-      <c r="J105" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -8822,14 +8822,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-10-09</t>
+        </is>
+      </c>
       <c r="I106" t="inlineStr">
         <is>
           <t xml:space="preserve">9/10/2025</t>
-        </is>
-      </c>
-      <c r="J106" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -8904,14 +8904,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-10-09</t>
+        </is>
+      </c>
       <c r="I107" t="inlineStr">
         <is>
           <t xml:space="preserve">9/10/2025</t>
-        </is>
-      </c>
-      <c r="J107" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -9314,14 +9314,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-06</t>
+        </is>
+      </c>
       <c r="I112" t="inlineStr">
         <is>
           <t xml:space="preserve">6/5/2026</t>
-        </is>
-      </c>
-      <c r="J112" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -9396,14 +9396,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-06</t>
+        </is>
+      </c>
       <c r="I113" t="inlineStr">
         <is>
           <t xml:space="preserve">6/5/2026</t>
-        </is>
-      </c>
-      <c r="J113" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -9642,14 +9642,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-01-06</t>
+        </is>
+      </c>
       <c r="I116" t="inlineStr">
         <is>
           <t xml:space="preserve">6/1/2025</t>
-        </is>
-      </c>
-      <c r="J116" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -10216,14 +10216,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-05</t>
+        </is>
+      </c>
       <c r="I123" t="inlineStr">
         <is>
           <t xml:space="preserve">5/12/2025</t>
-        </is>
-      </c>
-      <c r="J123" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -10298,14 +10298,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-11</t>
+        </is>
+      </c>
       <c r="I124" t="inlineStr">
         <is>
           <t xml:space="preserve">11/12/2025</t>
-        </is>
-      </c>
-      <c r="J124" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -10380,14 +10380,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-10-07</t>
+        </is>
+      </c>
       <c r="I125" t="inlineStr">
         <is>
           <t xml:space="preserve">7/10/2025</t>
-        </is>
-      </c>
-      <c r="J125" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -10954,14 +10954,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-12</t>
+        </is>
+      </c>
       <c r="I132" t="inlineStr">
         <is>
           <t xml:space="preserve">12/12/2025</t>
-        </is>
-      </c>
-      <c r="J132" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -11036,14 +11036,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-12</t>
+        </is>
+      </c>
       <c r="I133" t="inlineStr">
         <is>
           <t xml:space="preserve">12/12/2025</t>
-        </is>
-      </c>
-      <c r="J133" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -11118,14 +11118,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-10-07</t>
+        </is>
+      </c>
       <c r="I134" t="inlineStr">
         <is>
           <t xml:space="preserve">7/10/2025</t>
-        </is>
-      </c>
-      <c r="J134" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -11364,14 +11364,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-12</t>
+        </is>
+      </c>
       <c r="I137" t="inlineStr">
         <is>
           <t xml:space="preserve">12/6/2026</t>
-        </is>
-      </c>
-      <c r="J137" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -11446,14 +11446,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-12</t>
+        </is>
+      </c>
       <c r="I138" t="inlineStr">
         <is>
           <t xml:space="preserve">12/6/2026</t>
-        </is>
-      </c>
-      <c r="J138" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -11528,14 +11528,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-12</t>
+        </is>
+      </c>
       <c r="I139" t="inlineStr">
         <is>
           <t xml:space="preserve">12/6/2026</t>
-        </is>
-      </c>
-      <c r="J139" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -11610,14 +11610,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-12</t>
+        </is>
+      </c>
       <c r="I140" t="inlineStr">
         <is>
           <t xml:space="preserve">12/6/2026</t>
-        </is>
-      </c>
-      <c r="J140" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -11692,14 +11692,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-12</t>
+        </is>
+      </c>
       <c r="I141" t="inlineStr">
         <is>
           <t xml:space="preserve">12/6/2026</t>
-        </is>
-      </c>
-      <c r="J141" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -11774,14 +11774,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-12</t>
+        </is>
+      </c>
       <c r="I142" t="inlineStr">
         <is>
           <t xml:space="preserve">12/6/2026</t>
-        </is>
-      </c>
-      <c r="J142" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -11856,14 +11856,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-10</t>
+        </is>
+      </c>
       <c r="I143" t="inlineStr">
         <is>
           <t xml:space="preserve">10/3/2026</t>
-        </is>
-      </c>
-      <c r="J143" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -13265,14 +13265,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-07-03</t>
+        </is>
+      </c>
       <c r="I160" t="inlineStr">
         <is>
           <t xml:space="preserve">3/7/2025</t>
-        </is>
-      </c>
-      <c r="J160" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -13357,14 +13357,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-07-03</t>
+        </is>
+      </c>
       <c r="I161" t="inlineStr">
         <is>
           <t xml:space="preserve">3/7/2025</t>
-        </is>
-      </c>
-      <c r="J161" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -14095,14 +14095,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-08-11</t>
+        </is>
+      </c>
       <c r="I170" t="inlineStr">
         <is>
           <t xml:space="preserve">11/8/2025</t>
-        </is>
-      </c>
-      <c r="J170" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -14259,14 +14259,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-01</t>
+        </is>
+      </c>
       <c r="I172" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
-        </is>
-      </c>
-      <c r="J172" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -14341,14 +14341,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-01</t>
+        </is>
+      </c>
       <c r="I173" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
-        </is>
-      </c>
-      <c r="J173" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -14423,14 +14423,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-06</t>
+        </is>
+      </c>
       <c r="I174" t="inlineStr">
         <is>
           <t xml:space="preserve">6/5/2026</t>
-        </is>
-      </c>
-      <c r="J174" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -14505,14 +14505,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-06</t>
+        </is>
+      </c>
       <c r="I175" t="inlineStr">
         <is>
           <t xml:space="preserve">6/5/2026</t>
-        </is>
-      </c>
-      <c r="J175" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -14587,14 +14587,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-06</t>
+        </is>
+      </c>
       <c r="I176" t="inlineStr">
         <is>
           <t xml:space="preserve">6/5/2026</t>
-        </is>
-      </c>
-      <c r="J176" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -14669,14 +14669,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-01</t>
+        </is>
+      </c>
       <c r="I177" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
-        </is>
-      </c>
-      <c r="J177" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -14751,14 +14751,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-01</t>
+        </is>
+      </c>
       <c r="I178" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
-        </is>
-      </c>
-      <c r="J178" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -15693,14 +15693,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-07-03</t>
+        </is>
+      </c>
       <c r="I189" t="inlineStr">
         <is>
           <t xml:space="preserve">3/7/2025</t>
-        </is>
-      </c>
-      <c r="J189" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -15775,14 +15775,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-07-03</t>
+        </is>
+      </c>
       <c r="I190" t="inlineStr">
         <is>
           <t xml:space="preserve">3/7/2025</t>
-        </is>
-      </c>
-      <c r="J190" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -16021,14 +16021,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-06-02</t>
+        </is>
+      </c>
       <c r="I193" t="inlineStr">
         <is>
           <t xml:space="preserve">2/6/2025</t>
-        </is>
-      </c>
-      <c r="J193" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -16103,14 +16103,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-07-03</t>
+        </is>
+      </c>
       <c r="I194" t="inlineStr">
         <is>
           <t xml:space="preserve">3/7/2025</t>
-        </is>
-      </c>
-      <c r="J194" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -16431,14 +16431,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-11-04</t>
+        </is>
+      </c>
       <c r="I198" t="inlineStr">
         <is>
           <t xml:space="preserve">4/11/2025</t>
-        </is>
-      </c>
-      <c r="J198" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -16595,14 +16595,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-11-04</t>
+        </is>
+      </c>
       <c r="I200" t="inlineStr">
         <is>
           <t xml:space="preserve">4/11/2025</t>
-        </is>
-      </c>
-      <c r="J200" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -17671,14 +17671,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-04</t>
+        </is>
+      </c>
       <c r="I213" t="inlineStr">
         <is>
           <t xml:space="preserve">4/6/2026</t>
-        </is>
-      </c>
-      <c r="J213" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K213" t="inlineStr">
@@ -17763,14 +17763,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-04</t>
+        </is>
+      </c>
       <c r="I214" t="inlineStr">
         <is>
           <t xml:space="preserve">4/6/2026</t>
-        </is>
-      </c>
-      <c r="J214" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -18511,14 +18511,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-05</t>
+        </is>
+      </c>
       <c r="I223" t="inlineStr">
         <is>
           <t xml:space="preserve">5/1/2024</t>
-        </is>
-      </c>
-      <c r="J223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K223" t="inlineStr">
@@ -18839,14 +18839,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-04-05</t>
+        </is>
+      </c>
       <c r="I227" t="inlineStr">
         <is>
           <t xml:space="preserve">5/4/2024</t>
-        </is>
-      </c>
-      <c r="J227" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K227" t="inlineStr">
@@ -19167,14 +19167,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-04</t>
+        </is>
+      </c>
       <c r="I231" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
-        </is>
-      </c>
-      <c r="J231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
@@ -19495,14 +19495,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-05</t>
+        </is>
+      </c>
       <c r="I235" t="inlineStr">
         <is>
           <t xml:space="preserve">5/3/2026</t>
-        </is>
-      </c>
-      <c r="J235" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
@@ -19813,14 +19813,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-11-06</t>
+        </is>
+      </c>
       <c r="I239" t="inlineStr">
         <is>
           <t xml:space="preserve">6/11/2025</t>
-        </is>
-      </c>
-      <c r="J239" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
@@ -19977,14 +19977,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-11-06</t>
+        </is>
+      </c>
       <c r="I241" t="inlineStr">
         <is>
           <t xml:space="preserve">6/11/2025</t>
-        </is>
-      </c>
-      <c r="J241" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
@@ -20136,14 +20136,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-12</t>
+        </is>
+      </c>
       <c r="I243" t="inlineStr">
         <is>
           <t xml:space="preserve">12/12/2025</t>
-        </is>
-      </c>
-      <c r="J243" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -20218,14 +20218,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-12</t>
+        </is>
+      </c>
       <c r="I244" t="inlineStr">
         <is>
           <t xml:space="preserve">12/12/2025</t>
-        </is>
-      </c>
-      <c r="J244" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -20300,14 +20300,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-12</t>
+        </is>
+      </c>
       <c r="I245" t="inlineStr">
         <is>
           <t xml:space="preserve">12/12/2025</t>
-        </is>
-      </c>
-      <c r="J245" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -20382,14 +20382,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-12</t>
+        </is>
+      </c>
       <c r="I246" t="inlineStr">
         <is>
           <t xml:space="preserve">12/12/2025</t>
-        </is>
-      </c>
-      <c r="J246" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
@@ -20546,14 +20546,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-11</t>
+        </is>
+      </c>
       <c r="I248" t="inlineStr">
         <is>
           <t xml:space="preserve">11/12/2025</t>
-        </is>
-      </c>
-      <c r="J248" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -20792,14 +20792,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-05</t>
+        </is>
+      </c>
       <c r="I251" t="inlineStr">
         <is>
           <t xml:space="preserve">5/12/2025</t>
-        </is>
-      </c>
-      <c r="J251" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -20874,14 +20874,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-11-10</t>
+        </is>
+      </c>
       <c r="I252" t="inlineStr">
         <is>
           <t xml:space="preserve">10/11/2025</t>
-        </is>
-      </c>
-      <c r="J252" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
@@ -20956,14 +20956,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-10</t>
+        </is>
+      </c>
       <c r="I253" t="inlineStr">
         <is>
           <t xml:space="preserve">10/8/2026</t>
-        </is>
-      </c>
-      <c r="J253" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
@@ -21038,14 +21038,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-02</t>
+        </is>
+      </c>
       <c r="I254" t="inlineStr">
         <is>
           <t xml:space="preserve">2/12/2025</t>
-        </is>
-      </c>
-      <c r="J254" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -21120,14 +21120,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-04</t>
+        </is>
+      </c>
       <c r="I255" t="inlineStr">
         <is>
           <t xml:space="preserve">4/12/2025</t>
-        </is>
-      </c>
-      <c r="J255" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -21202,14 +21202,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-04</t>
+        </is>
+      </c>
       <c r="I256" t="inlineStr">
         <is>
           <t xml:space="preserve">4/12/2025</t>
-        </is>
-      </c>
-      <c r="J256" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -21284,14 +21284,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-05</t>
+        </is>
+      </c>
       <c r="I257" t="inlineStr">
         <is>
           <t xml:space="preserve">5/12/2025</t>
-        </is>
-      </c>
-      <c r="J257" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -21366,14 +21366,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-02</t>
+        </is>
+      </c>
       <c r="I258" t="inlineStr">
         <is>
           <t xml:space="preserve">2/12/2025</t>
-        </is>
-      </c>
-      <c r="J258" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -21448,14 +21448,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-02</t>
+        </is>
+      </c>
       <c r="I259" t="inlineStr">
         <is>
           <t xml:space="preserve">2/12/2025</t>
-        </is>
-      </c>
-      <c r="J259" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
@@ -22176,14 +22176,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-02</t>
+        </is>
+      </c>
       <c r="I268" t="inlineStr">
         <is>
           <t xml:space="preserve">2/1/2026</t>
-        </is>
-      </c>
-      <c r="J268" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -22258,14 +22258,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-02</t>
+        </is>
+      </c>
       <c r="I269" t="inlineStr">
         <is>
           <t xml:space="preserve">2/1/2026</t>
-        </is>
-      </c>
-      <c r="J269" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K269" t="inlineStr">
@@ -22340,14 +22340,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-02</t>
+        </is>
+      </c>
       <c r="I270" t="inlineStr">
         <is>
           <t xml:space="preserve">2/1/2026</t>
-        </is>
-      </c>
-      <c r="J270" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K270" t="inlineStr">
@@ -22422,14 +22422,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-08</t>
+        </is>
+      </c>
       <c r="I271" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
-        </is>
-      </c>
-      <c r="J271" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
@@ -22914,14 +22914,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-08</t>
+        </is>
+      </c>
       <c r="I277" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
-        </is>
-      </c>
-      <c r="J277" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
@@ -23483,14 +23483,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-05</t>
+        </is>
+      </c>
       <c r="I284" t="inlineStr">
         <is>
           <t xml:space="preserve">5/1/2026</t>
-        </is>
-      </c>
-      <c r="J284" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -23811,14 +23811,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-04</t>
+        </is>
+      </c>
       <c r="I288" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
-        </is>
-      </c>
-      <c r="J288" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">
@@ -23893,14 +23893,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-04</t>
+        </is>
+      </c>
       <c r="I289" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
-        </is>
-      </c>
-      <c r="J289" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K289" t="inlineStr">
@@ -23975,14 +23975,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-08</t>
+        </is>
+      </c>
       <c r="I290" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
-        </is>
-      </c>
-      <c r="J290" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K290" t="inlineStr">
@@ -24057,14 +24057,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-08</t>
+        </is>
+      </c>
       <c r="I291" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
-        </is>
-      </c>
-      <c r="J291" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K291" t="inlineStr">
@@ -24139,14 +24139,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-08</t>
+        </is>
+      </c>
       <c r="I292" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
-        </is>
-      </c>
-      <c r="J292" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K292" t="inlineStr">
@@ -24221,14 +24221,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-08</t>
+        </is>
+      </c>
       <c r="I293" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
-        </is>
-      </c>
-      <c r="J293" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K293" t="inlineStr">
@@ -24303,14 +24303,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-08</t>
+        </is>
+      </c>
       <c r="I294" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
-        </is>
-      </c>
-      <c r="J294" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K294" t="inlineStr">
@@ -24631,14 +24631,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-05</t>
+        </is>
+      </c>
       <c r="I298" t="inlineStr">
         <is>
           <t xml:space="preserve">5/5/2025</t>
-        </is>
-      </c>
-      <c r="J298" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K298" t="inlineStr">
@@ -24713,14 +24713,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-01</t>
+        </is>
+      </c>
       <c r="I299" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
-        </is>
-      </c>
-      <c r="J299" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K299" t="inlineStr">
@@ -24795,14 +24795,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-01</t>
+        </is>
+      </c>
       <c r="I300" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
-        </is>
-      </c>
-      <c r="J300" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K300" t="inlineStr">
@@ -24877,14 +24877,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-01</t>
+        </is>
+      </c>
       <c r="I301" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
-        </is>
-      </c>
-      <c r="J301" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K301" t="inlineStr">
@@ -24959,14 +24959,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-01</t>
+        </is>
+      </c>
       <c r="I302" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
-        </is>
-      </c>
-      <c r="J302" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K302" t="inlineStr">
@@ -25369,14 +25369,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-02</t>
+        </is>
+      </c>
       <c r="I307" t="inlineStr">
         <is>
           <t xml:space="preserve">2/5/2025</t>
-        </is>
-      </c>
-      <c r="J307" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K307" t="inlineStr">
@@ -25451,14 +25451,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-04</t>
+        </is>
+      </c>
       <c r="I308" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
-        </is>
-      </c>
-      <c r="J308" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K308" t="inlineStr">
@@ -25533,14 +25533,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-04</t>
+        </is>
+      </c>
       <c r="I309" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
-        </is>
-      </c>
-      <c r="J309" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K309" t="inlineStr">
@@ -25615,14 +25615,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-04</t>
+        </is>
+      </c>
       <c r="I310" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
-        </is>
-      </c>
-      <c r="J310" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K310" t="inlineStr">
@@ -25697,14 +25697,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-04</t>
+        </is>
+      </c>
       <c r="I311" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
-        </is>
-      </c>
-      <c r="J311" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K311" t="inlineStr">
@@ -25779,14 +25779,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-04</t>
+        </is>
+      </c>
       <c r="I312" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
-        </is>
-      </c>
-      <c r="J312" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K312" t="inlineStr">
@@ -25861,14 +25861,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-04</t>
+        </is>
+      </c>
       <c r="I313" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
-        </is>
-      </c>
-      <c r="J313" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K313" t="inlineStr">
@@ -26025,14 +26025,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-02</t>
+        </is>
+      </c>
       <c r="I315" t="inlineStr">
         <is>
           <t xml:space="preserve">2/5/2025</t>
-        </is>
-      </c>
-      <c r="J315" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K315" t="inlineStr">
@@ -26373,14 +26373,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-04</t>
+        </is>
+      </c>
       <c r="I319" t="inlineStr">
         <is>
           <t xml:space="preserve">4/6/2026</t>
-        </is>
-      </c>
-      <c r="J319" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K319" t="inlineStr">
@@ -26942,14 +26942,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-04-10</t>
+        </is>
+      </c>
       <c r="I326" t="inlineStr">
         <is>
           <t xml:space="preserve">10/4/2026</t>
-        </is>
-      </c>
-      <c r="J326" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K326" t="inlineStr">
@@ -27106,14 +27106,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-04-10</t>
+        </is>
+      </c>
       <c r="I328" t="inlineStr">
         <is>
           <t xml:space="preserve">10/4/2026</t>
-        </is>
-      </c>
-      <c r="J328" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K328" t="inlineStr">
@@ -27188,14 +27188,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-04-10</t>
+        </is>
+      </c>
       <c r="I329" t="inlineStr">
         <is>
           <t xml:space="preserve">10/4/2026</t>
-        </is>
-      </c>
-      <c r="J329" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K329" t="inlineStr">
@@ -27270,14 +27270,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-04-10</t>
+        </is>
+      </c>
       <c r="I330" t="inlineStr">
         <is>
           <t xml:space="preserve">10/4/2026</t>
-        </is>
-      </c>
-      <c r="J330" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K330" t="inlineStr">
@@ -27352,14 +27352,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-10</t>
+        </is>
+      </c>
       <c r="I331" t="inlineStr">
         <is>
           <t xml:space="preserve">10/2/2026</t>
-        </is>
-      </c>
-      <c r="J331" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K331" t="inlineStr">
@@ -27516,14 +27516,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-06</t>
+        </is>
+      </c>
       <c r="I333" t="inlineStr">
         <is>
           <t xml:space="preserve">6/2/2026</t>
-        </is>
-      </c>
-      <c r="J333" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K333" t="inlineStr">

</xml_diff>

<commit_message>
Import 486 vials from Cell Stocks UC -80.xlsx from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -184,14 +184,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-05-05</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t xml:space="preserve">5/5/2025</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -266,14 +266,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-05-05</t>
-        </is>
-      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t xml:space="preserve">5/5/2025</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -348,14 +348,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-05-05</t>
-        </is>
-      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t xml:space="preserve">5/5/2025</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -430,14 +430,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-05-05</t>
-        </is>
-      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t xml:space="preserve">5/5/2025</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -512,14 +512,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-04-09</t>
-        </is>
-      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t xml:space="preserve">9/4/2026</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -594,14 +594,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-04-09</t>
-        </is>
-      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t xml:space="preserve">9/4/2026</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -840,14 +840,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-02-10</t>
-        </is>
-      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t xml:space="preserve">10/2/2026</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1578,14 +1578,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-05-08</t>
-        </is>
-      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t xml:space="preserve">8/5/2025</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1660,14 +1660,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-05-08</t>
-        </is>
-      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t xml:space="preserve">8/5/2025</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1742,14 +1742,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-05-08</t>
-        </is>
-      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t xml:space="preserve">8/5/2025</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1824,14 +1824,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-05-08</t>
-        </is>
-      </c>
       <c r="I22" t="inlineStr">
         <is>
           <t xml:space="preserve">8/5/2025</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1906,14 +1906,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-05-07</t>
-        </is>
-      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t xml:space="preserve">7/5/2025</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1988,14 +1988,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-05-07</t>
-        </is>
-      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t xml:space="preserve">7/5/2025</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2070,14 +2070,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-05-07</t>
-        </is>
-      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t xml:space="preserve">7/5/2025</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -3176,14 +3176,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2023-02-03</t>
-        </is>
-      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t xml:space="preserve">3/2/2023</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3340,14 +3340,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-05-02</t>
-        </is>
-      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t xml:space="preserve">2/5/2025</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3750,14 +3750,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-02-06</t>
-        </is>
-      </c>
       <c r="I45" t="inlineStr">
         <is>
           <t xml:space="preserve">6/2/2026</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3914,14 +3914,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-02-05</t>
-        </is>
-      </c>
       <c r="I47" t="inlineStr">
         <is>
           <t xml:space="preserve">5/2/2026</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3996,14 +3996,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-02-02</t>
-        </is>
-      </c>
       <c r="I48" t="inlineStr">
         <is>
           <t xml:space="preserve">2/2/2026</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -4160,14 +4160,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-02-02</t>
-        </is>
-      </c>
       <c r="I50" t="inlineStr">
         <is>
           <t xml:space="preserve">2/2/2026</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -4324,14 +4324,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-03</t>
-        </is>
-      </c>
       <c r="I52" t="inlineStr">
         <is>
           <t xml:space="preserve">3/3/2026</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -4406,14 +4406,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-03</t>
-        </is>
-      </c>
       <c r="I53" t="inlineStr">
         <is>
           <t xml:space="preserve">3/3/2026</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -5686,14 +5686,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-02-02</t>
-        </is>
-      </c>
       <c r="I68" t="inlineStr">
         <is>
           <t xml:space="preserve">2/2/2026</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -5850,14 +5850,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-02-02</t>
-        </is>
-      </c>
       <c r="I70" t="inlineStr">
         <is>
           <t xml:space="preserve">2/2/2026</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -6096,14 +6096,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-04-10</t>
-        </is>
-      </c>
       <c r="I73" t="inlineStr">
         <is>
           <t xml:space="preserve">10/4/2026</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -6178,14 +6178,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-04-10</t>
-        </is>
-      </c>
       <c r="I74" t="inlineStr">
         <is>
           <t xml:space="preserve">10/4/2026</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -6752,14 +6752,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-10</t>
-        </is>
-      </c>
       <c r="I81" t="inlineStr">
         <is>
           <t xml:space="preserve">10/3/2026</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -6834,14 +6834,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-11</t>
-        </is>
-      </c>
       <c r="I82" t="inlineStr">
         <is>
           <t xml:space="preserve">11/3/2026</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -6916,14 +6916,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-11</t>
-        </is>
-      </c>
       <c r="I83" t="inlineStr">
         <is>
           <t xml:space="preserve">11/3/2026</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -6998,14 +6998,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-10</t>
-        </is>
-      </c>
       <c r="I84" t="inlineStr">
         <is>
           <t xml:space="preserve">10/3/2026</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -7162,14 +7162,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-07-07</t>
-        </is>
-      </c>
       <c r="I86" t="inlineStr">
         <is>
           <t xml:space="preserve">7/7/2025</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -7254,14 +7254,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-09</t>
-        </is>
-      </c>
       <c r="I87" t="inlineStr">
         <is>
           <t xml:space="preserve">9/6/2026</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -7418,14 +7418,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-09</t>
-        </is>
-      </c>
       <c r="I89" t="inlineStr">
         <is>
           <t xml:space="preserve">9/6/2026</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -7500,14 +7500,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-08</t>
-        </is>
-      </c>
       <c r="I90" t="inlineStr">
         <is>
           <t xml:space="preserve">8/5/2026</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -8320,14 +8320,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-11-10</t>
-        </is>
-      </c>
       <c r="I100" t="inlineStr">
         <is>
           <t xml:space="preserve">10/11/2025</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -8402,14 +8402,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H101" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-11-10</t>
-        </is>
-      </c>
       <c r="I101" t="inlineStr">
         <is>
           <t xml:space="preserve">10/11/2025</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -8484,14 +8484,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-06-02</t>
-        </is>
-      </c>
       <c r="I102" t="inlineStr">
         <is>
           <t xml:space="preserve">2/6/2025</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -8576,14 +8576,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H103" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-08</t>
-        </is>
-      </c>
       <c r="I103" t="inlineStr">
         <is>
           <t xml:space="preserve">8/5/2026</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -8740,14 +8740,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-10-09</t>
-        </is>
-      </c>
       <c r="I105" t="inlineStr">
         <is>
           <t xml:space="preserve">9/10/2025</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -8822,14 +8822,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-10-09</t>
-        </is>
-      </c>
       <c r="I106" t="inlineStr">
         <is>
           <t xml:space="preserve">9/10/2025</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -8904,14 +8904,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-10-09</t>
-        </is>
-      </c>
       <c r="I107" t="inlineStr">
         <is>
           <t xml:space="preserve">9/10/2025</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -9314,14 +9314,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H112" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-06</t>
-        </is>
-      </c>
       <c r="I112" t="inlineStr">
         <is>
           <t xml:space="preserve">6/5/2026</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -9396,14 +9396,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H113" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-06</t>
-        </is>
-      </c>
       <c r="I113" t="inlineStr">
         <is>
           <t xml:space="preserve">6/5/2026</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -9642,14 +9642,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-01-06</t>
-        </is>
-      </c>
       <c r="I116" t="inlineStr">
         <is>
           <t xml:space="preserve">6/1/2025</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -10216,14 +10216,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-12-05</t>
-        </is>
-      </c>
       <c r="I123" t="inlineStr">
         <is>
           <t xml:space="preserve">5/12/2025</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -10298,14 +10298,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H124" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-12-11</t>
-        </is>
-      </c>
       <c r="I124" t="inlineStr">
         <is>
           <t xml:space="preserve">11/12/2025</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -10380,14 +10380,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H125" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-10-07</t>
-        </is>
-      </c>
       <c r="I125" t="inlineStr">
         <is>
           <t xml:space="preserve">7/10/2025</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -10954,14 +10954,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H132" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-12-12</t>
-        </is>
-      </c>
       <c r="I132" t="inlineStr">
         <is>
           <t xml:space="preserve">12/12/2025</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -11036,14 +11036,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-12-12</t>
-        </is>
-      </c>
       <c r="I133" t="inlineStr">
         <is>
           <t xml:space="preserve">12/12/2025</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -11118,14 +11118,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H134" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-10-07</t>
-        </is>
-      </c>
       <c r="I134" t="inlineStr">
         <is>
           <t xml:space="preserve">7/10/2025</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -11364,14 +11364,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-12</t>
-        </is>
-      </c>
       <c r="I137" t="inlineStr">
         <is>
           <t xml:space="preserve">12/6/2026</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -11446,14 +11446,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H138" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-12</t>
-        </is>
-      </c>
       <c r="I138" t="inlineStr">
         <is>
           <t xml:space="preserve">12/6/2026</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -11528,14 +11528,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H139" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-12</t>
-        </is>
-      </c>
       <c r="I139" t="inlineStr">
         <is>
           <t xml:space="preserve">12/6/2026</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -11610,14 +11610,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H140" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-12</t>
-        </is>
-      </c>
       <c r="I140" t="inlineStr">
         <is>
           <t xml:space="preserve">12/6/2026</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -11692,14 +11692,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H141" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-12</t>
-        </is>
-      </c>
       <c r="I141" t="inlineStr">
         <is>
           <t xml:space="preserve">12/6/2026</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -11774,14 +11774,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H142" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-12</t>
-        </is>
-      </c>
       <c r="I142" t="inlineStr">
         <is>
           <t xml:space="preserve">12/6/2026</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -11856,14 +11856,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H143" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-10</t>
-        </is>
-      </c>
       <c r="I143" t="inlineStr">
         <is>
           <t xml:space="preserve">10/3/2026</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -13265,14 +13265,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H160" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-07-03</t>
-        </is>
-      </c>
       <c r="I160" t="inlineStr">
         <is>
           <t xml:space="preserve">3/7/2025</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -13357,14 +13357,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H161" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-07-03</t>
-        </is>
-      </c>
       <c r="I161" t="inlineStr">
         <is>
           <t xml:space="preserve">3/7/2025</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -14095,14 +14095,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H170" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-08-11</t>
-        </is>
-      </c>
       <c r="I170" t="inlineStr">
         <is>
           <t xml:space="preserve">11/8/2025</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -14259,14 +14259,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H172" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-01</t>
-        </is>
-      </c>
       <c r="I172" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -14341,14 +14341,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H173" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-01</t>
-        </is>
-      </c>
       <c r="I173" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -14423,14 +14423,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H174" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-06</t>
-        </is>
-      </c>
       <c r="I174" t="inlineStr">
         <is>
           <t xml:space="preserve">6/5/2026</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -14505,14 +14505,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H175" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-06</t>
-        </is>
-      </c>
       <c r="I175" t="inlineStr">
         <is>
           <t xml:space="preserve">6/5/2026</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -14587,14 +14587,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H176" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-06</t>
-        </is>
-      </c>
       <c r="I176" t="inlineStr">
         <is>
           <t xml:space="preserve">6/5/2026</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -14669,14 +14669,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H177" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-01</t>
-        </is>
-      </c>
       <c r="I177" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -14751,14 +14751,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H178" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-01</t>
-        </is>
-      </c>
       <c r="I178" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -15693,14 +15693,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H189" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-07-03</t>
-        </is>
-      </c>
       <c r="I189" t="inlineStr">
         <is>
           <t xml:space="preserve">3/7/2025</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -15775,14 +15775,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H190" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-07-03</t>
-        </is>
-      </c>
       <c r="I190" t="inlineStr">
         <is>
           <t xml:space="preserve">3/7/2025</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -16021,14 +16021,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H193" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-06-02</t>
-        </is>
-      </c>
       <c r="I193" t="inlineStr">
         <is>
           <t xml:space="preserve">2/6/2025</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -16103,14 +16103,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H194" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-07-03</t>
-        </is>
-      </c>
       <c r="I194" t="inlineStr">
         <is>
           <t xml:space="preserve">3/7/2025</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -16431,14 +16431,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H198" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-11-04</t>
-        </is>
-      </c>
       <c r="I198" t="inlineStr">
         <is>
           <t xml:space="preserve">4/11/2025</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -16595,14 +16595,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H200" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-11-04</t>
-        </is>
-      </c>
       <c r="I200" t="inlineStr">
         <is>
           <t xml:space="preserve">4/11/2025</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -17671,14 +17671,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H213" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-04</t>
-        </is>
-      </c>
       <c r="I213" t="inlineStr">
         <is>
           <t xml:space="preserve">4/6/2026</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K213" t="inlineStr">
@@ -17763,14 +17763,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H214" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-04</t>
-        </is>
-      </c>
       <c r="I214" t="inlineStr">
         <is>
           <t xml:space="preserve">4/6/2026</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -18511,14 +18511,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2024-01-05</t>
-        </is>
-      </c>
       <c r="I223" t="inlineStr">
         <is>
           <t xml:space="preserve">5/1/2024</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K223" t="inlineStr">
@@ -18839,14 +18839,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H227" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2024-04-05</t>
-        </is>
-      </c>
       <c r="I227" t="inlineStr">
         <is>
           <t xml:space="preserve">5/4/2024</t>
+        </is>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K227" t="inlineStr">
@@ -19167,14 +19167,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-04</t>
-        </is>
-      </c>
       <c r="I231" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
@@ -19495,14 +19495,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H235" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-05</t>
-        </is>
-      </c>
       <c r="I235" t="inlineStr">
         <is>
           <t xml:space="preserve">5/3/2026</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
@@ -19813,14 +19813,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H239" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-11-06</t>
-        </is>
-      </c>
       <c r="I239" t="inlineStr">
         <is>
           <t xml:space="preserve">6/11/2025</t>
+        </is>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
@@ -19977,14 +19977,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H241" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-11-06</t>
-        </is>
-      </c>
       <c r="I241" t="inlineStr">
         <is>
           <t xml:space="preserve">6/11/2025</t>
+        </is>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
@@ -20136,14 +20136,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H243" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-12-12</t>
-        </is>
-      </c>
       <c r="I243" t="inlineStr">
         <is>
           <t xml:space="preserve">12/12/2025</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -20218,14 +20218,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H244" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-12-12</t>
-        </is>
-      </c>
       <c r="I244" t="inlineStr">
         <is>
           <t xml:space="preserve">12/12/2025</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -20300,14 +20300,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H245" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-12-12</t>
-        </is>
-      </c>
       <c r="I245" t="inlineStr">
         <is>
           <t xml:space="preserve">12/12/2025</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -20382,14 +20382,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H246" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-12-12</t>
-        </is>
-      </c>
       <c r="I246" t="inlineStr">
         <is>
           <t xml:space="preserve">12/12/2025</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
@@ -20546,14 +20546,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H248" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-12-11</t>
-        </is>
-      </c>
       <c r="I248" t="inlineStr">
         <is>
           <t xml:space="preserve">11/12/2025</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -20792,14 +20792,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H251" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-12-05</t>
-        </is>
-      </c>
       <c r="I251" t="inlineStr">
         <is>
           <t xml:space="preserve">5/12/2025</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -20874,14 +20874,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H252" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-11-10</t>
-        </is>
-      </c>
       <c r="I252" t="inlineStr">
         <is>
           <t xml:space="preserve">10/11/2025</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
@@ -20956,14 +20956,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H253" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-10</t>
-        </is>
-      </c>
       <c r="I253" t="inlineStr">
         <is>
           <t xml:space="preserve">10/8/2026</t>
+        </is>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
@@ -21038,14 +21038,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H254" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-12-02</t>
-        </is>
-      </c>
       <c r="I254" t="inlineStr">
         <is>
           <t xml:space="preserve">2/12/2025</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -21120,14 +21120,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H255" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-12-04</t>
-        </is>
-      </c>
       <c r="I255" t="inlineStr">
         <is>
           <t xml:space="preserve">4/12/2025</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -21202,14 +21202,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H256" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-12-04</t>
-        </is>
-      </c>
       <c r="I256" t="inlineStr">
         <is>
           <t xml:space="preserve">4/12/2025</t>
+        </is>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -21284,14 +21284,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H257" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-12-05</t>
-        </is>
-      </c>
       <c r="I257" t="inlineStr">
         <is>
           <t xml:space="preserve">5/12/2025</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -21366,14 +21366,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H258" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-12-02</t>
-        </is>
-      </c>
       <c r="I258" t="inlineStr">
         <is>
           <t xml:space="preserve">2/12/2025</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -21448,14 +21448,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H259" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-12-02</t>
-        </is>
-      </c>
       <c r="I259" t="inlineStr">
         <is>
           <t xml:space="preserve">2/12/2025</t>
+        </is>
+      </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
@@ -22176,14 +22176,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H268" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-01-02</t>
-        </is>
-      </c>
       <c r="I268" t="inlineStr">
         <is>
           <t xml:space="preserve">2/1/2026</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -22258,14 +22258,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H269" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-01-02</t>
-        </is>
-      </c>
       <c r="I269" t="inlineStr">
         <is>
           <t xml:space="preserve">2/1/2026</t>
+        </is>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K269" t="inlineStr">
@@ -22340,14 +22340,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H270" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-01-02</t>
-        </is>
-      </c>
       <c r="I270" t="inlineStr">
         <is>
           <t xml:space="preserve">2/1/2026</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K270" t="inlineStr">
@@ -22422,14 +22422,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H271" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-01-08</t>
-        </is>
-      </c>
       <c r="I271" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
@@ -22914,14 +22914,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H277" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-01-08</t>
-        </is>
-      </c>
       <c r="I277" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
@@ -23483,14 +23483,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H284" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-01-05</t>
-        </is>
-      </c>
       <c r="I284" t="inlineStr">
         <is>
           <t xml:space="preserve">5/1/2026</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -23811,14 +23811,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H288" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-04</t>
-        </is>
-      </c>
       <c r="I288" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">
@@ -23893,14 +23893,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H289" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-04</t>
-        </is>
-      </c>
       <c r="I289" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K289" t="inlineStr">
@@ -23975,14 +23975,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H290" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-01-08</t>
-        </is>
-      </c>
       <c r="I290" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K290" t="inlineStr">
@@ -24057,14 +24057,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H291" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-01-08</t>
-        </is>
-      </c>
       <c r="I291" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K291" t="inlineStr">
@@ -24139,14 +24139,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H292" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-01-08</t>
-        </is>
-      </c>
       <c r="I292" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K292" t="inlineStr">
@@ -24221,14 +24221,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H293" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-01-08</t>
-        </is>
-      </c>
       <c r="I293" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K293" t="inlineStr">
@@ -24303,14 +24303,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H294" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-01-08</t>
-        </is>
-      </c>
       <c r="I294" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K294" t="inlineStr">
@@ -24631,14 +24631,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H298" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-05-05</t>
-        </is>
-      </c>
       <c r="I298" t="inlineStr">
         <is>
           <t xml:space="preserve">5/5/2025</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K298" t="inlineStr">
@@ -24713,14 +24713,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H299" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-01</t>
-        </is>
-      </c>
       <c r="I299" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K299" t="inlineStr">
@@ -24795,14 +24795,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H300" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-01</t>
-        </is>
-      </c>
       <c r="I300" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K300" t="inlineStr">
@@ -24877,14 +24877,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H301" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-01</t>
-        </is>
-      </c>
       <c r="I301" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K301" t="inlineStr">
@@ -24959,14 +24959,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H302" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-01</t>
-        </is>
-      </c>
       <c r="I302" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K302" t="inlineStr">
@@ -25369,14 +25369,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H307" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-05-02</t>
-        </is>
-      </c>
       <c r="I307" t="inlineStr">
         <is>
           <t xml:space="preserve">2/5/2025</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K307" t="inlineStr">
@@ -25451,14 +25451,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H308" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-04</t>
-        </is>
-      </c>
       <c r="I308" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K308" t="inlineStr">
@@ -25533,14 +25533,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H309" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-04</t>
-        </is>
-      </c>
       <c r="I309" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K309" t="inlineStr">
@@ -25615,14 +25615,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H310" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-04</t>
-        </is>
-      </c>
       <c r="I310" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K310" t="inlineStr">
@@ -25697,14 +25697,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H311" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-04</t>
-        </is>
-      </c>
       <c r="I311" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K311" t="inlineStr">
@@ -25779,14 +25779,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H312" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-04</t>
-        </is>
-      </c>
       <c r="I312" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K312" t="inlineStr">
@@ -25861,14 +25861,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H313" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-04</t>
-        </is>
-      </c>
       <c r="I313" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K313" t="inlineStr">
@@ -26025,14 +26025,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H315" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-05-02</t>
-        </is>
-      </c>
       <c r="I315" t="inlineStr">
         <is>
           <t xml:space="preserve">2/5/2025</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K315" t="inlineStr">
@@ -26373,14 +26373,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
-      <c r="H319" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-04</t>
-        </is>
-      </c>
       <c r="I319" t="inlineStr">
         <is>
           <t xml:space="preserve">4/6/2026</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K319" t="inlineStr">
@@ -26942,14 +26942,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H326" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-04-10</t>
-        </is>
-      </c>
       <c r="I326" t="inlineStr">
         <is>
           <t xml:space="preserve">10/4/2026</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K326" t="inlineStr">
@@ -27106,14 +27106,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H328" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-04-10</t>
-        </is>
-      </c>
       <c r="I328" t="inlineStr">
         <is>
           <t xml:space="preserve">10/4/2026</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K328" t="inlineStr">
@@ -27188,14 +27188,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H329" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-04-10</t>
-        </is>
-      </c>
       <c r="I329" t="inlineStr">
         <is>
           <t xml:space="preserve">10/4/2026</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K329" t="inlineStr">
@@ -27270,14 +27270,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H330" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-04-10</t>
-        </is>
-      </c>
       <c r="I330" t="inlineStr">
         <is>
           <t xml:space="preserve">10/4/2026</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K330" t="inlineStr">
@@ -27352,14 +27352,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H331" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-02-10</t>
-        </is>
-      </c>
       <c r="I331" t="inlineStr">
         <is>
           <t xml:space="preserve">10/2/2026</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K331" t="inlineStr">
@@ -27516,14 +27516,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H333" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-02-06</t>
-        </is>
-      </c>
       <c r="I333" t="inlineStr">
         <is>
           <t xml:space="preserve">6/2/2026</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K333" t="inlineStr">

</xml_diff>

<commit_message>
Add 2 × hek gnt from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -20123,7 +20123,7 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">hek gnt</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
@@ -20168,7 +20168,7 @@
       </c>
       <c r="O243" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R243" t="inlineStr">
@@ -20178,7 +20178,7 @@
       </c>
       <c r="S243" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdw768-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
@@ -20205,7 +20205,7 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">hek gnt</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
@@ -20250,7 +20250,7 @@
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R244" t="inlineStr">
@@ -20260,7 +20260,7 @@
       </c>
       <c r="S244" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdw768-1</t>
+          <t xml:space="preserve">v-mtrdx0po-1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark a date Unknown from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -20879,9 +20879,9 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="J252" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">

</xml_diff>

<commit_message>
Add a caspex rule
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -3039,7 +3039,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
@@ -5007,7 +5007,7 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
@@ -5089,7 +5089,7 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
@@ -5181,7 +5181,7 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O62" t="inlineStr">
@@ -5273,7 +5273,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O63" t="inlineStr">
@@ -5365,7 +5365,7 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
@@ -5539,7 +5539,7 @@
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O66" t="inlineStr">
@@ -5621,7 +5621,7 @@
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
@@ -5703,7 +5703,7 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
@@ -5785,7 +5785,7 @@
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
@@ -5867,7 +5867,7 @@
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O70" t="inlineStr">
@@ -5949,7 +5949,7 @@
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O71" t="inlineStr">
@@ -6697,7 +6697,7 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
@@ -11883,7 +11883,7 @@
       </c>
       <c r="N143" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O143" t="inlineStr">
@@ -11965,7 +11965,7 @@
       </c>
       <c r="N144" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O144" t="inlineStr">
@@ -12047,7 +12047,7 @@
       </c>
       <c r="N145" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O145" t="inlineStr">
@@ -12129,7 +12129,7 @@
       </c>
       <c r="N146" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O146" t="inlineStr">
@@ -12293,7 +12293,7 @@
       </c>
       <c r="N148" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O148" t="inlineStr">
@@ -12375,7 +12375,7 @@
       </c>
       <c r="N149" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O149" t="inlineStr">
@@ -12457,7 +12457,7 @@
       </c>
       <c r="N150" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O150" t="inlineStr">
@@ -12703,7 +12703,7 @@
       </c>
       <c r="N153" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O153" t="inlineStr">
@@ -12785,7 +12785,7 @@
       </c>
       <c r="N154" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O154" t="inlineStr">
@@ -12867,7 +12867,7 @@
       </c>
       <c r="N155" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O155" t="inlineStr">
@@ -17196,7 +17196,7 @@
       </c>
       <c r="N207" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O207" t="inlineStr">
@@ -17278,7 +17278,7 @@
       </c>
       <c r="N208" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O208" t="inlineStr">
@@ -18026,7 +18026,7 @@
       </c>
       <c r="N217" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O217" t="inlineStr">
@@ -18118,7 +18118,7 @@
       </c>
       <c r="N218" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O218" t="inlineStr">
@@ -23023,7 +23023,7 @@
       </c>
       <c r="N278" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O278" t="inlineStr">
@@ -27528,7 +27528,7 @@
       </c>
       <c r="N333" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O333" t="inlineStr">
@@ -27620,7 +27620,7 @@
       </c>
       <c r="N334" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O334" t="inlineStr">
@@ -27712,7 +27712,7 @@
       </c>
       <c r="N335" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O335" t="inlineStr">
@@ -27794,7 +27794,7 @@
       </c>
       <c r="N336" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O336" t="inlineStr">

</xml_diff>

<commit_message>
Remove 144 empty spaces from the sheet from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -201,7 +201,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -283,7 +283,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -365,7 +365,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -447,7 +447,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1349,7 +1349,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
@@ -4669,7 +4669,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
@@ -4751,7 +4751,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
@@ -5007,7 +5007,7 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
@@ -5089,7 +5089,7 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
@@ -5181,7 +5181,7 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O62" t="inlineStr">
@@ -5273,7 +5273,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O63" t="inlineStr">
@@ -5365,7 +5365,7 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
@@ -5539,7 +5539,7 @@
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O66" t="inlineStr">
@@ -5621,7 +5621,7 @@
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
@@ -5703,7 +5703,7 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
@@ -5785,7 +5785,7 @@
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
@@ -5867,7 +5867,7 @@
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O70" t="inlineStr">
@@ -5949,7 +5949,7 @@
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O71" t="inlineStr">
@@ -6697,7 +6697,7 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
@@ -8337,7 +8337,7 @@
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M100" t="inlineStr">
@@ -9495,7 +9495,7 @@
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M114" t="inlineStr">
@@ -9577,7 +9577,7 @@
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M115" t="inlineStr">
@@ -9987,7 +9987,7 @@
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M120" t="inlineStr">
@@ -10561,7 +10561,7 @@
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M127" t="inlineStr">
@@ -10643,7 +10643,7 @@
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M128" t="inlineStr">
@@ -11883,7 +11883,7 @@
       </c>
       <c r="N143" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O143" t="inlineStr">
@@ -11965,7 +11965,7 @@
       </c>
       <c r="N144" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O144" t="inlineStr">
@@ -12047,7 +12047,7 @@
       </c>
       <c r="N145" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O145" t="inlineStr">
@@ -12129,7 +12129,7 @@
       </c>
       <c r="N146" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O146" t="inlineStr">
@@ -12293,7 +12293,7 @@
       </c>
       <c r="N148" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O148" t="inlineStr">
@@ -12375,7 +12375,7 @@
       </c>
       <c r="N149" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O149" t="inlineStr">
@@ -12457,7 +12457,7 @@
       </c>
       <c r="N150" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O150" t="inlineStr">
@@ -12703,7 +12703,7 @@
       </c>
       <c r="N153" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O153" t="inlineStr">
@@ -12785,7 +12785,7 @@
       </c>
       <c r="N154" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O154" t="inlineStr">
@@ -12867,7 +12867,7 @@
       </c>
       <c r="N155" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O155" t="inlineStr">
@@ -15352,7 +15352,7 @@
       </c>
       <c r="L185" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M185" t="inlineStr">
@@ -15874,7 +15874,7 @@
       </c>
       <c r="L191" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M191" t="inlineStr">
@@ -16530,7 +16530,7 @@
       </c>
       <c r="L199" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M199" t="inlineStr">
@@ -16612,7 +16612,7 @@
       </c>
       <c r="L200" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M200" t="inlineStr">
@@ -17196,7 +17196,7 @@
       </c>
       <c r="N207" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O207" t="inlineStr">
@@ -17278,7 +17278,7 @@
       </c>
       <c r="N208" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O208" t="inlineStr">
@@ -17432,7 +17432,7 @@
       </c>
       <c r="L210" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M210" t="inlineStr">
@@ -18026,7 +18026,7 @@
       </c>
       <c r="N217" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O217" t="inlineStr">
@@ -18118,7 +18118,7 @@
       </c>
       <c r="N218" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O218" t="inlineStr">
@@ -21547,7 +21547,7 @@
       </c>
       <c r="L260" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M260" t="inlineStr">
@@ -21793,7 +21793,7 @@
       </c>
       <c r="L263" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M263" t="inlineStr">
@@ -22367,7 +22367,7 @@
       </c>
       <c r="L270" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M270" t="inlineStr">
@@ -22449,7 +22449,7 @@
       </c>
       <c r="L271" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M271" t="inlineStr">
@@ -22531,7 +22531,7 @@
       </c>
       <c r="L272" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M272" t="inlineStr">
@@ -22613,7 +22613,7 @@
       </c>
       <c r="L273" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M273" t="inlineStr">
@@ -22695,7 +22695,7 @@
       </c>
       <c r="L274" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M274" t="inlineStr">
@@ -22777,7 +22777,7 @@
       </c>
       <c r="L275" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M275" t="inlineStr">
@@ -23023,7 +23023,7 @@
       </c>
       <c r="N278" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O278" t="inlineStr">
@@ -23095,7 +23095,7 @@
       </c>
       <c r="L279" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M279" t="inlineStr">
@@ -23177,7 +23177,7 @@
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M280" t="inlineStr">
@@ -23259,7 +23259,7 @@
       </c>
       <c r="L281" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M281" t="inlineStr">
@@ -23341,7 +23341,7 @@
       </c>
       <c r="L282" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M282" t="inlineStr">
@@ -23423,7 +23423,7 @@
       </c>
       <c r="L283" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M283" t="inlineStr">
@@ -23505,7 +23505,7 @@
       </c>
       <c r="L284" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M284" t="inlineStr">
@@ -23587,7 +23587,7 @@
       </c>
       <c r="L285" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M285" t="inlineStr">
@@ -23669,7 +23669,7 @@
       </c>
       <c r="L286" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M286" t="inlineStr">
@@ -23751,7 +23751,7 @@
       </c>
       <c r="L287" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M287" t="inlineStr">
@@ -25304,7 +25304,7 @@
       </c>
       <c r="L306" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M306" t="inlineStr">
@@ -25386,7 +25386,7 @@
       </c>
       <c r="L307" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M307" t="inlineStr">
@@ -25468,7 +25468,7 @@
       </c>
       <c r="L308" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M308" t="inlineStr">
@@ -25714,7 +25714,7 @@
       </c>
       <c r="L311" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M311" t="inlineStr">
@@ -25796,7 +25796,7 @@
       </c>
       <c r="L312" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M312" t="inlineStr">
@@ -25878,7 +25878,7 @@
       </c>
       <c r="L313" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M313" t="inlineStr">
@@ -25960,7 +25960,7 @@
       </c>
       <c r="L314" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M314" t="inlineStr">
@@ -27528,7 +27528,7 @@
       </c>
       <c r="N333" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O333" t="inlineStr">
@@ -27620,7 +27620,7 @@
       </c>
       <c r="N334" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O334" t="inlineStr">
@@ -27712,7 +27712,7 @@
       </c>
       <c r="N335" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O335" t="inlineStr">
@@ -27794,7 +27794,7 @@
       </c>
       <c r="N336" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O336" t="inlineStr">
@@ -28107,7 +28107,7 @@
       </c>
       <c r="L340" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M340" t="inlineStr">
@@ -28189,7 +28189,7 @@
       </c>
       <c r="L341" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M341" t="inlineStr">
@@ -28681,7 +28681,7 @@
       </c>
       <c r="L347" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M347" t="inlineStr">
@@ -29009,7 +29009,7 @@
       </c>
       <c r="L351" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M351" t="inlineStr">
@@ -29091,7 +29091,7 @@
       </c>
       <c r="L352" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M352" t="inlineStr">
@@ -29173,7 +29173,7 @@
       </c>
       <c r="L353" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M353" t="inlineStr">
@@ -29255,7 +29255,7 @@
       </c>
       <c r="L354" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M354" t="inlineStr">
@@ -29337,7 +29337,7 @@
       </c>
       <c r="L355" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M355" t="inlineStr">
@@ -29419,7 +29419,7 @@
       </c>
       <c r="L356" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M356" t="inlineStr">
@@ -29665,7 +29665,7 @@
       </c>
       <c r="L359" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="M359" t="inlineStr">

</xml_diff>

<commit_message>
Edit HEK gNT from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -20943,7 +20943,7 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t xml:space="preserve">hek gnt</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
@@ -20988,7 +20988,7 @@
       </c>
       <c r="O253" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R253" t="inlineStr">

</xml_diff>

<commit_message>
Edit HEK ATF3 KO rep2 from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -19892,7 +19892,7 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t xml:space="preserve">hek atf3 ko rep2</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
@@ -31043,7 +31043,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CASPEX Single</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -31053,7 +31053,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -31074,7 +31074,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
+          <t xml:space="preserve">HEK CASPEX Single</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -31084,12 +31084,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E45">
@@ -31105,7 +31105,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh1</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -31115,12 +31115,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E46">
@@ -31136,7 +31136,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh2</t>
+          <t xml:space="preserve">HEK E2F1 sh1</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -31167,7 +31167,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g1</t>
+          <t xml:space="preserve">HEK E2F1 sh2</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -31177,12 +31177,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E48">
@@ -31198,7 +31198,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g2</t>
+          <t xml:space="preserve">HEK FOXA1 KO g1</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -31213,7 +31213,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E49">
@@ -31229,7 +31229,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 OX</t>
+          <t xml:space="preserve">HEK FOXA1 KO g2</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -31244,7 +31244,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E50">
@@ -31260,7 +31260,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g1</t>
+          <t xml:space="preserve">HEK HOXB6 OX</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -31270,12 +31270,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E51">
@@ -31285,13 +31285,13 @@
         <v>0</v>
       </c>
       <c r="G51">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g1</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -31306,7 +31306,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E52">
@@ -31316,13 +31316,13 @@
         <v>0</v>
       </c>
       <c r="G52">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g2</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -31353,7 +31353,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT(20)</t>
+          <t xml:space="preserve">HEK STAT1 KO g2</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -31363,12 +31363,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E54">
@@ -31378,28 +31378,28 @@
         <v>0</v>
       </c>
       <c r="G54">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">HEK gNT(20)</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E55">
@@ -31409,13 +31409,13 @@
         <v>0</v>
       </c>
       <c r="G55">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -31425,7 +31425,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -31446,7 +31446,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -31456,7 +31456,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -31477,17 +31477,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V</t>
+          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -31502,13 +31502,13 @@
         <v>0</v>
       </c>
       <c r="G58">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V 99.17%</t>
+          <t xml:space="preserve">LCC-V</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -31539,12 +31539,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gP2</t>
+          <t xml:space="preserve">LCC-V 99.17%</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -31554,7 +31554,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t xml:space="preserve">gP2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E60">
@@ -31564,18 +31564,18 @@
         <v>0</v>
       </c>
       <c r="G60">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap (m3) (sortER)</t>
+          <t xml:space="preserve">LUCX gP2</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -31585,7 +31585,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gP2</t>
         </is>
       </c>
       <c r="E61">
@@ -31601,7 +31601,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada CASPEX mCherry 1 (no use)</t>
+          <t xml:space="preserve">LnCap (m3) (sortER)</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -31611,7 +31611,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -31632,7 +31632,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canadaa V1G1</t>
+          <t xml:space="preserve">LnCap Canada CASPEX mCherry 1 (no use)</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -31642,7 +31642,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -31663,7 +31663,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select +P+D #1</t>
+          <t xml:space="preserve">LnCap Canadaa V1G1</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -31673,7 +31673,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -31688,13 +31688,13 @@
         <v>0</v>
       </c>
       <c r="G64">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select +P+D #2</t>
+          <t xml:space="preserve">LnCapCASPEX no select +P+D #1</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -31719,13 +31719,13 @@
         <v>0</v>
       </c>
       <c r="G65">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select E</t>
+          <t xml:space="preserve">LnCapCASPEX no select +P+D #2</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -31750,13 +31750,13 @@
         <v>0</v>
       </c>
       <c r="G66">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select H</t>
+          <t xml:space="preserve">LnCapCASPEX no select E</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -31781,23 +31781,23 @@
         <v>0</v>
       </c>
       <c r="G67">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">hek atf3 ko rep2</t>
+          <t xml:space="preserve">LnCapCASPEX no select H</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">

</xml_diff>

<commit_message>
Edit HEK ATF3 OX rep3 from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -20220,7 +20220,7 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t xml:space="preserve">hek atf3 ox rep3</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
@@ -31074,7 +31074,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CASPEX Single</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -31084,7 +31084,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -31105,7 +31105,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
+          <t xml:space="preserve">HEK CASPEX Single</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -31115,12 +31115,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E46">
@@ -31136,7 +31136,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh1</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -31146,12 +31146,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E47">
@@ -31167,7 +31167,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh2</t>
+          <t xml:space="preserve">HEK E2F1 sh1</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -31198,7 +31198,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g1</t>
+          <t xml:space="preserve">HEK E2F1 sh2</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -31208,12 +31208,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E49">
@@ -31229,7 +31229,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g2</t>
+          <t xml:space="preserve">HEK FOXA1 KO g1</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -31244,7 +31244,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E50">
@@ -31260,7 +31260,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 OX</t>
+          <t xml:space="preserve">HEK FOXA1 KO g2</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -31275,7 +31275,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E51">
@@ -31291,7 +31291,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g1</t>
+          <t xml:space="preserve">HEK HOXB6 OX</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -31301,12 +31301,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E52">
@@ -31316,13 +31316,13 @@
         <v>0</v>
       </c>
       <c r="G52">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g1</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -31337,7 +31337,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E53">
@@ -31347,13 +31347,13 @@
         <v>0</v>
       </c>
       <c r="G53">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g2</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -31384,7 +31384,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT(20)</t>
+          <t xml:space="preserve">HEK STAT1 KO g2</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -31394,12 +31394,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E55">
@@ -31409,28 +31409,28 @@
         <v>0</v>
       </c>
       <c r="G55">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">HEK gNT(20)</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E56">
@@ -31440,13 +31440,13 @@
         <v>0</v>
       </c>
       <c r="G56">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -31456,7 +31456,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -31477,7 +31477,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -31487,7 +31487,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -31508,17 +31508,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V</t>
+          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -31533,13 +31533,13 @@
         <v>0</v>
       </c>
       <c r="G59">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V 99.17%</t>
+          <t xml:space="preserve">LCC-V</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -31570,12 +31570,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gP2</t>
+          <t xml:space="preserve">LCC-V 99.17%</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -31585,7 +31585,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t xml:space="preserve">gP2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E61">
@@ -31595,18 +31595,18 @@
         <v>0</v>
       </c>
       <c r="G61">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap (m3) (sortER)</t>
+          <t xml:space="preserve">LUCX gP2</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -31616,7 +31616,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gP2</t>
         </is>
       </c>
       <c r="E62">
@@ -31632,7 +31632,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada CASPEX mCherry 1 (no use)</t>
+          <t xml:space="preserve">LnCap (m3) (sortER)</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -31642,7 +31642,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -31663,7 +31663,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canadaa V1G1</t>
+          <t xml:space="preserve">LnCap Canada CASPEX mCherry 1 (no use)</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -31673,7 +31673,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -31694,7 +31694,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select +P+D #1</t>
+          <t xml:space="preserve">LnCap Canadaa V1G1</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -31704,7 +31704,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -31719,13 +31719,13 @@
         <v>0</v>
       </c>
       <c r="G65">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select +P+D #2</t>
+          <t xml:space="preserve">LnCapCASPEX no select +P+D #1</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -31750,13 +31750,13 @@
         <v>0</v>
       </c>
       <c r="G66">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select E</t>
+          <t xml:space="preserve">LnCapCASPEX no select +P+D #2</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -31781,13 +31781,13 @@
         <v>0</v>
       </c>
       <c r="G67">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select H</t>
+          <t xml:space="preserve">LnCapCASPEX no select E</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -31812,23 +31812,23 @@
         <v>0</v>
       </c>
       <c r="G68">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">hek atf3 ox rep3</t>
+          <t xml:space="preserve">LnCapCASPEX no select H</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">

</xml_diff>

<commit_message>
Edit LnCapCASPEX no select E from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -20302,7 +20302,7 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">hek atf3 ox rep3</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
@@ -28087,12 +28087,12 @@
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t xml:space="preserve">p45769</t>
+          <t xml:space="preserve">p?</t>
         </is>
       </c>
       <c r="G340" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H340" t="inlineStr">

</xml_diff>

<commit_message>
Add a guide rule
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -4356,7 +4356,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">sh</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -4520,7 +4520,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">sh</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">sh</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
@@ -6210,7 +6210,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">sh</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">

</xml_diff>

<commit_message>
Add 1 × klm ox from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -29039,39 +29039,49 @@
       </c>
     </row>
     <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unnamed box</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A1</t>
+        </is>
+      </c>
       <c r="E352" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
-        </is>
-      </c>
-      <c r="F352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="G352" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H352" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I352" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="K352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L352" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M352" t="inlineStr">
@@ -29086,24 +29096,24 @@
       </c>
       <c r="O352" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R352" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">stored</t>
         </is>
       </c>
       <c r="S352" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="E353" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F353" t="inlineStr">
@@ -29133,7 +29143,7 @@
       </c>
       <c r="L353" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M353" t="inlineStr">
@@ -29148,7 +29158,7 @@
       </c>
       <c r="O353" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R353" t="inlineStr">
@@ -29158,14 +29168,14 @@
       </c>
       <c r="S353" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="E354" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F354" t="inlineStr">
@@ -29195,7 +29205,7 @@
       </c>
       <c r="L354" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M354" t="inlineStr">
@@ -29220,19 +29230,19 @@
       </c>
       <c r="S354" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="E355" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F355" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G355" t="inlineStr">
@@ -29257,7 +29267,7 @@
       </c>
       <c r="L355" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M355" t="inlineStr">
@@ -29282,19 +29292,19 @@
       </c>
       <c r="S355" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="E356" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
@@ -29314,12 +29324,12 @@
       </c>
       <c r="K356" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L356" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M356" t="inlineStr">
@@ -29334,7 +29344,7 @@
       </c>
       <c r="O356" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R356" t="inlineStr">
@@ -29344,19 +29354,19 @@
       </c>
       <c r="S356" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="E357" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
@@ -29381,7 +29391,7 @@
       </c>
       <c r="L357" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M357" t="inlineStr">
@@ -29396,7 +29406,7 @@
       </c>
       <c r="O357" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R357" t="inlineStr">
@@ -29406,19 +29416,19 @@
       </c>
       <c r="S357" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="E358" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
@@ -29443,7 +29453,7 @@
       </c>
       <c r="L358" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M358" t="inlineStr">
@@ -29468,19 +29478,19 @@
       </c>
       <c r="S358" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="E359" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
@@ -29505,7 +29515,7 @@
       </c>
       <c r="L359" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M359" t="inlineStr">
@@ -29530,67 +29540,129 @@
       </c>
       <c r="S359" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="E360" t="inlineStr">
         <is>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K360" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L360" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OX</t>
+        </is>
+      </c>
+      <c r="M360" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N360" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O360" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R360" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S360" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="E361" t="inlineStr">
+        <is>
           <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
-      <c r="F360" t="inlineStr">
+      <c r="F361" t="inlineStr">
         <is>
           <t xml:space="preserve">p6</t>
         </is>
       </c>
-      <c r="G360" t="inlineStr">
+      <c r="G361" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H360" t="inlineStr">
+      <c r="H361" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
-      <c r="I360" t="inlineStr">
+      <c r="I361" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
-      <c r="K360" t="inlineStr">
+      <c r="K361" t="inlineStr">
         <is>
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L360" t="inlineStr">
+      <c r="L361" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M360" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="N360" t="inlineStr">
+      <c r="M361" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N361" t="inlineStr">
         <is>
           <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
-      <c r="O360" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="R360" t="inlineStr">
+      <c r="O361" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R361" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
-      <c r="S360" t="inlineStr">
+      <c r="S361" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mtski3re-0</t>
         </is>
@@ -34004,16 +34076,32 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
+          <t xml:space="preserve">klm ox</t>
+        </is>
+      </c>
+      <c r="E143">
+        <v>1</v>
+      </c>
+      <c r="F143">
+        <v>0</v>
+      </c>
+      <c r="G143">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
           <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
-      <c r="E143">
+      <c r="E144">
         <v>0</v>
       </c>
-      <c r="F143">
+      <c r="F144">
         <v>1</v>
       </c>
-      <c r="G143">
+      <c r="G144">
         <v>0</v>
       </c>
     </row>
@@ -34774,10 +34862,10 @@
         <v>81</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Add 3 × jkl from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -29111,34 +29111,44 @@
       </c>
     </row>
     <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unnamed box</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A2</t>
+        </is>
+      </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
-        </is>
-      </c>
-      <c r="F353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H353" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I353" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="K353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L353" t="inlineStr">
@@ -29158,54 +29168,64 @@
       </c>
       <c r="O353" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R353" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">stored</t>
         </is>
       </c>
       <c r="S353" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
     <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unnamed box</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A3</t>
+        </is>
+      </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
-        </is>
-      </c>
-      <c r="F354" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G354" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H354" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I354" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="K354" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L354" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M354" t="inlineStr">
@@ -29225,49 +29245,59 @@
       </c>
       <c r="R354" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">stored</t>
         </is>
       </c>
       <c r="S354" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
     <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unnamed box</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A4</t>
+        </is>
+      </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
-        </is>
-      </c>
-      <c r="F355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H355" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I355" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="K355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L355" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M355" t="inlineStr">
@@ -29287,24 +29317,24 @@
       </c>
       <c r="R355" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">stored</t>
         </is>
       </c>
       <c r="S355" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="E356" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
@@ -29329,7 +29359,7 @@
       </c>
       <c r="L356" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M356" t="inlineStr">
@@ -29344,7 +29374,7 @@
       </c>
       <c r="O356" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R356" t="inlineStr">
@@ -29354,19 +29384,19 @@
       </c>
       <c r="S356" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="E357" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
@@ -29386,12 +29416,12 @@
       </c>
       <c r="K357" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L357" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M357" t="inlineStr">
@@ -29406,7 +29436,7 @@
       </c>
       <c r="O357" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R357" t="inlineStr">
@@ -29416,19 +29446,19 @@
       </c>
       <c r="S357" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="E358" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
@@ -29448,12 +29478,12 @@
       </c>
       <c r="K358" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L358" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M358" t="inlineStr">
@@ -29478,19 +29508,19 @@
       </c>
       <c r="S358" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="E359" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
@@ -29510,12 +29540,12 @@
       </c>
       <c r="K359" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L359" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M359" t="inlineStr">
@@ -29540,19 +29570,19 @@
       </c>
       <c r="S359" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="E360" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
@@ -29577,7 +29607,7 @@
       </c>
       <c r="L360" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M360" t="inlineStr">
@@ -29592,7 +29622,7 @@
       </c>
       <c r="O360" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R360" t="inlineStr">
@@ -29602,67 +29632,253 @@
       </c>
       <c r="S360" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="E361" t="inlineStr">
         <is>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K361" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L361" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KO</t>
+        </is>
+      </c>
+      <c r="M361" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N361" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O361" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R361" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S361" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtre0daw-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="E362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p17</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FLAG</t>
+        </is>
+      </c>
+      <c r="M362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="E363" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K363" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L363" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OX</t>
+        </is>
+      </c>
+      <c r="M363" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N363" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O363" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R363" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S363" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="E364" t="inlineStr">
+        <is>
           <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
-      <c r="F361" t="inlineStr">
+      <c r="F364" t="inlineStr">
         <is>
           <t xml:space="preserve">p6</t>
         </is>
       </c>
-      <c r="G361" t="inlineStr">
+      <c r="G364" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H361" t="inlineStr">
+      <c r="H364" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
-      <c r="I361" t="inlineStr">
+      <c r="I364" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
-      <c r="K361" t="inlineStr">
+      <c r="K364" t="inlineStr">
         <is>
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L361" t="inlineStr">
+      <c r="L364" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M361" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="N361" t="inlineStr">
+      <c r="M364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N364" t="inlineStr">
         <is>
           <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
-      <c r="O361" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="R361" t="inlineStr">
+      <c r="O364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R364" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
-      <c r="S361" t="inlineStr">
+      <c r="S364" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mtski3re-0</t>
         </is>
@@ -30707,26 +30923,11 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 TOX4 KO g2.2</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OX</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">g2.2</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="E34">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F34">
         <v>0</v>
@@ -30738,7 +30939,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR</t>
+          <t xml:space="preserve">Du145 TOX4 KO g2.2</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -30748,12 +30949,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2.2</t>
         </is>
       </c>
       <c r="E35">
@@ -30769,7 +30970,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATF3 KO</t>
+          <t xml:space="preserve">DuDtxR</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -30779,7 +30980,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -30800,7 +31001,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATP7B KO</t>
+          <t xml:space="preserve">DuPar50CR ATF3 KO</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -30831,7 +31032,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR MTF1 KO</t>
+          <t xml:space="preserve">DuPar50CR ATP7B KO</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -30862,7 +31063,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR NT KO</t>
+          <t xml:space="preserve">DuPar50CR MTF1 KO</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -30893,7 +31094,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2</t>
+          <t xml:space="preserve">DuPar50CR NT KO</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -30903,12 +31104,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E40">
@@ -30924,7 +31125,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2</t>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -30939,7 +31140,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2.2</t>
+          <t xml:space="preserve">g1.2</t>
         </is>
       </c>
       <c r="E41">
@@ -30955,22 +31156,22 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CASPEX Single</t>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2.2</t>
         </is>
       </c>
       <c r="E42">
@@ -30986,7 +31187,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
+          <t xml:space="preserve">HEK CASPEX Single</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -30996,12 +31197,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E43">
@@ -31017,7 +31218,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh1</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -31027,12 +31228,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E44">
@@ -31048,7 +31249,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh2</t>
+          <t xml:space="preserve">HEK E2F1 sh1</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -31079,7 +31280,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g1</t>
+          <t xml:space="preserve">HEK E2F1 sh2</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -31089,12 +31290,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E46">
@@ -31110,7 +31311,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g2</t>
+          <t xml:space="preserve">HEK FOXA1 KO g1</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -31125,7 +31326,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E47">
@@ -31141,7 +31342,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 OX</t>
+          <t xml:space="preserve">HEK FOXA1 KO g2</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -31156,7 +31357,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E48">
@@ -31172,7 +31373,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g1</t>
+          <t xml:space="preserve">HEK HOXB6 OX</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -31182,12 +31383,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E49">
@@ -31197,13 +31398,13 @@
         <v>0</v>
       </c>
       <c r="G49">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g1</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -31218,7 +31419,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E50">
@@ -31228,13 +31429,13 @@
         <v>0</v>
       </c>
       <c r="G50">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g2</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -31265,7 +31466,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT(20)</t>
+          <t xml:space="preserve">HEK STAT1 KO g2</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -31275,12 +31476,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E52">
@@ -31290,35 +31491,35 @@
         <v>0</v>
       </c>
       <c r="G52">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK gNT(20)</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E53">
         <v>2</v>
       </c>
       <c r="F53">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G53">
         <v>2</v>
@@ -31327,7 +31528,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -31337,7 +31538,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -31349,16 +31550,16 @@
         <v>2</v>
       </c>
       <c r="F54">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G54">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -31368,33 +31569,33 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E55">
         <v>2</v>
       </c>
       <c r="F55">
+        <v>0</v>
+      </c>
+      <c r="G55">
         <v>1</v>
-      </c>
-      <c r="G55">
-        <v>2</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -31404,14 +31605,14 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E56">
         <v>2</v>
       </c>
       <c r="F56">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G56">
         <v>2</v>
@@ -31420,7 +31621,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V 99.17%</t>
+          <t xml:space="preserve">LCC-V</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -31451,12 +31652,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gP2</t>
+          <t xml:space="preserve">LCC-V 99.17%</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -31466,7 +31667,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t xml:space="preserve">gP2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E58">
@@ -31476,18 +31677,18 @@
         <v>0</v>
       </c>
       <c r="G58">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap (m3) (sortER)</t>
+          <t xml:space="preserve">LUCX gP2</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -31497,7 +31698,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gP2</t>
         </is>
       </c>
       <c r="E59">
@@ -31513,7 +31714,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada CASPEX mCherry 1 (no use)</t>
+          <t xml:space="preserve">LnCap (m3) (sortER)</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -31523,7 +31724,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -31544,7 +31745,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canadaa V1G1</t>
+          <t xml:space="preserve">LnCap Canada CASPEX mCherry 1 (no use)</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -31554,7 +31755,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -31575,7 +31776,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select +P+D #1</t>
+          <t xml:space="preserve">LnCap Canadaa V1G1</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -31585,7 +31786,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -31600,13 +31801,13 @@
         <v>0</v>
       </c>
       <c r="G62">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select +P+D #2</t>
+          <t xml:space="preserve">LnCapCASPEX no select +P+D #1</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -31631,13 +31832,13 @@
         <v>0</v>
       </c>
       <c r="G63">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select E</t>
+          <t xml:space="preserve">LnCapCASPEX no select +P+D #2</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -31662,13 +31863,13 @@
         <v>0</v>
       </c>
       <c r="G64">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select H</t>
+          <t xml:space="preserve">LnCapCASPEX no select E</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -31693,23 +31894,23 @@
         <v>0</v>
       </c>
       <c r="G65">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 ATF3 KO rep2</t>
+          <t xml:space="preserve">LnCapCASPEX no select H</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -31718,7 +31919,7 @@
         </is>
       </c>
       <c r="E66">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F66">
         <v>0</v>
@@ -31730,7 +31931,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 ATF3 OX rep2</t>
+          <t xml:space="preserve">Du145 ATF3 KO rep2</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -31740,7 +31941,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -31761,7 +31962,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEXe g3</t>
+          <t xml:space="preserve">Du145 ATF3 OX rep2</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -31771,12 +31972,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t xml:space="preserve">g3</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E68">
@@ -31792,22 +31993,22 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK APEX1 KO g2</t>
+          <t xml:space="preserve">DuDtxR CASPEXe g3</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g3</t>
         </is>
       </c>
       <c r="E69">
@@ -31823,7 +32024,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK APEX1 OX</t>
+          <t xml:space="preserve">HEK APEX1 KO g2</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -31833,12 +32034,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E70">
@@ -31854,7 +32055,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK APEX1 g1</t>
+          <t xml:space="preserve">HEK APEX1 OX</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -31864,12 +32065,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E71">
@@ -31885,7 +32086,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO 20</t>
+          <t xml:space="preserve">HEK APEX1 g1</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -31895,12 +32096,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E72">
@@ -31916,7 +32117,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">HEK ATF3 KO 20</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -31938,7 +32139,7 @@
         <v>1</v>
       </c>
       <c r="F73">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G73">
         <v>1</v>
@@ -31947,7 +32148,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO10</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -31969,7 +32170,7 @@
         <v>1</v>
       </c>
       <c r="F74">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G74">
         <v>1</v>
@@ -31978,7 +32179,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX</t>
+          <t xml:space="preserve">HEK ATF3 KO10</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -31988,7 +32189,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -32009,7 +32210,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep2</t>
+          <t xml:space="preserve">HEK ATF3 OX</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -32040,7 +32241,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK ATF3 OX rep2</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -32062,7 +32263,7 @@
         <v>1</v>
       </c>
       <c r="F77">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G77">
         <v>1</v>
@@ -32071,7 +32272,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX10r1</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -32093,7 +32294,7 @@
         <v>1</v>
       </c>
       <c r="F78">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G78">
         <v>1</v>
@@ -32102,7 +32303,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX20r1</t>
+          <t xml:space="preserve">HEK ATF3 OX10r1</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -32133,7 +32334,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3OX10r1</t>
+          <t xml:space="preserve">HEK ATF3 OX20r1</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -32164,7 +32365,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO-1</t>
+          <t xml:space="preserve">HEK ATF3OX10r1</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -32174,7 +32375,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -32195,7 +32396,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO-2</t>
+          <t xml:space="preserve">HEK ATP7B KO-1</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -32226,7 +32427,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO-3</t>
+          <t xml:space="preserve">HEK ATP7B KO-2</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -32257,7 +32458,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CASPEX gNT</t>
+          <t xml:space="preserve">HEK ATP7B KO-3</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -32267,12 +32468,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E84">
@@ -32288,7 +32489,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 plv-GFP</t>
+          <t xml:space="preserve">HEK CASPEX gNT</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -32298,12 +32499,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E85">
@@ -32319,7 +32520,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 OX</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 plv-GFP</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -32329,12 +32530,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E86">
@@ -32350,7 +32551,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK GATA6 KO g1</t>
+          <t xml:space="preserve">HEK CBX3 OX</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -32360,12 +32561,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E87">
@@ -32381,7 +32582,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK GATA6 KO g2</t>
+          <t xml:space="preserve">HEK GATA6 KO g1</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -32396,7 +32597,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E88">
@@ -32412,7 +32613,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 KO g2</t>
+          <t xml:space="preserve">HEK GATA6 KO g2</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -32422,7 +32623,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -32443,7 +32644,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK JUN KO g1</t>
+          <t xml:space="preserve">HEK HOXB6 KO g2</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -32453,12 +32654,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E90">
@@ -32474,7 +32675,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK JUN KO g2</t>
+          <t xml:space="preserve">HEK JUN KO g1</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -32489,7 +32690,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E91">
@@ -32505,7 +32706,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK JUN1 KO g2</t>
+          <t xml:space="preserve">HEK JUN KO g2</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -32536,7 +32737,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK NRF2 KO g1</t>
+          <t xml:space="preserve">HEK JUN1 KO g2</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -32551,7 +32752,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E93">
@@ -32567,7 +32768,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK NRF2 KO g2</t>
+          <t xml:space="preserve">HEK NRF2 KO g1</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -32582,7 +32783,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E94">
@@ -32598,7 +32799,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK RFX KO g1</t>
+          <t xml:space="preserve">HEK NRF2 KO g2</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -32613,7 +32814,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E95">
@@ -32629,7 +32830,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK RFX KO g2</t>
+          <t xml:space="preserve">HEK RFX KO g1</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -32644,7 +32845,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E96">
@@ -32660,7 +32861,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK SMARCE1 KO g1</t>
+          <t xml:space="preserve">HEK RFX KO g2</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -32675,7 +32876,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E97">
@@ -32691,7 +32892,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK SMARCE1 KO g2</t>
+          <t xml:space="preserve">HEK SMARCE1 KO g1</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -32706,7 +32907,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E98">
@@ -32722,7 +32923,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK SPEN KO g2</t>
+          <t xml:space="preserve">HEK SMARCE1 KO g2</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -32753,7 +32954,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g1</t>
+          <t xml:space="preserve">HEK SPEN KO g2</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -32768,7 +32969,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E100">
@@ -32784,7 +32985,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK TOX4 OX 3xFLAG</t>
+          <t xml:space="preserve">HEK STAT1 KO g1</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -32794,12 +32995,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E101">
@@ -32815,7 +33016,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT (10)</t>
+          <t xml:space="preserve">HEK TOX4 OX 3xFLAG</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -32825,12 +33026,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E102">
@@ -32846,7 +33047,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK lef1 OX</t>
+          <t xml:space="preserve">HEK gNT (10)</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -32856,12 +33057,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E103">
@@ -32877,17 +33078,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep2</t>
+          <t xml:space="preserve">HEK lef1 OX</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -32908,7 +33109,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep2</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -32930,7 +33131,7 @@
         <v>1</v>
       </c>
       <c r="F105">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G105">
         <v>1</v>
@@ -32939,7 +33140,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO20</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -32961,7 +33162,7 @@
         <v>1</v>
       </c>
       <c r="F106">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G106">
         <v>1</v>
@@ -32970,7 +33171,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep2</t>
+          <t xml:space="preserve">Huh7 ATF3 KO20</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -32980,7 +33181,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -33001,7 +33202,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep2</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -33023,7 +33224,7 @@
         <v>1</v>
       </c>
       <c r="F108">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G108">
         <v>1</v>
@@ -33032,7 +33233,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX20r1</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -33054,7 +33255,7 @@
         <v>1</v>
       </c>
       <c r="F109">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G109">
         <v>1</v>
@@ -33063,7 +33264,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3KO10</t>
+          <t xml:space="preserve">Huh7 ATF3 OX20r1</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -33073,7 +33274,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -33094,7 +33295,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATP7B KO</t>
+          <t xml:space="preserve">Huh7 ATF3KO10</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -33125,7 +33326,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 CASPEX gNT</t>
+          <t xml:space="preserve">Huh7 ATP7B KO</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -33135,12 +33336,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E112">
@@ -33156,7 +33357,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 CBX3 KO g1</t>
+          <t xml:space="preserve">Huh7 CASPEX gNT</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -33166,12 +33367,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E113">
@@ -33187,7 +33388,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 CBX3 KO g2</t>
+          <t xml:space="preserve">Huh7 CBX3 KO g1</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -33202,7 +33403,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E114">
@@ -33218,7 +33419,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 CBX3 OX</t>
+          <t xml:space="preserve">Huh7 CBX3 KO g2</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -33228,12 +33429,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E115">
@@ -33249,7 +33450,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 HOXB6 KO g1</t>
+          <t xml:space="preserve">Huh7 CBX3 OX</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -33264,7 +33465,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E116">
@@ -33280,7 +33481,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 HOXB6 OX</t>
+          <t xml:space="preserve">Huh7 HOXB6 KO g1</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -33295,7 +33496,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E117">
@@ -33311,7 +33512,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 POU3F2 KO g1</t>
+          <t xml:space="preserve">Huh7 HOXB6 OX</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -33321,12 +33522,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E118">
@@ -33342,7 +33543,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 POU3F3 KO g1</t>
+          <t xml:space="preserve">Huh7 POU3F2 KO g1</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -33373,7 +33574,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 POU3F3 KO g2</t>
+          <t xml:space="preserve">Huh7 POU3F3 KO g1</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -33388,7 +33589,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E120">
@@ -33404,7 +33605,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 TOX4 KO g1</t>
+          <t xml:space="preserve">Huh7 POU3F3 KO g2</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -33414,12 +33615,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E121">
@@ -33435,7 +33636,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 TOX4 OX</t>
+          <t xml:space="preserve">Huh7 TOX4 KO g1</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -33450,7 +33651,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E122">
@@ -33466,7 +33667,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 lef1 OX</t>
+          <t xml:space="preserve">Huh7 TOX4 OX</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -33497,17 +33698,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-C*</t>
+          <t xml:space="preserve">Huh7 lef1 OX</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -33528,7 +33729,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-E</t>
+          <t xml:space="preserve">LCC-C*</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -33559,7 +33760,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-H</t>
+          <t xml:space="preserve">LCC-E</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -33590,7 +33791,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNC478 #1</t>
+          <t xml:space="preserve">LCC-H</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -33621,7 +33822,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNC478 #2 98%</t>
+          <t xml:space="preserve">LNC478 #1</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -33652,7 +33853,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNC478 #3</t>
+          <t xml:space="preserve">LNC478 #2 98%</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -33683,7 +33884,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCAP BMK</t>
+          <t xml:space="preserve">LNC478 #3</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -33714,7 +33915,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap (m3) no sort</t>
+          <t xml:space="preserve">LNCAP BMK</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -33745,7 +33946,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G2</t>
+          <t xml:space="preserve">LnCap (m3) no sort</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -33776,7 +33977,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G3</t>
+          <t xml:space="preserve">LnCap Canada V1G2</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -33807,7 +34008,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G4</t>
+          <t xml:space="preserve">LnCap Canada V1G3</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -33838,7 +34039,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap ER</t>
+          <t xml:space="preserve">LnCap Canada V1G4</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -33869,7 +34070,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap V1G1</t>
+          <t xml:space="preserve">LnCap ER</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -33900,7 +34101,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap478 #2 98%</t>
+          <t xml:space="preserve">LnCap V1G1</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -33931,7 +34132,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select</t>
+          <t xml:space="preserve">LnCap478 #2 98%</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -33941,7 +34142,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -33962,7 +34163,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select C</t>
+          <t xml:space="preserve">LnCapCASPEX no select</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -33993,17 +34194,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap (m1) no sort</t>
+          <t xml:space="preserve">LnCapCASPEX no select C</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -34024,7 +34225,12 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDA-MB g1.1 p10</t>
+          <t xml:space="preserve">LuCap (m1) no sort</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -34034,7 +34240,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E141">
@@ -34050,7 +34256,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDA-MB gNT</t>
+          <t xml:space="preserve">MDA-MB g1.1 p10</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -34060,7 +34266,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g1.1</t>
         </is>
       </c>
       <c r="E142">
@@ -34076,7 +34282,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">MDA-MB gNT</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E143">
@@ -34092,16 +34308,32 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
+          <t xml:space="preserve">klm ox</t>
+        </is>
+      </c>
+      <c r="E144">
+        <v>1</v>
+      </c>
+      <c r="F144">
+        <v>0</v>
+      </c>
+      <c r="G144">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
           <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
-      <c r="E144">
+      <c r="E145">
         <v>0</v>
       </c>
-      <c r="F144">
+      <c r="F145">
         <v>1</v>
       </c>
-      <c r="G144">
+      <c r="G145">
         <v>0</v>
       </c>
     </row>
@@ -34862,10 +35094,10 @@
         <v>81</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J7">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Add 1 × khk from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -29327,34 +29327,44 @@
       </c>
     </row>
     <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unnamed box</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D4</t>
+        </is>
+      </c>
       <c r="E356" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
-        </is>
-      </c>
-      <c r="F356" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H356" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I356" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="K356" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L356" t="inlineStr">
@@ -29374,24 +29384,24 @@
       </c>
       <c r="O356" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R356" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">stored</t>
         </is>
       </c>
       <c r="S356" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
+          <t xml:space="preserve">v-mtt5ckqo-0</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="E357" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
@@ -29421,7 +29431,7 @@
       </c>
       <c r="L357" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M357" t="inlineStr">
@@ -29436,7 +29446,7 @@
       </c>
       <c r="O357" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R357" t="inlineStr">
@@ -29446,14 +29456,14 @@
       </c>
       <c r="S357" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="E358" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
@@ -29483,7 +29493,7 @@
       </c>
       <c r="L358" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M358" t="inlineStr">
@@ -29508,19 +29518,19 @@
       </c>
       <c r="S358" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="E359" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
@@ -29545,7 +29555,7 @@
       </c>
       <c r="L359" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M359" t="inlineStr">
@@ -29570,19 +29580,19 @@
       </c>
       <c r="S359" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="E360" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
@@ -29602,12 +29612,12 @@
       </c>
       <c r="K360" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L360" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M360" t="inlineStr">
@@ -29622,7 +29632,7 @@
       </c>
       <c r="O360" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R360" t="inlineStr">
@@ -29632,19 +29642,19 @@
       </c>
       <c r="S360" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="E361" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="F361" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
@@ -29669,7 +29679,7 @@
       </c>
       <c r="L361" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M361" t="inlineStr">
@@ -29684,7 +29694,7 @@
       </c>
       <c r="O361" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R361" t="inlineStr">
@@ -29694,19 +29704,19 @@
       </c>
       <c r="S361" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="E362" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G362" t="inlineStr">
@@ -29731,7 +29741,7 @@
       </c>
       <c r="L362" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M362" t="inlineStr">
@@ -29756,19 +29766,19 @@
       </c>
       <c r="S362" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="E363" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
@@ -29793,7 +29803,7 @@
       </c>
       <c r="L363" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M363" t="inlineStr">
@@ -29818,67 +29828,129 @@
       </c>
       <c r="S363" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="E364" t="inlineStr">
         <is>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OX</t>
+        </is>
+      </c>
+      <c r="M364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="E365" t="inlineStr">
+        <is>
           <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
-      <c r="F364" t="inlineStr">
+      <c r="F365" t="inlineStr">
         <is>
           <t xml:space="preserve">p6</t>
         </is>
       </c>
-      <c r="G364" t="inlineStr">
+      <c r="G365" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H364" t="inlineStr">
+      <c r="H365" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
-      <c r="I364" t="inlineStr">
+      <c r="I365" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
-      <c r="K364" t="inlineStr">
+      <c r="K365" t="inlineStr">
         <is>
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L364" t="inlineStr">
+      <c r="L365" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M364" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="N364" t="inlineStr">
+      <c r="M365" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N365" t="inlineStr">
         <is>
           <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
-      <c r="O364" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="R364" t="inlineStr">
+      <c r="O365" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R365" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
-      <c r="S364" t="inlineStr">
+      <c r="S365" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mtski3re-0</t>
         </is>
@@ -34308,7 +34380,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="E144">
@@ -34324,16 +34396,32 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
+          <t xml:space="preserve">klm ox</t>
+        </is>
+      </c>
+      <c r="E145">
+        <v>1</v>
+      </c>
+      <c r="F145">
+        <v>0</v>
+      </c>
+      <c r="G145">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
           <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
-      <c r="E145">
+      <c r="E146">
         <v>0</v>
       </c>
-      <c r="F145">
+      <c r="F146">
         <v>1</v>
       </c>
-      <c r="G145">
+      <c r="G146">
         <v>0</v>
       </c>
     </row>
@@ -35094,10 +35182,10 @@
         <v>81</v>
       </c>
       <c r="I7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J7">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Take out khk from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -29327,44 +29327,34 @@
       </c>
     </row>
     <row r="356">
-      <c r="A356" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Freezer 1</t>
-        </is>
-      </c>
-      <c r="B356" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rack 1</t>
-        </is>
-      </c>
-      <c r="C356" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Unnamed box</t>
-        </is>
-      </c>
-      <c r="D356" t="inlineStr">
-        <is>
-          <t xml:space="preserve">D4</t>
-        </is>
-      </c>
       <c r="E356" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">HEK gNT</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H356" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I356" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K356" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L356" t="inlineStr">
@@ -29384,24 +29374,24 @@
       </c>
       <c r="O356" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R356" t="inlineStr">
         <is>
-          <t xml:space="preserve">stored</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="S356" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt5ckqo-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="E357" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
@@ -29431,7 +29421,7 @@
       </c>
       <c r="L357" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M357" t="inlineStr">
@@ -29446,7 +29436,7 @@
       </c>
       <c r="O357" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R357" t="inlineStr">
@@ -29456,14 +29446,14 @@
       </c>
       <c r="S357" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="E358" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
@@ -29493,7 +29483,7 @@
       </c>
       <c r="L358" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M358" t="inlineStr">
@@ -29518,19 +29508,19 @@
       </c>
       <c r="S358" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="E359" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
@@ -29555,7 +29545,7 @@
       </c>
       <c r="L359" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M359" t="inlineStr">
@@ -29580,19 +29570,19 @@
       </c>
       <c r="S359" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="E360" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
@@ -29612,12 +29602,12 @@
       </c>
       <c r="K360" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L360" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M360" t="inlineStr">
@@ -29632,7 +29622,7 @@
       </c>
       <c r="O360" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R360" t="inlineStr">
@@ -29642,19 +29632,19 @@
       </c>
       <c r="S360" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="E361" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="F361" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
@@ -29679,7 +29669,7 @@
       </c>
       <c r="L361" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M361" t="inlineStr">
@@ -29694,7 +29684,7 @@
       </c>
       <c r="O361" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R361" t="inlineStr">
@@ -29704,19 +29694,19 @@
       </c>
       <c r="S361" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="E362" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G362" t="inlineStr">
@@ -29741,7 +29731,7 @@
       </c>
       <c r="L362" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M362" t="inlineStr">
@@ -29766,19 +29756,19 @@
       </c>
       <c r="S362" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="E363" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
@@ -29803,7 +29793,7 @@
       </c>
       <c r="L363" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M363" t="inlineStr">
@@ -29828,19 +29818,19 @@
       </c>
       <c r="S363" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="E364" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G364" t="inlineStr">
@@ -29850,22 +29840,22 @@
       </c>
       <c r="H364" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I364" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="K364" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L364" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M364" t="inlineStr">
@@ -29875,7 +29865,7 @@
       </c>
       <c r="N364" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O364" t="inlineStr">
@@ -29890,24 +29880,19 @@
       </c>
       <c r="S364" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="E365" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
-        </is>
-      </c>
-      <c r="F365" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="G365" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H365" t="inlineStr">
@@ -29920,11 +29905,6 @@
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
-      <c r="K365" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
       <c r="L365" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -29937,7 +29917,7 @@
       </c>
       <c r="N365" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O365" t="inlineStr">
@@ -29952,7 +29932,7 @@
       </c>
       <c r="S365" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtt5ckqo-0</t>
         </is>
       </c>
     </row>
@@ -34380,7 +34360,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="E144">
@@ -34396,23 +34376,23 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
       <c r="E145">
+        <v>0</v>
+      </c>
+      <c r="F145">
         <v>1</v>
       </c>
-      <c r="F145">
+      <c r="G145">
         <v>0</v>
-      </c>
-      <c r="G145">
-        <v>1</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="E146">
@@ -34907,6 +34887,53 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">khk</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unnamed box</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D4</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown device</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt5ckqo-0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -35182,10 +35209,10 @@
         <v>81</v>
       </c>
       <c r="I7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J7">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Take out klm ox from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -29056,12 +29056,12 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">A2</t>
         </is>
       </c>
       <c r="E352" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G352" t="inlineStr">
@@ -29081,7 +29081,7 @@
       </c>
       <c r="L352" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M352" t="inlineStr">
@@ -29106,7 +29106,7 @@
       </c>
       <c r="S352" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
@@ -29128,7 +29128,7 @@
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">A3</t>
         </is>
       </c>
       <c r="E353" t="inlineStr">
@@ -29178,7 +29178,7 @@
       </c>
       <c r="S353" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
@@ -29200,7 +29200,7 @@
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">A4</t>
         </is>
       </c>
       <c r="E354" t="inlineStr">
@@ -29250,49 +29250,39 @@
       </c>
       <c r="S354" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
       </c>
     </row>
     <row r="355">
-      <c r="A355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Freezer 1</t>
-        </is>
-      </c>
-      <c r="B355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rack 1</t>
-        </is>
-      </c>
-      <c r="C355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Unnamed box</t>
-        </is>
-      </c>
-      <c r="D355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A4</t>
-        </is>
-      </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">HEK gNT</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H355" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I355" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L355" t="inlineStr">
@@ -29312,24 +29302,24 @@
       </c>
       <c r="O355" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R355" t="inlineStr">
         <is>
-          <t xml:space="preserve">stored</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="S355" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="E356" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F356" t="inlineStr">
@@ -29359,7 +29349,7 @@
       </c>
       <c r="L356" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M356" t="inlineStr">
@@ -29374,7 +29364,7 @@
       </c>
       <c r="O356" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R356" t="inlineStr">
@@ -29384,14 +29374,14 @@
       </c>
       <c r="S356" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="E357" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
@@ -29421,7 +29411,7 @@
       </c>
       <c r="L357" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M357" t="inlineStr">
@@ -29446,19 +29436,19 @@
       </c>
       <c r="S357" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="E358" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
@@ -29483,7 +29473,7 @@
       </c>
       <c r="L358" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M358" t="inlineStr">
@@ -29508,19 +29498,19 @@
       </c>
       <c r="S358" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="E359" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
@@ -29540,12 +29530,12 @@
       </c>
       <c r="K359" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L359" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M359" t="inlineStr">
@@ -29560,7 +29550,7 @@
       </c>
       <c r="O359" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R359" t="inlineStr">
@@ -29570,19 +29560,19 @@
       </c>
       <c r="S359" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="E360" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
@@ -29607,7 +29597,7 @@
       </c>
       <c r="L360" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M360" t="inlineStr">
@@ -29622,7 +29612,7 @@
       </c>
       <c r="O360" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R360" t="inlineStr">
@@ -29632,19 +29622,19 @@
       </c>
       <c r="S360" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="E361" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="F361" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
@@ -29669,7 +29659,7 @@
       </c>
       <c r="L361" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M361" t="inlineStr">
@@ -29694,19 +29684,19 @@
       </c>
       <c r="S361" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="E362" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G362" t="inlineStr">
@@ -29731,7 +29721,7 @@
       </c>
       <c r="L362" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M362" t="inlineStr">
@@ -29756,19 +29746,19 @@
       </c>
       <c r="S362" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="E363" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
@@ -29778,22 +29768,22 @@
       </c>
       <c r="H363" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I363" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="K363" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L363" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M363" t="inlineStr">
@@ -29803,7 +29793,7 @@
       </c>
       <c r="N363" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O363" t="inlineStr">
@@ -29818,24 +29808,19 @@
       </c>
       <c r="S363" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="E364" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
-        </is>
-      </c>
-      <c r="F364" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="G364" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H364" t="inlineStr">
@@ -29848,14 +29833,9 @@
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
-      <c r="K364" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
       <c r="L364" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M364" t="inlineStr">
@@ -29865,7 +29845,7 @@
       </c>
       <c r="N364" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O364" t="inlineStr">
@@ -29880,7 +29860,7 @@
       </c>
       <c r="S364" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
@@ -34360,23 +34340,23 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
       <c r="E144">
+        <v>0</v>
+      </c>
+      <c r="F144">
         <v>1</v>
       </c>
-      <c r="F144">
+      <c r="G144">
         <v>0</v>
-      </c>
-      <c r="G144">
-        <v>1</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="E145">
@@ -34392,7 +34372,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="E146">
@@ -34934,6 +34914,53 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">klm ox</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unnamed box</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A1</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown device</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt0h140-0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -35209,10 +35236,10 @@
         <v>81</v>
       </c>
       <c r="I7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J7">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Take out jkl from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -29056,12 +29056,12 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">A1</t>
         </is>
       </c>
       <c r="E352" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="G352" t="inlineStr">
@@ -29081,7 +29081,7 @@
       </c>
       <c r="L352" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M352" t="inlineStr">
@@ -29106,7 +29106,7 @@
       </c>
       <c r="S352" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
@@ -29128,7 +29128,7 @@
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">A2</t>
         </is>
       </c>
       <c r="E353" t="inlineStr">
@@ -29178,7 +29178,7 @@
       </c>
       <c r="S353" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
@@ -29200,126 +29200,136 @@
       </c>
       <c r="D354" t="inlineStr">
         <is>
+          <t xml:space="preserve">A3</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unnamed box</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
           <t xml:space="preserve">A4</t>
         </is>
       </c>
-      <c r="E354" t="inlineStr">
+      <c r="E355" t="inlineStr">
         <is>
           <t xml:space="preserve">jkl</t>
         </is>
       </c>
-      <c r="G354" t="inlineStr">
+      <c r="G355" t="inlineStr">
         <is>
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H354" t="inlineStr">
+      <c r="H355" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
-      <c r="I354" t="inlineStr">
+      <c r="I355" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
-      <c r="L354" t="inlineStr">
+      <c r="L355" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M354" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="N354" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="O354" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="R354" t="inlineStr">
+      <c r="M355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R355" t="inlineStr">
         <is>
           <t xml:space="preserve">stored</t>
         </is>
       </c>
-      <c r="S354" t="inlineStr">
+      <c r="S355" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mtt3mo6u-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="355">
-      <c r="E355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK gNT</t>
-        </is>
-      </c>
-      <c r="F355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p21</t>
-        </is>
-      </c>
-      <c r="G355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="I355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="K355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="L355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="N355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="O355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gNT</t>
-        </is>
-      </c>
-      <c r="R355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="E356" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F356" t="inlineStr">
@@ -29349,7 +29359,7 @@
       </c>
       <c r="L356" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M356" t="inlineStr">
@@ -29364,7 +29374,7 @@
       </c>
       <c r="O356" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R356" t="inlineStr">
@@ -29374,14 +29384,14 @@
       </c>
       <c r="S356" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="E357" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
@@ -29411,7 +29421,7 @@
       </c>
       <c r="L357" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M357" t="inlineStr">
@@ -29436,19 +29446,19 @@
       </c>
       <c r="S357" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="E358" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
@@ -29473,7 +29483,7 @@
       </c>
       <c r="L358" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M358" t="inlineStr">
@@ -29498,19 +29508,19 @@
       </c>
       <c r="S358" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="E359" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
@@ -29530,12 +29540,12 @@
       </c>
       <c r="K359" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L359" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M359" t="inlineStr">
@@ -29550,7 +29560,7 @@
       </c>
       <c r="O359" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R359" t="inlineStr">
@@ -29560,19 +29570,19 @@
       </c>
       <c r="S359" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="E360" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
@@ -29597,7 +29607,7 @@
       </c>
       <c r="L360" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M360" t="inlineStr">
@@ -29612,7 +29622,7 @@
       </c>
       <c r="O360" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R360" t="inlineStr">
@@ -29622,19 +29632,19 @@
       </c>
       <c r="S360" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="E361" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="F361" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
@@ -29659,7 +29669,7 @@
       </c>
       <c r="L361" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M361" t="inlineStr">
@@ -29684,19 +29694,19 @@
       </c>
       <c r="S361" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="E362" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G362" t="inlineStr">
@@ -29721,7 +29731,7 @@
       </c>
       <c r="L362" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M362" t="inlineStr">
@@ -29746,19 +29756,19 @@
       </c>
       <c r="S362" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="E363" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
@@ -29768,22 +29778,22 @@
       </c>
       <c r="H363" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I363" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="K363" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L363" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M363" t="inlineStr">
@@ -29793,7 +29803,7 @@
       </c>
       <c r="N363" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O363" t="inlineStr">
@@ -29808,19 +29818,24 @@
       </c>
       <c r="S363" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="E364" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">Hek caspex</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G364" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H364" t="inlineStr">
@@ -29833,9 +29848,14 @@
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
+      <c r="K364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
       <c r="L364" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M364" t="inlineStr">
@@ -29845,7 +29865,7 @@
       </c>
       <c r="N364" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O364" t="inlineStr">
@@ -29860,7 +29880,7 @@
       </c>
       <c r="S364" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
@@ -34340,23 +34360,23 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="E144">
+        <v>1</v>
+      </c>
+      <c r="F144">
         <v>0</v>
       </c>
-      <c r="F144">
+      <c r="G144">
         <v>1</v>
-      </c>
-      <c r="G144">
-        <v>0</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
       <c r="E145">
@@ -34372,7 +34392,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="E146">
@@ -34961,6 +34981,53 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unnamed box</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A2</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown device</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -35236,10 +35303,10 @@
         <v>81</v>
       </c>
       <c r="I7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J7">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Save work this device had kept from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -29200,126 +29200,136 @@
       </c>
       <c r="D354" t="inlineStr">
         <is>
+          <t xml:space="preserve">A3</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unnamed box</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
           <t xml:space="preserve">A4</t>
         </is>
       </c>
-      <c r="E354" t="inlineStr">
+      <c r="E355" t="inlineStr">
         <is>
           <t xml:space="preserve">jkl</t>
         </is>
       </c>
-      <c r="G354" t="inlineStr">
+      <c r="G355" t="inlineStr">
         <is>
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H354" t="inlineStr">
+      <c r="H355" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
-      <c r="I354" t="inlineStr">
+      <c r="I355" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
-      <c r="L354" t="inlineStr">
+      <c r="L355" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M354" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="N354" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="O354" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="R354" t="inlineStr">
+      <c r="M355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R355" t="inlineStr">
         <is>
           <t xml:space="preserve">stored</t>
         </is>
       </c>
-      <c r="S354" t="inlineStr">
+      <c r="S355" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mtt3mo6u-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="355">
-      <c r="E355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK gNT</t>
-        </is>
-      </c>
-      <c r="F355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p21</t>
-        </is>
-      </c>
-      <c r="G355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="I355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="K355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="L355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="N355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="O355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gNT</t>
-        </is>
-      </c>
-      <c r="R355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="E356" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F356" t="inlineStr">
@@ -29349,7 +29359,7 @@
       </c>
       <c r="L356" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M356" t="inlineStr">
@@ -29364,7 +29374,7 @@
       </c>
       <c r="O356" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R356" t="inlineStr">
@@ -29374,14 +29384,14 @@
       </c>
       <c r="S356" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="E357" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
@@ -29411,7 +29421,7 @@
       </c>
       <c r="L357" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M357" t="inlineStr">
@@ -29436,19 +29446,19 @@
       </c>
       <c r="S357" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="E358" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
@@ -29473,7 +29483,7 @@
       </c>
       <c r="L358" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M358" t="inlineStr">
@@ -29498,19 +29508,19 @@
       </c>
       <c r="S358" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="E359" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
@@ -29530,12 +29540,12 @@
       </c>
       <c r="K359" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L359" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M359" t="inlineStr">
@@ -29550,7 +29560,7 @@
       </c>
       <c r="O359" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R359" t="inlineStr">
@@ -29560,19 +29570,19 @@
       </c>
       <c r="S359" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="E360" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
@@ -29597,7 +29607,7 @@
       </c>
       <c r="L360" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M360" t="inlineStr">
@@ -29612,7 +29622,7 @@
       </c>
       <c r="O360" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R360" t="inlineStr">
@@ -29622,19 +29632,19 @@
       </c>
       <c r="S360" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="E361" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="F361" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
@@ -29659,7 +29669,7 @@
       </c>
       <c r="L361" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M361" t="inlineStr">
@@ -29684,19 +29694,19 @@
       </c>
       <c r="S361" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="E362" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G362" t="inlineStr">
@@ -29721,7 +29731,7 @@
       </c>
       <c r="L362" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M362" t="inlineStr">
@@ -29746,19 +29756,19 @@
       </c>
       <c r="S362" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="E363" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
@@ -29768,22 +29778,22 @@
       </c>
       <c r="H363" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I363" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="K363" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L363" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M363" t="inlineStr">
@@ -29793,7 +29803,7 @@
       </c>
       <c r="N363" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O363" t="inlineStr">
@@ -29808,19 +29818,24 @@
       </c>
       <c r="S363" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="E364" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Hek caspex</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G364" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H364" t="inlineStr">
@@ -29833,6 +29848,11 @@
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
+      <c r="K364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
       <c r="L364" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -29845,7 +29865,7 @@
       </c>
       <c r="N364" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O364" t="inlineStr">
@@ -29860,7 +29880,7 @@
       </c>
       <c r="S364" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
@@ -30955,26 +30975,11 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 TOX4 KO g2.2</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OX</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">g2.2</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="E34">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F34">
         <v>0</v>
@@ -30986,7 +30991,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR</t>
+          <t xml:space="preserve">Du145 TOX4 KO g2.2</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -30996,12 +31001,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2.2</t>
         </is>
       </c>
       <c r="E35">
@@ -31017,7 +31022,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATF3 KO</t>
+          <t xml:space="preserve">DuDtxR</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -31027,7 +31032,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -31048,7 +31053,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATP7B KO</t>
+          <t xml:space="preserve">DuPar50CR ATF3 KO</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -31079,7 +31084,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR MTF1 KO</t>
+          <t xml:space="preserve">DuPar50CR ATP7B KO</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -31110,7 +31115,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR NT KO</t>
+          <t xml:space="preserve">DuPar50CR MTF1 KO</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -31141,7 +31146,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2</t>
+          <t xml:space="preserve">DuPar50CR NT KO</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -31151,12 +31156,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E40">
@@ -31172,7 +31177,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2</t>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -31187,7 +31192,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2.2</t>
+          <t xml:space="preserve">g1.2</t>
         </is>
       </c>
       <c r="E41">
@@ -31203,22 +31208,22 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CASPEX Single</t>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2.2</t>
         </is>
       </c>
       <c r="E42">
@@ -31234,7 +31239,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
+          <t xml:space="preserve">HEK CASPEX Single</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -31244,12 +31249,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E43">
@@ -31265,7 +31270,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh1</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -31275,12 +31280,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E44">
@@ -31296,7 +31301,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh2</t>
+          <t xml:space="preserve">HEK E2F1 sh1</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -31327,7 +31332,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g1</t>
+          <t xml:space="preserve">HEK E2F1 sh2</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -31337,12 +31342,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E46">
@@ -31358,7 +31363,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g2</t>
+          <t xml:space="preserve">HEK FOXA1 KO g1</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -31373,7 +31378,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E47">
@@ -31389,7 +31394,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 OX</t>
+          <t xml:space="preserve">HEK FOXA1 KO g2</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -31404,7 +31409,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E48">
@@ -31420,7 +31425,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g1</t>
+          <t xml:space="preserve">HEK HOXB6 OX</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -31430,12 +31435,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E49">
@@ -31445,13 +31450,13 @@
         <v>0</v>
       </c>
       <c r="G49">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g1</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -31466,7 +31471,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E50">
@@ -31476,13 +31481,13 @@
         <v>0</v>
       </c>
       <c r="G50">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g2</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -31513,7 +31518,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT(20)</t>
+          <t xml:space="preserve">HEK STAT1 KO g2</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -31523,12 +31528,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E52">
@@ -31538,35 +31543,35 @@
         <v>0</v>
       </c>
       <c r="G52">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK gNT(20)</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E53">
         <v>2</v>
       </c>
       <c r="F53">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G53">
         <v>2</v>
@@ -31575,7 +31580,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -31585,7 +31590,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -31597,16 +31602,16 @@
         <v>2</v>
       </c>
       <c r="F54">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G54">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -31616,33 +31621,33 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E55">
         <v>2</v>
       </c>
       <c r="F55">
+        <v>0</v>
+      </c>
+      <c r="G55">
         <v>1</v>
-      </c>
-      <c r="G55">
-        <v>2</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -31652,14 +31657,14 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E56">
         <v>2</v>
       </c>
       <c r="F56">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G56">
         <v>2</v>
@@ -31668,7 +31673,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V 99.17%</t>
+          <t xml:space="preserve">LCC-V</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -31699,12 +31704,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gP2</t>
+          <t xml:space="preserve">LCC-V 99.17%</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -31714,7 +31719,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t xml:space="preserve">gP2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E58">
@@ -31724,18 +31729,18 @@
         <v>0</v>
       </c>
       <c r="G58">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap (m3) (sortER)</t>
+          <t xml:space="preserve">LUCX gP2</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -31745,7 +31750,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gP2</t>
         </is>
       </c>
       <c r="E59">
@@ -31761,7 +31766,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada CASPEX mCherry 1 (no use)</t>
+          <t xml:space="preserve">LnCap (m3) (sortER)</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -31771,7 +31776,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -31792,7 +31797,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canadaa V1G1</t>
+          <t xml:space="preserve">LnCap Canada CASPEX mCherry 1 (no use)</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -31802,7 +31807,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -31823,7 +31828,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select +P+D #1</t>
+          <t xml:space="preserve">LnCap Canadaa V1G1</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -31833,7 +31838,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -31848,13 +31853,13 @@
         <v>0</v>
       </c>
       <c r="G62">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select +P+D #2</t>
+          <t xml:space="preserve">LnCapCASPEX no select +P+D #1</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -31879,13 +31884,13 @@
         <v>0</v>
       </c>
       <c r="G63">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select E</t>
+          <t xml:space="preserve">LnCapCASPEX no select +P+D #2</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -31910,13 +31915,13 @@
         <v>0</v>
       </c>
       <c r="G64">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select H</t>
+          <t xml:space="preserve">LnCapCASPEX no select E</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -31941,20 +31946,35 @@
         <v>0</v>
       </c>
       <c r="G65">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">LnCapCASPEX no select H</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E66">
         <v>2</v>
       </c>
       <c r="F66">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G66">
         <v>1</v>
@@ -35760,6 +35780,53 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unnamed box</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A4</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown device</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -36035,10 +36102,10 @@
         <v>81</v>
       </c>
       <c r="I7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J7">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Add 1 × kkk from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -22399,42 +22399,32 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t xml:space="preserve">UMUT CELLS -80</t>
+          <t xml:space="preserve">UMUT CELLS -4-</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">H1</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g5.1</t>
-        </is>
-      </c>
-      <c r="F271" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p4</t>
+          <t xml:space="preserve">kkk</t>
         </is>
       </c>
       <c r="G271" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-12-31</t>
+          <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
         <is>
-          <t xml:space="preserve">31-12-25</t>
-        </is>
-      </c>
-      <c r="K271" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
       <c r="L271" t="inlineStr">
@@ -22444,17 +22434,17 @@
       </c>
       <c r="M271" t="inlineStr">
         <is>
-          <t xml:space="preserve">DtxR</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="N271" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t xml:space="preserve">g5.1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R271" t="inlineStr">
@@ -22464,7 +22454,7 @@
       </c>
       <c r="S271" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-83</t>
+          <t xml:space="preserve">v-mttmmw7m-0</t>
         </is>
       </c>
     </row>
@@ -22486,7 +22476,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">A1</t>
         </is>
       </c>
       <c r="E272" t="inlineStr">
@@ -22546,7 +22536,7 @@
       </c>
       <c r="S272" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-84</t>
+          <t xml:space="preserve">v-83</t>
         </is>
       </c>
     </row>
@@ -22568,32 +22558,32 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">A2</t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX DSg1.2</t>
+          <t xml:space="preserve">DuDtxR CASPEX g5.1</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t xml:space="preserve">p?</t>
+          <t xml:space="preserve">p4</t>
         </is>
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-12-23</t>
+          <t xml:space="preserve">2025-12-31</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
         <is>
-          <t xml:space="preserve">23-12-25</t>
+          <t xml:space="preserve">31-12-25</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
@@ -22618,7 +22608,7 @@
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t xml:space="preserve">DSg1.2</t>
+          <t xml:space="preserve">g5.1</t>
         </is>
       </c>
       <c r="R273" t="inlineStr">
@@ -22628,7 +22618,7 @@
       </c>
       <c r="S273" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-85</t>
+          <t xml:space="preserve">v-84</t>
         </is>
       </c>
     </row>
@@ -22650,22 +22640,22 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">A3</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX gNT</t>
+          <t xml:space="preserve">DuDtxR CASPEX DSg1.2</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+6</t>
+          <t xml:space="preserve">p?</t>
         </is>
       </c>
       <c r="G274" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H274" t="inlineStr">
@@ -22700,7 +22690,7 @@
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">DSg1.2</t>
         </is>
       </c>
       <c r="R274" t="inlineStr">
@@ -22710,7 +22700,7 @@
       </c>
       <c r="S274" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-86</t>
+          <t xml:space="preserve">v-85</t>
         </is>
       </c>
     </row>
@@ -22732,7 +22722,7 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t xml:space="preserve">A5</t>
+          <t xml:space="preserve">A4</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
@@ -22792,7 +22782,7 @@
       </c>
       <c r="S275" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-87</t>
+          <t xml:space="preserve">v-86</t>
         </is>
       </c>
     </row>
@@ -22814,17 +22804,17 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t xml:space="preserve">A6</t>
+          <t xml:space="preserve">A5</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1</t>
+          <t xml:space="preserve">DuDtxR CASPEX gNT</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+5</t>
+          <t xml:space="preserve">p+6</t>
         </is>
       </c>
       <c r="G276" t="inlineStr">
@@ -22834,12 +22824,12 @@
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-01-02</t>
+          <t xml:space="preserve">2025-12-23</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
         <is>
-          <t xml:space="preserve">2/1/2026</t>
+          <t xml:space="preserve">23-12-25</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
@@ -22864,7 +22854,7 @@
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.1</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R276" t="inlineStr">
@@ -22874,7 +22864,7 @@
       </c>
       <c r="S276" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-88</t>
+          <t xml:space="preserve">v-87</t>
         </is>
       </c>
     </row>
@@ -22896,17 +22886,17 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t xml:space="preserve">A7</t>
+          <t xml:space="preserve">A6</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g3</t>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+7</t>
+          <t xml:space="preserve">p+5</t>
         </is>
       </c>
       <c r="G277" t="inlineStr">
@@ -22946,7 +22936,7 @@
       </c>
       <c r="O277" t="inlineStr">
         <is>
-          <t xml:space="preserve">g3</t>
+          <t xml:space="preserve">g1.1</t>
         </is>
       </c>
       <c r="R277" t="inlineStr">
@@ -22956,7 +22946,7 @@
       </c>
       <c r="S277" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-89</t>
+          <t xml:space="preserve">v-88</t>
         </is>
       </c>
     </row>
@@ -22978,22 +22968,22 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t xml:space="preserve">A8</t>
+          <t xml:space="preserve">A7</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g5.1</t>
+          <t xml:space="preserve">DuDtxR CASPEX g3</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t xml:space="preserve">p5</t>
+          <t xml:space="preserve">p+7</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H278" t="inlineStr">
@@ -23028,7 +23018,7 @@
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t xml:space="preserve">g5.1</t>
+          <t xml:space="preserve">g3</t>
         </is>
       </c>
       <c r="R278" t="inlineStr">
@@ -23038,7 +23028,7 @@
       </c>
       <c r="S278" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-90</t>
+          <t xml:space="preserve">v-89</t>
         </is>
       </c>
     </row>
@@ -23060,32 +23050,32 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t xml:space="preserve">A9</t>
+          <t xml:space="preserve">A8</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1</t>
+          <t xml:space="preserve">DuDtxR CASPEX g5.1</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+7</t>
+          <t xml:space="preserve">p5</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-01-08</t>
+          <t xml:space="preserve">2026-01-02</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
         <is>
-          <t xml:space="preserve">8/1/2026</t>
+          <t xml:space="preserve">2/1/2026</t>
         </is>
       </c>
       <c r="K279" t="inlineStr">
@@ -23110,7 +23100,7 @@
       </c>
       <c r="O279" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.1</t>
+          <t xml:space="preserve">g5.1</t>
         </is>
       </c>
       <c r="R279" t="inlineStr">
@@ -23120,7 +23110,7 @@
       </c>
       <c r="S279" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-91</t>
+          <t xml:space="preserve">v-90</t>
         </is>
       </c>
     </row>
@@ -23142,57 +23132,57 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t xml:space="preserve">B1</t>
+          <t xml:space="preserve">A9</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 KO g1</t>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p+7</t>
         </is>
       </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-12-29</t>
+          <t xml:space="preserve">2026-01-08</t>
         </is>
       </c>
       <c r="I280" t="inlineStr">
         <is>
-          <t xml:space="preserve">29-12-25</t>
+          <t xml:space="preserve">8/1/2026</t>
         </is>
       </c>
       <c r="K280" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M280" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">DtxR</t>
         </is>
       </c>
       <c r="N280" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g1.1</t>
         </is>
       </c>
       <c r="R280" t="inlineStr">
@@ -23202,7 +23192,7 @@
       </c>
       <c r="S280" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-92</t>
+          <t xml:space="preserve">v-91</t>
         </is>
       </c>
     </row>
@@ -23224,7 +23214,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t xml:space="preserve">B2</t>
+          <t xml:space="preserve">B1</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -23284,7 +23274,7 @@
       </c>
       <c r="S281" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-93</t>
+          <t xml:space="preserve">v-92</t>
         </is>
       </c>
     </row>
@@ -23306,12 +23296,12 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t xml:space="preserve">B3</t>
+          <t xml:space="preserve">B2</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1</t>
+          <t xml:space="preserve">HEK HOXB6 KO g1</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
@@ -23341,7 +23331,7 @@
       </c>
       <c r="L282" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M282" t="inlineStr">
@@ -23366,7 +23356,7 @@
       </c>
       <c r="S282" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-94</t>
+          <t xml:space="preserve">v-93</t>
         </is>
       </c>
     </row>
@@ -23388,7 +23378,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t xml:space="preserve">B4</t>
+          <t xml:space="preserve">B3</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -23448,7 +23438,7 @@
       </c>
       <c r="S283" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-95</t>
+          <t xml:space="preserve">v-94</t>
         </is>
       </c>
     </row>
@@ -23470,17 +23460,17 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t xml:space="preserve">B5</t>
+          <t xml:space="preserve">B4</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK JUN KO g1</t>
+          <t xml:space="preserve">HEK CBX3 KO g1</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t xml:space="preserve">p19</t>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G284" t="inlineStr">
@@ -23490,12 +23480,12 @@
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-12-18</t>
+          <t xml:space="preserve">2025-12-29</t>
         </is>
       </c>
       <c r="I284" t="inlineStr">
         <is>
-          <t xml:space="preserve">18-12-25</t>
+          <t xml:space="preserve">29-12-25</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -23530,7 +23520,7 @@
       </c>
       <c r="S284" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-96</t>
+          <t xml:space="preserve">v-95</t>
         </is>
       </c>
     </row>
@@ -23552,17 +23542,17 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t xml:space="preserve">B6</t>
+          <t xml:space="preserve">B5</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g2</t>
+          <t xml:space="preserve">HEK JUN KO g1</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t xml:space="preserve">p30</t>
+          <t xml:space="preserve">p19</t>
         </is>
       </c>
       <c r="G285" t="inlineStr">
@@ -23572,12 +23562,12 @@
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-01-08</t>
+          <t xml:space="preserve">2025-12-18</t>
         </is>
       </c>
       <c r="I285" t="inlineStr">
         <is>
-          <t xml:space="preserve">8/1/2026</t>
+          <t xml:space="preserve">18-12-25</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
@@ -23602,7 +23592,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="R285" t="inlineStr">
@@ -23612,7 +23602,7 @@
       </c>
       <c r="S285" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-97</t>
+          <t xml:space="preserve">v-96</t>
         </is>
       </c>
     </row>
@@ -23634,17 +23624,17 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t xml:space="preserve">B7</t>
+          <t xml:space="preserve">B6</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g1</t>
+          <t xml:space="preserve">HEK STAT1 KO g2</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t xml:space="preserve">p19</t>
+          <t xml:space="preserve">p30</t>
         </is>
       </c>
       <c r="G286" t="inlineStr">
@@ -23654,12 +23644,12 @@
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-12-18</t>
+          <t xml:space="preserve">2026-01-08</t>
         </is>
       </c>
       <c r="I286" t="inlineStr">
         <is>
-          <t xml:space="preserve">18-12-25</t>
+          <t xml:space="preserve">8/1/2026</t>
         </is>
       </c>
       <c r="K286" t="inlineStr">
@@ -23684,7 +23674,7 @@
       </c>
       <c r="O286" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="R286" t="inlineStr">
@@ -23694,7 +23684,7 @@
       </c>
       <c r="S286" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-98</t>
+          <t xml:space="preserve">v-97</t>
         </is>
       </c>
     </row>
@@ -23716,12 +23706,12 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t xml:space="preserve">B8</t>
+          <t xml:space="preserve">B7</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK SMARCE1 KO g2</t>
+          <t xml:space="preserve">HEK STAT1 KO g1</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
@@ -23766,7 +23756,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="R287" t="inlineStr">
@@ -23776,7 +23766,7 @@
       </c>
       <c r="S287" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-99</t>
+          <t xml:space="preserve">v-98</t>
         </is>
       </c>
     </row>
@@ -23798,12 +23788,12 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t xml:space="preserve">B9</t>
+          <t xml:space="preserve">B8</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK SMARCE1 KO g1</t>
+          <t xml:space="preserve">HEK SMARCE1 KO g2</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
@@ -23848,7 +23838,7 @@
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="R288" t="inlineStr">
@@ -23858,7 +23848,7 @@
       </c>
       <c r="S288" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-100</t>
+          <t xml:space="preserve">v-99</t>
         </is>
       </c>
     </row>
@@ -23880,37 +23870,42 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t xml:space="preserve">C1</t>
+          <t xml:space="preserve">B9</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
         <is>
+          <t xml:space="preserve">HEK SMARCE1 KO g1</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p19</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-18</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18-12-25</t>
+        </is>
+      </c>
+      <c r="K289" t="inlineStr">
+        <is>
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="F289" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p14</t>
-        </is>
-      </c>
-      <c r="G289" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H289" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Unknown</t>
-        </is>
-      </c>
-      <c r="K289" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
       <c r="L289" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M289" t="inlineStr">
@@ -23925,7 +23920,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="R289" t="inlineStr">
@@ -23935,7 +23930,7 @@
       </c>
       <c r="S289" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-101</t>
+          <t xml:space="preserve">v-100</t>
         </is>
       </c>
     </row>
@@ -23957,7 +23952,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t xml:space="preserve">C2</t>
+          <t xml:space="preserve">C1</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -23967,7 +23962,7 @@
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t xml:space="preserve">p19</t>
+          <t xml:space="preserve">p14</t>
         </is>
       </c>
       <c r="G290" t="inlineStr">
@@ -23977,12 +23972,7 @@
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-12-18</t>
-        </is>
-      </c>
-      <c r="I290" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18-12-25</t>
+          <t xml:space="preserve">Unknown</t>
         </is>
       </c>
       <c r="K290" t="inlineStr">
@@ -24017,7 +24007,7 @@
       </c>
       <c r="S290" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-102</t>
+          <t xml:space="preserve">v-101</t>
         </is>
       </c>
     </row>
@@ -24039,12 +24029,12 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t xml:space="preserve">C3</t>
+          <t xml:space="preserve">C2</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK APEX1 g1</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
@@ -24089,7 +24079,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R291" t="inlineStr">
@@ -24099,7 +24089,7 @@
       </c>
       <c r="S291" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-103</t>
+          <t xml:space="preserve">v-102</t>
         </is>
       </c>
     </row>
@@ -24121,17 +24111,17 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t xml:space="preserve">C4</t>
+          <t xml:space="preserve">C3</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g2</t>
+          <t xml:space="preserve">HEK APEX1 g1</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p19</t>
         </is>
       </c>
       <c r="G292" t="inlineStr">
@@ -24141,12 +24131,12 @@
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-01-05</t>
+          <t xml:space="preserve">2025-12-18</t>
         </is>
       </c>
       <c r="I292" t="inlineStr">
         <is>
-          <t xml:space="preserve">5/1/2026</t>
+          <t xml:space="preserve">18-12-25</t>
         </is>
       </c>
       <c r="K292" t="inlineStr">
@@ -24156,7 +24146,7 @@
       </c>
       <c r="L292" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M292" t="inlineStr">
@@ -24171,7 +24161,7 @@
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="R292" t="inlineStr">
@@ -24181,7 +24171,7 @@
       </c>
       <c r="S292" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-104</t>
+          <t xml:space="preserve">v-103</t>
         </is>
       </c>
     </row>
@@ -24203,17 +24193,17 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t xml:space="preserve">C5</t>
+          <t xml:space="preserve">C4</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT(20)</t>
+          <t xml:space="preserve">HEK STAT1 KO g2</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t xml:space="preserve">p13</t>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G293" t="inlineStr">
@@ -24223,12 +24213,12 @@
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-01-14</t>
+          <t xml:space="preserve">2026-01-05</t>
         </is>
       </c>
       <c r="I293" t="inlineStr">
         <is>
-          <t xml:space="preserve">14-01-26</t>
+          <t xml:space="preserve">5/1/2026</t>
         </is>
       </c>
       <c r="K293" t="inlineStr">
@@ -24238,7 +24228,7 @@
       </c>
       <c r="L293" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M293" t="inlineStr">
@@ -24253,7 +24243,7 @@
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="R293" t="inlineStr">
@@ -24263,7 +24253,7 @@
       </c>
       <c r="S293" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-105</t>
+          <t xml:space="preserve">v-104</t>
         </is>
       </c>
     </row>
@@ -24285,12 +24275,12 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t xml:space="preserve">C6</t>
+          <t xml:space="preserve">C5</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g1</t>
+          <t xml:space="preserve">HEK gNT(20)</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
@@ -24320,7 +24310,7 @@
       </c>
       <c r="L294" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M294" t="inlineStr">
@@ -24335,7 +24325,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R294" t="inlineStr">
@@ -24345,7 +24335,7 @@
       </c>
       <c r="S294" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-106</t>
+          <t xml:space="preserve">v-105</t>
         </is>
       </c>
     </row>
@@ -24367,12 +24357,12 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t xml:space="preserve">C7</t>
+          <t xml:space="preserve">C6</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1</t>
+          <t xml:space="preserve">HEK POU3F3 KO g1</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
@@ -24427,7 +24417,7 @@
       </c>
       <c r="S295" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-107</t>
+          <t xml:space="preserve">v-106</t>
         </is>
       </c>
     </row>
@@ -24449,32 +24439,32 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t xml:space="preserve">C8</t>
+          <t xml:space="preserve">C7</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">HEK CBX3 KO g1</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+6</t>
+          <t xml:space="preserve">p13</t>
         </is>
       </c>
       <c r="G296" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-05-04</t>
+          <t xml:space="preserve">2026-01-14</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
         <is>
-          <t xml:space="preserve">4/5/2026</t>
+          <t xml:space="preserve">14-01-26</t>
         </is>
       </c>
       <c r="K296" t="inlineStr">
@@ -24484,7 +24474,7 @@
       </c>
       <c r="L296" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M296" t="inlineStr">
@@ -24499,7 +24489,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="R296" t="inlineStr">
@@ -24509,7 +24499,7 @@
       </c>
       <c r="S296" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-108</t>
+          <t xml:space="preserve">v-107</t>
         </is>
       </c>
     </row>
@@ -24531,22 +24521,22 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t xml:space="preserve">C9</t>
+          <t xml:space="preserve">C8</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g2</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t xml:space="preserve">p37</t>
+          <t xml:space="preserve">p+6</t>
         </is>
       </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H297" t="inlineStr">
@@ -24566,7 +24556,7 @@
       </c>
       <c r="L297" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M297" t="inlineStr">
@@ -24581,7 +24571,7 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R297" t="inlineStr">
@@ -24591,7 +24581,7 @@
       </c>
       <c r="S297" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-109</t>
+          <t xml:space="preserve">v-108</t>
         </is>
       </c>
     </row>
@@ -24613,57 +24603,57 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t xml:space="preserve">D1</t>
+          <t xml:space="preserve">C9</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g3</t>
+          <t xml:space="preserve">HEK POU3F3 KO g2</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+9</t>
+          <t xml:space="preserve">p37</t>
         </is>
       </c>
       <c r="G298" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-01-08</t>
+          <t xml:space="preserve">2026-05-04</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
         <is>
-          <t xml:space="preserve">8/1/2026</t>
+          <t xml:space="preserve">4/5/2026</t>
         </is>
       </c>
       <c r="K298" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L298" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M298" t="inlineStr">
         <is>
-          <t xml:space="preserve">DtxR</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="N298" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t xml:space="preserve">g3</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="R298" t="inlineStr">
@@ -24673,7 +24663,7 @@
       </c>
       <c r="S298" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-110</t>
+          <t xml:space="preserve">v-109</t>
         </is>
       </c>
     </row>
@@ -24695,22 +24685,22 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t xml:space="preserve">D2</t>
+          <t xml:space="preserve">D1</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g5.1</t>
+          <t xml:space="preserve">DuDtxR CASPEX g3</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t xml:space="preserve">p7</t>
+          <t xml:space="preserve">p+9</t>
         </is>
       </c>
       <c r="G299" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H299" t="inlineStr">
@@ -24745,7 +24735,7 @@
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t xml:space="preserve">g5.1</t>
+          <t xml:space="preserve">g3</t>
         </is>
       </c>
       <c r="R299" t="inlineStr">
@@ -24755,7 +24745,7 @@
       </c>
       <c r="S299" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-111</t>
+          <t xml:space="preserve">v-110</t>
         </is>
       </c>
     </row>
@@ -24777,22 +24767,22 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t xml:space="preserve">D3</t>
+          <t xml:space="preserve">D2</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX DSg1.2</t>
+          <t xml:space="preserve">DuDtxR CASPEX g5.1</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t xml:space="preserve">p|+7</t>
+          <t xml:space="preserve">p7</t>
         </is>
       </c>
       <c r="G300" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H300" t="inlineStr">
@@ -24827,7 +24817,7 @@
       </c>
       <c r="O300" t="inlineStr">
         <is>
-          <t xml:space="preserve">DSg1.2</t>
+          <t xml:space="preserve">g5.1</t>
         </is>
       </c>
       <c r="R300" t="inlineStr">
@@ -24837,7 +24827,7 @@
       </c>
       <c r="S300" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-112</t>
+          <t xml:space="preserve">v-111</t>
         </is>
       </c>
     </row>
@@ -24859,39 +24849,39 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t xml:space="preserve">D4</t>
+          <t xml:space="preserve">D3</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
         <is>
+          <t xml:space="preserve">DuDtxR CASPEX DSg1.2</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p|+7</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-08</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/1/2026</t>
+        </is>
+      </c>
+      <c r="K301" t="inlineStr">
+        <is>
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="F301" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p11</t>
-        </is>
-      </c>
-      <c r="G301" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H301" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-01-08</t>
-        </is>
-      </c>
-      <c r="I301" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8/1/2026</t>
-        </is>
-      </c>
-      <c r="K301" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
       <c r="L301" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -24899,17 +24889,17 @@
       </c>
       <c r="M301" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">DtxR</t>
         </is>
       </c>
       <c r="N301" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">DSg1.2</t>
         </is>
       </c>
       <c r="R301" t="inlineStr">
@@ -24919,7 +24909,7 @@
       </c>
       <c r="S301" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-113</t>
+          <t xml:space="preserve">v-112</t>
         </is>
       </c>
     </row>
@@ -24941,7 +24931,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t xml:space="preserve">D5</t>
+          <t xml:space="preserve">D4</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -25001,7 +24991,7 @@
       </c>
       <c r="S302" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-114</t>
+          <t xml:space="preserve">v-113</t>
         </is>
       </c>
     </row>
@@ -25023,32 +25013,32 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t xml:space="preserve">D6</t>
+          <t xml:space="preserve">D5</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX DSg1.2</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+9</t>
+          <t xml:space="preserve">p11</t>
         </is>
       </c>
       <c r="G303" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-01-16</t>
+          <t xml:space="preserve">2026-01-08</t>
         </is>
       </c>
       <c r="I303" t="inlineStr">
         <is>
-          <t xml:space="preserve">16-01-26</t>
+          <t xml:space="preserve">8/1/2026</t>
         </is>
       </c>
       <c r="K303" t="inlineStr">
@@ -25063,17 +25053,17 @@
       </c>
       <c r="M303" t="inlineStr">
         <is>
-          <t xml:space="preserve">DtxR</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="N303" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O303" t="inlineStr">
         <is>
-          <t xml:space="preserve">DSg1.2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R303" t="inlineStr">
@@ -25083,7 +25073,7 @@
       </c>
       <c r="S303" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-115</t>
+          <t xml:space="preserve">v-114</t>
         </is>
       </c>
     </row>
@@ -25105,22 +25095,22 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t xml:space="preserve">D7</t>
+          <t xml:space="preserve">D6</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX gNT</t>
+          <t xml:space="preserve">DuDtxR CASPEX DSg1.2</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t xml:space="preserve">p14</t>
+          <t xml:space="preserve">p+9</t>
         </is>
       </c>
       <c r="G304" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H304" t="inlineStr">
@@ -25155,7 +25145,7 @@
       </c>
       <c r="O304" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">DSg1.2</t>
         </is>
       </c>
       <c r="R304" t="inlineStr">
@@ -25165,7 +25155,7 @@
       </c>
       <c r="S304" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-116</t>
+          <t xml:space="preserve">v-115</t>
         </is>
       </c>
     </row>
@@ -25187,32 +25177,32 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t xml:space="preserve">D8</t>
+          <t xml:space="preserve">D7</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1</t>
+          <t xml:space="preserve">DuDtxR CASPEX gNT</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+12</t>
+          <t xml:space="preserve">p14</t>
         </is>
       </c>
       <c r="G305" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-04-24</t>
+          <t xml:space="preserve">2026-01-16</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
         <is>
-          <t xml:space="preserve">24-04-25</t>
+          <t xml:space="preserve">16-01-26</t>
         </is>
       </c>
       <c r="K305" t="inlineStr">
@@ -25237,7 +25227,7 @@
       </c>
       <c r="O305" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.1</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R305" t="inlineStr">
@@ -25247,7 +25237,7 @@
       </c>
       <c r="S305" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-117</t>
+          <t xml:space="preserve">v-116</t>
         </is>
       </c>
     </row>
@@ -25269,32 +25259,32 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t xml:space="preserve">D9</t>
+          <t xml:space="preserve">D8</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g3</t>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t xml:space="preserve">p10</t>
+          <t xml:space="preserve">p+12</t>
         </is>
       </c>
       <c r="G306" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-05-05</t>
+          <t xml:space="preserve">2025-04-24</t>
         </is>
       </c>
       <c r="I306" t="inlineStr">
         <is>
-          <t xml:space="preserve">5/5/2025</t>
+          <t xml:space="preserve">24-04-25</t>
         </is>
       </c>
       <c r="K306" t="inlineStr">
@@ -25319,7 +25309,7 @@
       </c>
       <c r="O306" t="inlineStr">
         <is>
-          <t xml:space="preserve">g3</t>
+          <t xml:space="preserve">g1.1</t>
         </is>
       </c>
       <c r="R306" t="inlineStr">
@@ -25329,7 +25319,7 @@
       </c>
       <c r="S306" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-118</t>
+          <t xml:space="preserve">v-117</t>
         </is>
       </c>
     </row>
@@ -25351,17 +25341,17 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t xml:space="preserve">E1</t>
+          <t xml:space="preserve">D9</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 HOXB6 OX</t>
+          <t xml:space="preserve">DuDtxR CASPEX g3</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">p10</t>
         </is>
       </c>
       <c r="G307" t="inlineStr">
@@ -25371,37 +25361,37 @@
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-01</t>
+          <t xml:space="preserve">2025-05-05</t>
         </is>
       </c>
       <c r="I307" t="inlineStr">
         <is>
-          <t xml:space="preserve">1/6/2026</t>
+          <t xml:space="preserve">5/5/2025</t>
         </is>
       </c>
       <c r="K307" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="L307" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M307" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">DtxR</t>
         </is>
       </c>
       <c r="N307" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O307" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g3</t>
         </is>
       </c>
       <c r="R307" t="inlineStr">
@@ -25411,7 +25401,7 @@
       </c>
       <c r="S307" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-119</t>
+          <t xml:space="preserve">v-118</t>
         </is>
       </c>
     </row>
@@ -25433,12 +25423,12 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t xml:space="preserve">E2</t>
+          <t xml:space="preserve">E1</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 POU3F3 KO g1</t>
+          <t xml:space="preserve">Huh7 HOXB6 OX</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
@@ -25468,7 +25458,7 @@
       </c>
       <c r="L308" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M308" t="inlineStr">
@@ -25483,7 +25473,7 @@
       </c>
       <c r="O308" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R308" t="inlineStr">
@@ -25493,7 +25483,7 @@
       </c>
       <c r="S308" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-120</t>
+          <t xml:space="preserve">v-119</t>
         </is>
       </c>
     </row>
@@ -25515,12 +25505,12 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t xml:space="preserve">E3</t>
+          <t xml:space="preserve">E2</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 CBX3 OX</t>
+          <t xml:space="preserve">Huh7 POU3F3 KO g1</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
@@ -25550,7 +25540,7 @@
       </c>
       <c r="L309" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M309" t="inlineStr">
@@ -25565,7 +25555,7 @@
       </c>
       <c r="O309" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="R309" t="inlineStr">
@@ -25575,7 +25565,7 @@
       </c>
       <c r="S309" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-121</t>
+          <t xml:space="preserve">v-120</t>
         </is>
       </c>
     </row>
@@ -25597,12 +25587,12 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t xml:space="preserve">E4</t>
+          <t xml:space="preserve">E3</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 POU3F3 KO g2</t>
+          <t xml:space="preserve">Huh7 CBX3 OX</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
@@ -25632,7 +25622,7 @@
       </c>
       <c r="L310" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M310" t="inlineStr">
@@ -25647,7 +25637,7 @@
       </c>
       <c r="O310" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R310" t="inlineStr">
@@ -25657,7 +25647,7 @@
       </c>
       <c r="S310" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-122</t>
+          <t xml:space="preserve">v-121</t>
         </is>
       </c>
     </row>
@@ -25679,32 +25669,32 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t xml:space="preserve">E5</t>
+          <t xml:space="preserve">E4</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 TOX4 KO</t>
+          <t xml:space="preserve">Huh7 POU3F3 KO g2</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+12</t>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G311" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H311" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-04-24</t>
+          <t xml:space="preserve">2026-06-01</t>
         </is>
       </c>
       <c r="I311" t="inlineStr">
         <is>
-          <t xml:space="preserve">24-04-25</t>
+          <t xml:space="preserve">1/6/2026</t>
         </is>
       </c>
       <c r="K311" t="inlineStr">
@@ -25714,7 +25704,7 @@
       </c>
       <c r="L311" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M311" t="inlineStr">
@@ -25729,7 +25719,7 @@
       </c>
       <c r="O311" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="R311" t="inlineStr">
@@ -25739,7 +25729,7 @@
       </c>
       <c r="S311" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-123</t>
+          <t xml:space="preserve">v-122</t>
         </is>
       </c>
     </row>
@@ -25761,22 +25751,22 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t xml:space="preserve">E6</t>
+          <t xml:space="preserve">E5</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
+          <t xml:space="preserve">Huh7 TOX4 KO</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t xml:space="preserve">p82</t>
+          <t xml:space="preserve">p+12</t>
         </is>
       </c>
       <c r="G312" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H312" t="inlineStr">
@@ -25796,7 +25786,7 @@
       </c>
       <c r="L312" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M312" t="inlineStr">
@@ -25821,7 +25811,7 @@
       </c>
       <c r="S312" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-124</t>
+          <t xml:space="preserve">v-123</t>
         </is>
       </c>
     </row>
@@ -25843,32 +25833,32 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t xml:space="preserve">E7</t>
+          <t xml:space="preserve">E6</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 TOX4 KO g1</t>
+          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t xml:space="preserve">p?</t>
+          <t xml:space="preserve">p82</t>
         </is>
       </c>
       <c r="G313" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unknown</t>
+          <t xml:space="preserve">2025-04-24</t>
         </is>
       </c>
       <c r="I313" t="inlineStr">
         <is>
-          <t xml:space="preserve">caNT read</t>
+          <t xml:space="preserve">24-04-25</t>
         </is>
       </c>
       <c r="K313" t="inlineStr">
@@ -25878,7 +25868,7 @@
       </c>
       <c r="L313" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M313" t="inlineStr">
@@ -25893,7 +25883,7 @@
       </c>
       <c r="O313" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R313" t="inlineStr">
@@ -25903,7 +25893,7 @@
       </c>
       <c r="S313" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-125</t>
+          <t xml:space="preserve">v-124</t>
         </is>
       </c>
     </row>
@@ -25925,32 +25915,32 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t xml:space="preserve">E8</t>
+          <t xml:space="preserve">E7</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATP7B KO</t>
+          <t xml:space="preserve">Huh7 TOX4 KO g1</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t xml:space="preserve">p81</t>
+          <t xml:space="preserve">p?</t>
         </is>
       </c>
       <c r="G314" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-04-21</t>
+          <t xml:space="preserve">Unknown</t>
         </is>
       </c>
       <c r="I314" t="inlineStr">
         <is>
-          <t xml:space="preserve">21-04-25</t>
+          <t xml:space="preserve">caNT read</t>
         </is>
       </c>
       <c r="K314" t="inlineStr">
@@ -25960,7 +25950,7 @@
       </c>
       <c r="L314" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M314" t="inlineStr">
@@ -25975,7 +25965,7 @@
       </c>
       <c r="O314" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="R314" t="inlineStr">
@@ -25985,7 +25975,7 @@
       </c>
       <c r="S314" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-126</t>
+          <t xml:space="preserve">v-125</t>
         </is>
       </c>
     </row>
@@ -26007,17 +25997,17 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t xml:space="preserve">E9</t>
+          <t xml:space="preserve">E8</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
+          <t xml:space="preserve">Huh7 ATP7B KO</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t xml:space="preserve">p84</t>
+          <t xml:space="preserve">p81</t>
         </is>
       </c>
       <c r="G315" t="inlineStr">
@@ -26027,12 +26017,12 @@
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-05-02</t>
+          <t xml:space="preserve">2025-04-21</t>
         </is>
       </c>
       <c r="I315" t="inlineStr">
         <is>
-          <t xml:space="preserve">2/5/2025</t>
+          <t xml:space="preserve">21-04-25</t>
         </is>
       </c>
       <c r="K315" t="inlineStr">
@@ -26067,7 +26057,7 @@
       </c>
       <c r="S315" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-127</t>
+          <t xml:space="preserve">v-126</t>
         </is>
       </c>
     </row>
@@ -26089,17 +26079,17 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t xml:space="preserve">F1</t>
+          <t xml:space="preserve">E9</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 KO g1</t>
+          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t xml:space="preserve">p48</t>
+          <t xml:space="preserve">p84</t>
         </is>
       </c>
       <c r="G316" t="inlineStr">
@@ -26109,22 +26099,22 @@
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-05-04</t>
+          <t xml:space="preserve">2025-05-02</t>
         </is>
       </c>
       <c r="I316" t="inlineStr">
         <is>
-          <t xml:space="preserve">4/5/2026</t>
+          <t xml:space="preserve">2/5/2025</t>
         </is>
       </c>
       <c r="K316" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L316" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M316" t="inlineStr">
@@ -26139,7 +26129,7 @@
       </c>
       <c r="O316" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R316" t="inlineStr">
@@ -26149,7 +26139,7 @@
       </c>
       <c r="S316" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-128</t>
+          <t xml:space="preserve">v-127</t>
         </is>
       </c>
     </row>
@@ -26171,7 +26161,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t xml:space="preserve">F2</t>
+          <t xml:space="preserve">F1</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -26231,7 +26221,7 @@
       </c>
       <c r="S317" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-129</t>
+          <t xml:space="preserve">v-128</t>
         </is>
       </c>
     </row>
@@ -26253,17 +26243,17 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t xml:space="preserve">F3</t>
+          <t xml:space="preserve">F2</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">HEK HOXB6 KO g1</t>
         </is>
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t xml:space="preserve">p22</t>
+          <t xml:space="preserve">p48</t>
         </is>
       </c>
       <c r="G318" t="inlineStr">
@@ -26288,7 +26278,7 @@
       </c>
       <c r="L318" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M318" t="inlineStr">
@@ -26303,7 +26293,7 @@
       </c>
       <c r="O318" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="R318" t="inlineStr">
@@ -26313,7 +26303,7 @@
       </c>
       <c r="S318" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-130</t>
+          <t xml:space="preserve">v-129</t>
         </is>
       </c>
     </row>
@@ -26335,7 +26325,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t xml:space="preserve">F4</t>
+          <t xml:space="preserve">F3</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -26395,7 +26385,7 @@
       </c>
       <c r="S319" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-131</t>
+          <t xml:space="preserve">v-130</t>
         </is>
       </c>
     </row>
@@ -26417,17 +26407,17 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t xml:space="preserve">F5</t>
+          <t xml:space="preserve">F4</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g2</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t xml:space="preserve">p37</t>
+          <t xml:space="preserve">p22</t>
         </is>
       </c>
       <c r="G320" t="inlineStr">
@@ -26452,7 +26442,7 @@
       </c>
       <c r="L320" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M320" t="inlineStr">
@@ -26467,7 +26457,7 @@
       </c>
       <c r="O320" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R320" t="inlineStr">
@@ -26477,7 +26467,7 @@
       </c>
       <c r="S320" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-132</t>
+          <t xml:space="preserve">v-131</t>
         </is>
       </c>
     </row>
@@ -26499,22 +26489,22 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t xml:space="preserve">F6</t>
+          <t xml:space="preserve">F5</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO g3</t>
+          <t xml:space="preserve">HEK POU3F3 KO g2</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+7</t>
+          <t xml:space="preserve">p37</t>
         </is>
       </c>
       <c r="G321" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H321" t="inlineStr">
@@ -26549,7 +26539,7 @@
       </c>
       <c r="O321" t="inlineStr">
         <is>
-          <t xml:space="preserve">g3</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="R321" t="inlineStr">
@@ -26559,7 +26549,7 @@
       </c>
       <c r="S321" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-133</t>
+          <t xml:space="preserve">v-132</t>
         </is>
       </c>
     </row>
@@ -26581,17 +26571,17 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t xml:space="preserve">F7</t>
+          <t xml:space="preserve">F6</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK TOX4 KO g2</t>
+          <t xml:space="preserve">HEK ATP7B KO g3</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+6</t>
+          <t xml:space="preserve">p+7</t>
         </is>
       </c>
       <c r="G322" t="inlineStr">
@@ -26601,12 +26591,12 @@
       </c>
       <c r="H322" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-04-24</t>
+          <t xml:space="preserve">2026-05-04</t>
         </is>
       </c>
       <c r="I322" t="inlineStr">
         <is>
-          <t xml:space="preserve">24-04-25</t>
+          <t xml:space="preserve">4/5/2026</t>
         </is>
       </c>
       <c r="K322" t="inlineStr">
@@ -26616,7 +26606,7 @@
       </c>
       <c r="L322" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M322" t="inlineStr">
@@ -26631,7 +26621,7 @@
       </c>
       <c r="O322" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g3</t>
         </is>
       </c>
       <c r="R322" t="inlineStr">
@@ -26641,7 +26631,7 @@
       </c>
       <c r="S322" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-134</t>
+          <t xml:space="preserve">v-133</t>
         </is>
       </c>
     </row>
@@ -26663,7 +26653,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t xml:space="preserve">F8</t>
+          <t xml:space="preserve">F7</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -26673,7 +26663,7 @@
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+7</t>
+          <t xml:space="preserve">p+6</t>
         </is>
       </c>
       <c r="G323" t="inlineStr">
@@ -26683,12 +26673,12 @@
       </c>
       <c r="H323" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-05-02</t>
+          <t xml:space="preserve">2025-04-24</t>
         </is>
       </c>
       <c r="I323" t="inlineStr">
         <is>
-          <t xml:space="preserve">2/5/2025</t>
+          <t xml:space="preserve">24-04-25</t>
         </is>
       </c>
       <c r="K323" t="inlineStr">
@@ -26723,7 +26713,7 @@
       </c>
       <c r="S323" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-135</t>
+          <t xml:space="preserve">v-134</t>
         </is>
       </c>
     </row>
@@ -26745,42 +26735,42 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t xml:space="preserve">F9</t>
+          <t xml:space="preserve">F8</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
         <is>
+          <t xml:space="preserve">HEK TOX4 KO g2</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p+7</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-02</t>
+        </is>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2/5/2025</t>
+        </is>
+      </c>
+      <c r="K324" t="inlineStr">
+        <is>
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="F324" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p19</t>
-        </is>
-      </c>
-      <c r="G324" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H324" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-05-19</t>
-        </is>
-      </c>
-      <c r="I324" t="inlineStr">
-        <is>
-          <t xml:space="preserve">19-05-25</t>
-        </is>
-      </c>
-      <c r="K324" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
       <c r="L324" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M324" t="inlineStr">
@@ -26795,7 +26785,7 @@
       </c>
       <c r="O324" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="R324" t="inlineStr">
@@ -26805,7 +26795,7 @@
       </c>
       <c r="S324" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-136</t>
+          <t xml:space="preserve">v-135</t>
         </is>
       </c>
     </row>
@@ -26827,37 +26817,37 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t xml:space="preserve">G1</t>
+          <t xml:space="preserve">F9</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+20</t>
+          <t xml:space="preserve">p19</t>
         </is>
       </c>
       <c r="G325" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H325" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-05-26</t>
+          <t xml:space="preserve">2025-05-19</t>
         </is>
       </c>
       <c r="I325" t="inlineStr">
         <is>
-          <t xml:space="preserve">26-05-26</t>
+          <t xml:space="preserve">19-05-25</t>
         </is>
       </c>
       <c r="K325" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L325" t="inlineStr">
@@ -26872,22 +26862,12 @@
       </c>
       <c r="N325" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O325" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
-        </is>
-      </c>
-      <c r="P325" t="inlineStr">
-        <is>
-          <t xml:space="preserve">chip-negative</t>
-        </is>
-      </c>
-      <c r="Q325" t="inlineStr">
-        <is>
-          <t xml:space="preserve">chip-</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R325" t="inlineStr">
@@ -26897,7 +26877,7 @@
       </c>
       <c r="S325" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-137</t>
+          <t xml:space="preserve">v-136</t>
         </is>
       </c>
     </row>
@@ -26919,7 +26899,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t xml:space="preserve">G2</t>
+          <t xml:space="preserve">G1</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -26989,7 +26969,7 @@
       </c>
       <c r="S326" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-138</t>
+          <t xml:space="preserve">v-137</t>
         </is>
       </c>
     </row>
@@ -27011,17 +26991,17 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t xml:space="preserve">G3</t>
+          <t xml:space="preserve">G2</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP2</t>
+          <t xml:space="preserve">LNCX gNT</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+21</t>
+          <t xml:space="preserve">p+20</t>
         </is>
       </c>
       <c r="G327" t="inlineStr">
@@ -27031,12 +27011,12 @@
       </c>
       <c r="H327" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-04</t>
+          <t xml:space="preserve">2026-05-26</t>
         </is>
       </c>
       <c r="I327" t="inlineStr">
         <is>
-          <t xml:space="preserve">4/6/2026</t>
+          <t xml:space="preserve">26-05-26</t>
         </is>
       </c>
       <c r="K327" t="inlineStr">
@@ -27061,7 +27041,17 @@
       </c>
       <c r="O327" t="inlineStr">
         <is>
-          <t xml:space="preserve">gP2</t>
+          <t xml:space="preserve">gNT</t>
+        </is>
+      </c>
+      <c r="P327" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chip-negative</t>
+        </is>
+      </c>
+      <c r="Q327" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chip-</t>
         </is>
       </c>
       <c r="R327" t="inlineStr">
@@ -27071,7 +27061,7 @@
       </c>
       <c r="S327" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-139</t>
+          <t xml:space="preserve">v-138</t>
         </is>
       </c>
     </row>
@@ -27093,7 +27083,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t xml:space="preserve">G4</t>
+          <t xml:space="preserve">G3</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -27103,7 +27093,7 @@
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+20</t>
+          <t xml:space="preserve">p+21</t>
         </is>
       </c>
       <c r="G328" t="inlineStr">
@@ -27113,12 +27103,12 @@
       </c>
       <c r="H328" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-05-26</t>
+          <t xml:space="preserve">2026-06-04</t>
         </is>
       </c>
       <c r="I328" t="inlineStr">
         <is>
-          <t xml:space="preserve">26-05-26</t>
+          <t xml:space="preserve">4/6/2026</t>
         </is>
       </c>
       <c r="K328" t="inlineStr">
@@ -27153,7 +27143,7 @@
       </c>
       <c r="S328" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-140</t>
+          <t xml:space="preserve">v-139</t>
         </is>
       </c>
     </row>
@@ -27175,32 +27165,32 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t xml:space="preserve">G5</t>
+          <t xml:space="preserve">G4</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G4</t>
+          <t xml:space="preserve">LNCX gP2</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t xml:space="preserve">p41</t>
+          <t xml:space="preserve">p+20</t>
         </is>
       </c>
       <c r="G329" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H329" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-05-19</t>
+          <t xml:space="preserve">2026-05-26</t>
         </is>
       </c>
       <c r="I329" t="inlineStr">
         <is>
-          <t xml:space="preserve">19-05-25</t>
+          <t xml:space="preserve">26-05-26</t>
         </is>
       </c>
       <c r="K329" t="inlineStr">
@@ -27220,12 +27210,12 @@
       </c>
       <c r="N329" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O329" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gP2</t>
         </is>
       </c>
       <c r="R329" t="inlineStr">
@@ -27235,7 +27225,7 @@
       </c>
       <c r="S329" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-141</t>
+          <t xml:space="preserve">v-140</t>
         </is>
       </c>
     </row>
@@ -27257,12 +27247,12 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t xml:space="preserve">G6</t>
+          <t xml:space="preserve">G5</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G3</t>
+          <t xml:space="preserve">LnCap Canada V1G4</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
@@ -27317,7 +27307,7 @@
       </c>
       <c r="S330" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-142</t>
+          <t xml:space="preserve">v-141</t>
         </is>
       </c>
     </row>
@@ -27339,12 +27329,12 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t xml:space="preserve">G7</t>
+          <t xml:space="preserve">G6</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G2</t>
+          <t xml:space="preserve">LnCap Canada V1G3</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
@@ -27399,7 +27389,7 @@
       </c>
       <c r="S331" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-143</t>
+          <t xml:space="preserve">v-142</t>
         </is>
       </c>
     </row>
@@ -27421,27 +27411,32 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t xml:space="preserve">G8</t>
+          <t xml:space="preserve">G7</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select E</t>
+          <t xml:space="preserve">LnCap Canada V1G2</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t xml:space="preserve">p?</t>
+          <t xml:space="preserve">p41</t>
         </is>
       </c>
       <c r="G332" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H332" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unknown</t>
+          <t xml:space="preserve">2025-05-19</t>
+        </is>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t xml:space="preserve">19-05-25</t>
         </is>
       </c>
       <c r="K332" t="inlineStr">
@@ -27461,7 +27456,7 @@
       </c>
       <c r="N332" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O332" t="inlineStr">
@@ -27476,7 +27471,7 @@
       </c>
       <c r="S332" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-144</t>
+          <t xml:space="preserve">v-143</t>
         </is>
       </c>
     </row>
@@ -27498,12 +27493,12 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t xml:space="preserve">G9</t>
+          <t xml:space="preserve">G8</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select +P+D #1</t>
+          <t xml:space="preserve">LnCapCASPEX no select E</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
@@ -27518,12 +27513,7 @@
       </c>
       <c r="H333" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-04-22</t>
-        </is>
-      </c>
-      <c r="I333" t="inlineStr">
-        <is>
-          <t xml:space="preserve">22-04-25</t>
+          <t xml:space="preserve">Unknown</t>
         </is>
       </c>
       <c r="K333" t="inlineStr">
@@ -27558,7 +27548,7 @@
       </c>
       <c r="S333" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-145</t>
+          <t xml:space="preserve">v-144</t>
         </is>
       </c>
     </row>
@@ -27580,42 +27570,42 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t xml:space="preserve">H1</t>
+          <t xml:space="preserve">G9</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 KO g1</t>
+          <t xml:space="preserve">LnCapCASPEX no select +P+D #1</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t xml:space="preserve">p43</t>
+          <t xml:space="preserve">p?</t>
         </is>
       </c>
       <c r="G334" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H334" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-04-10</t>
+          <t xml:space="preserve">2025-04-22</t>
         </is>
       </c>
       <c r="I334" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/4/2026</t>
+          <t xml:space="preserve">22-04-25</t>
         </is>
       </c>
       <c r="K334" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L334" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M334" t="inlineStr">
@@ -27625,12 +27615,12 @@
       </c>
       <c r="N334" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O334" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R334" t="inlineStr">
@@ -27640,7 +27630,7 @@
       </c>
       <c r="S334" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-146</t>
+          <t xml:space="preserve">v-145</t>
         </is>
       </c>
     </row>
@@ -27662,17 +27652,17 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t xml:space="preserve">H2</t>
+          <t xml:space="preserve">H1</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
+          <t xml:space="preserve">HEK HOXB6 KO g1</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t xml:space="preserve">p42</t>
+          <t xml:space="preserve">p43</t>
         </is>
       </c>
       <c r="G335" t="inlineStr">
@@ -27682,12 +27672,12 @@
       </c>
       <c r="H335" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-03-24</t>
+          <t xml:space="preserve">2026-04-10</t>
         </is>
       </c>
       <c r="I335" t="inlineStr">
         <is>
-          <t xml:space="preserve">24-03-26</t>
+          <t xml:space="preserve">10/4/2026</t>
         </is>
       </c>
       <c r="K335" t="inlineStr">
@@ -27722,7 +27712,7 @@
       </c>
       <c r="S335" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-147</t>
+          <t xml:space="preserve">v-146</t>
         </is>
       </c>
     </row>
@@ -27744,17 +27734,17 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t xml:space="preserve">H3</t>
+          <t xml:space="preserve">H2</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 KO g1</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t xml:space="preserve">p43</t>
+          <t xml:space="preserve">p42</t>
         </is>
       </c>
       <c r="G336" t="inlineStr">
@@ -27764,12 +27754,12 @@
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-04-10</t>
+          <t xml:space="preserve">2026-03-24</t>
         </is>
       </c>
       <c r="I336" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/4/2026</t>
+          <t xml:space="preserve">24-03-26</t>
         </is>
       </c>
       <c r="K336" t="inlineStr">
@@ -27804,7 +27794,7 @@
       </c>
       <c r="S336" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-148</t>
+          <t xml:space="preserve">v-147</t>
         </is>
       </c>
     </row>
@@ -27826,17 +27816,17 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t xml:space="preserve">H4</t>
+          <t xml:space="preserve">H3</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B GFP</t>
+          <t xml:space="preserve">HEK HOXB6 KO g1</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t xml:space="preserve">p42</t>
+          <t xml:space="preserve">p43</t>
         </is>
       </c>
       <c r="G337" t="inlineStr">
@@ -27861,7 +27851,7 @@
       </c>
       <c r="L337" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M337" t="inlineStr">
@@ -27876,7 +27866,7 @@
       </c>
       <c r="O337" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="R337" t="inlineStr">
@@ -27886,7 +27876,7 @@
       </c>
       <c r="S337" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-149</t>
+          <t xml:space="preserve">v-148</t>
         </is>
       </c>
     </row>
@@ -27908,7 +27898,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t xml:space="preserve">H5</t>
+          <t xml:space="preserve">H4</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -27968,7 +27958,7 @@
       </c>
       <c r="S338" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-150</t>
+          <t xml:space="preserve">v-149</t>
         </is>
       </c>
     </row>
@@ -27990,32 +27980,32 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t xml:space="preserve">H6</t>
+          <t xml:space="preserve">H5</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CASPEX gNT</t>
+          <t xml:space="preserve">HEK ATP7B GFP</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t xml:space="preserve">p?</t>
+          <t xml:space="preserve">p42</t>
         </is>
       </c>
       <c r="G339" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H339" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-02-10</t>
+          <t xml:space="preserve">2026-04-10</t>
         </is>
       </c>
       <c r="I339" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/2/2026</t>
+          <t xml:space="preserve">10/4/2026</t>
         </is>
       </c>
       <c r="K339" t="inlineStr">
@@ -28035,12 +28025,12 @@
       </c>
       <c r="N339" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O339" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R339" t="inlineStr">
@@ -28050,7 +28040,7 @@
       </c>
       <c r="S339" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-151</t>
+          <t xml:space="preserve">v-150</t>
         </is>
       </c>
     </row>
@@ -28072,32 +28062,32 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t xml:space="preserve">H7</t>
+          <t xml:space="preserve">H6</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
+          <t xml:space="preserve">HEK CASPEX gNT</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t xml:space="preserve">p42</t>
+          <t xml:space="preserve">p?</t>
         </is>
       </c>
       <c r="G340" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H340" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-03-24</t>
+          <t xml:space="preserve">2026-02-10</t>
         </is>
       </c>
       <c r="I340" t="inlineStr">
         <is>
-          <t xml:space="preserve">24-03-26</t>
+          <t xml:space="preserve">10/2/2026</t>
         </is>
       </c>
       <c r="K340" t="inlineStr">
@@ -28107,7 +28097,7 @@
       </c>
       <c r="L340" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M340" t="inlineStr">
@@ -28117,12 +28107,12 @@
       </c>
       <c r="N340" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O340" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R340" t="inlineStr">
@@ -28132,7 +28122,7 @@
       </c>
       <c r="S340" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-152</t>
+          <t xml:space="preserve">v-151</t>
         </is>
       </c>
     </row>
@@ -28154,17 +28144,17 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t xml:space="preserve">H8</t>
+          <t xml:space="preserve">H7</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK APEX1 OX</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
         </is>
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p42</t>
         </is>
       </c>
       <c r="G341" t="inlineStr">
@@ -28174,12 +28164,12 @@
       </c>
       <c r="H341" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-02-06</t>
+          <t xml:space="preserve">2026-03-24</t>
         </is>
       </c>
       <c r="I341" t="inlineStr">
         <is>
-          <t xml:space="preserve">6/2/2026</t>
+          <t xml:space="preserve">24-03-26</t>
         </is>
       </c>
       <c r="K341" t="inlineStr">
@@ -28204,7 +28194,7 @@
       </c>
       <c r="O341" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="R341" t="inlineStr">
@@ -28214,7 +28204,7 @@
       </c>
       <c r="S341" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-153</t>
+          <t xml:space="preserve">v-152</t>
         </is>
       </c>
     </row>
@@ -28236,17 +28226,17 @@
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t xml:space="preserve">H9</t>
+          <t xml:space="preserve">H8</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 OX</t>
+          <t xml:space="preserve">HEK APEX1 OX</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G342" t="inlineStr">
@@ -28256,12 +28246,12 @@
       </c>
       <c r="H342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-03-24</t>
+          <t xml:space="preserve">2026-02-06</t>
         </is>
       </c>
       <c r="I342" t="inlineStr">
         <is>
-          <t xml:space="preserve">24-03-26</t>
+          <t xml:space="preserve">6/2/2026</t>
         </is>
       </c>
       <c r="K342" t="inlineStr">
@@ -28296,7 +28286,7 @@
       </c>
       <c r="S342" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-154</t>
+          <t xml:space="preserve">v-153</t>
         </is>
       </c>
     </row>
@@ -28318,57 +28308,57 @@
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t xml:space="preserve">I1</t>
+          <t xml:space="preserve">H9</t>
         </is>
       </c>
       <c r="E343" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1</t>
+          <t xml:space="preserve">HEK CBX3 OX</t>
         </is>
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+3</t>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G343" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H343" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-05-16</t>
+          <t xml:space="preserve">2026-03-24</t>
         </is>
       </c>
       <c r="I343" t="inlineStr">
         <is>
-          <t xml:space="preserve">16-05-25</t>
+          <t xml:space="preserve">24-03-26</t>
         </is>
       </c>
       <c r="K343" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L343" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M343" t="inlineStr">
         <is>
-          <t xml:space="preserve">DtxR</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="N343" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O343" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R343" t="inlineStr">
@@ -28378,7 +28368,7 @@
       </c>
       <c r="S343" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-155</t>
+          <t xml:space="preserve">v-154</t>
         </is>
       </c>
     </row>
@@ -28400,7 +28390,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t xml:space="preserve">I2</t>
+          <t xml:space="preserve">I1</t>
         </is>
       </c>
       <c r="E344" t="inlineStr">
@@ -28410,7 +28400,7 @@
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+4</t>
+          <t xml:space="preserve">p+3</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
@@ -28420,12 +28410,12 @@
       </c>
       <c r="H344" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-05-14</t>
+          <t xml:space="preserve">2025-05-16</t>
         </is>
       </c>
       <c r="I344" t="inlineStr">
         <is>
-          <t xml:space="preserve">14-05-25</t>
+          <t xml:space="preserve">16-05-25</t>
         </is>
       </c>
       <c r="K344" t="inlineStr">
@@ -28460,7 +28450,7 @@
       </c>
       <c r="S344" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-156</t>
+          <t xml:space="preserve">v-155</t>
         </is>
       </c>
     </row>
@@ -28482,7 +28472,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t xml:space="preserve">I3</t>
+          <t xml:space="preserve">I2</t>
         </is>
       </c>
       <c r="E345" t="inlineStr">
@@ -28542,7 +28532,7 @@
       </c>
       <c r="S345" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-157</t>
+          <t xml:space="preserve">v-156</t>
         </is>
       </c>
     </row>
@@ -28564,7 +28554,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t xml:space="preserve">I4</t>
+          <t xml:space="preserve">I3</t>
         </is>
       </c>
       <c r="E346" t="inlineStr">
@@ -28624,7 +28614,7 @@
       </c>
       <c r="S346" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-158</t>
+          <t xml:space="preserve">v-157</t>
         </is>
       </c>
     </row>
@@ -28646,7 +28636,7 @@
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t xml:space="preserve">I5</t>
+          <t xml:space="preserve">I4</t>
         </is>
       </c>
       <c r="E347" t="inlineStr">
@@ -28706,7 +28696,7 @@
       </c>
       <c r="S347" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-159</t>
+          <t xml:space="preserve">v-158</t>
         </is>
       </c>
     </row>
@@ -28728,7 +28718,7 @@
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t xml:space="preserve">I6</t>
+          <t xml:space="preserve">I5</t>
         </is>
       </c>
       <c r="E348" t="inlineStr">
@@ -28788,7 +28778,7 @@
       </c>
       <c r="S348" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-160</t>
+          <t xml:space="preserve">v-159</t>
         </is>
       </c>
     </row>
@@ -28810,39 +28800,39 @@
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t xml:space="preserve">I7</t>
+          <t xml:space="preserve">I6</t>
         </is>
       </c>
       <c r="E349" t="inlineStr">
         <is>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p+4</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-14</t>
+        </is>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14-05-25</t>
+        </is>
+      </c>
+      <c r="K349" t="inlineStr">
+        <is>
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="F349" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p?</t>
-        </is>
-      </c>
-      <c r="G349" t="inlineStr">
-        <is>
-          <t xml:space="preserve">unknown</t>
-        </is>
-      </c>
-      <c r="H349" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-04-24</t>
-        </is>
-      </c>
-      <c r="I349" t="inlineStr">
-        <is>
-          <t xml:space="preserve">24-04-25</t>
-        </is>
-      </c>
-      <c r="K349" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
       <c r="L349" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -28850,17 +28840,17 @@
       </c>
       <c r="M349" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">DtxR</t>
         </is>
       </c>
       <c r="N349" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O349" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1.1</t>
         </is>
       </c>
       <c r="R349" t="inlineStr">
@@ -28870,7 +28860,7 @@
       </c>
       <c r="S349" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-161</t>
+          <t xml:space="preserve">v-160</t>
         </is>
       </c>
     </row>
@@ -28892,22 +28882,22 @@
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t xml:space="preserve">I8</t>
+          <t xml:space="preserve">I7</t>
         </is>
       </c>
       <c r="E350" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR+1</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="F350" t="inlineStr">
         <is>
-          <t xml:space="preserve">P218</t>
+          <t xml:space="preserve">p?</t>
         </is>
       </c>
       <c r="G350" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H350" t="inlineStr">
@@ -28932,7 +28922,7 @@
       </c>
       <c r="M350" t="inlineStr">
         <is>
-          <t xml:space="preserve">CisR</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="N350" t="inlineStr">
@@ -28952,7 +28942,7 @@
       </c>
       <c r="S350" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-162</t>
+          <t xml:space="preserve">v-161</t>
         </is>
       </c>
     </row>
@@ -28974,136 +28964,156 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
+          <t xml:space="preserve">I8</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuPar50CR+1</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P218</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-04-24</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24-04-25</t>
+        </is>
+      </c>
+      <c r="K351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Du145</t>
+        </is>
+      </c>
+      <c r="L351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CisR</t>
+        </is>
+      </c>
+      <c r="N351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-162</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UMUT CELLS -80</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
           <t xml:space="preserve">I9</t>
         </is>
       </c>
-      <c r="E351" t="inlineStr">
+      <c r="E352" t="inlineStr">
         <is>
           <t xml:space="preserve">DuDtxR CASPEX g3</t>
         </is>
       </c>
-      <c r="F351" t="inlineStr">
+      <c r="F352" t="inlineStr">
         <is>
           <t xml:space="preserve">p8</t>
         </is>
       </c>
-      <c r="G351" t="inlineStr">
+      <c r="G352" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H351" t="inlineStr">
+      <c r="H352" t="inlineStr">
         <is>
           <t xml:space="preserve">2025-04-24</t>
         </is>
       </c>
-      <c r="I351" t="inlineStr">
+      <c r="I352" t="inlineStr">
         <is>
           <t xml:space="preserve">24-04-25</t>
         </is>
       </c>
-      <c r="K351" t="inlineStr">
+      <c r="K352" t="inlineStr">
         <is>
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L351" t="inlineStr">
+      <c r="L352" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M351" t="inlineStr">
+      <c r="M352" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
         </is>
       </c>
-      <c r="N351" t="inlineStr">
+      <c r="N352" t="inlineStr">
         <is>
           <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
-      <c r="O351" t="inlineStr">
+      <c r="O352" t="inlineStr">
         <is>
           <t xml:space="preserve">g3</t>
         </is>
       </c>
-      <c r="R351" t="inlineStr">
+      <c r="R352" t="inlineStr">
         <is>
           <t xml:space="preserve">stored</t>
         </is>
       </c>
-      <c r="S351" t="inlineStr">
+      <c r="S352" t="inlineStr">
         <is>
           <t xml:space="preserve">v-163</t>
-        </is>
-      </c>
-    </row>
-    <row r="352">
-      <c r="E352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK gNT</t>
-        </is>
-      </c>
-      <c r="F352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p21</t>
-        </is>
-      </c>
-      <c r="G352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="I352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="K352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="L352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="N352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="O352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gNT</t>
-        </is>
-      </c>
-      <c r="R352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="E353" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F353" t="inlineStr">
@@ -29133,7 +29143,7 @@
       </c>
       <c r="L353" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M353" t="inlineStr">
@@ -29148,7 +29158,7 @@
       </c>
       <c r="O353" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R353" t="inlineStr">
@@ -29158,14 +29168,14 @@
       </c>
       <c r="S353" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="E354" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F354" t="inlineStr">
@@ -29195,7 +29205,7 @@
       </c>
       <c r="L354" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M354" t="inlineStr">
@@ -29220,19 +29230,19 @@
       </c>
       <c r="S354" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="E355" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F355" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G355" t="inlineStr">
@@ -29257,7 +29267,7 @@
       </c>
       <c r="L355" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M355" t="inlineStr">
@@ -29282,19 +29292,19 @@
       </c>
       <c r="S355" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="E356" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
@@ -29314,12 +29324,12 @@
       </c>
       <c r="K356" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L356" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M356" t="inlineStr">
@@ -29334,7 +29344,7 @@
       </c>
       <c r="O356" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R356" t="inlineStr">
@@ -29344,19 +29354,19 @@
       </c>
       <c r="S356" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="E357" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
@@ -29381,7 +29391,7 @@
       </c>
       <c r="L357" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M357" t="inlineStr">
@@ -29396,7 +29406,7 @@
       </c>
       <c r="O357" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R357" t="inlineStr">
@@ -29406,19 +29416,19 @@
       </c>
       <c r="S357" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="E358" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
@@ -29443,7 +29453,7 @@
       </c>
       <c r="L358" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M358" t="inlineStr">
@@ -29468,19 +29478,19 @@
       </c>
       <c r="S358" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="E359" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
@@ -29505,7 +29515,7 @@
       </c>
       <c r="L359" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M359" t="inlineStr">
@@ -29530,19 +29540,19 @@
       </c>
       <c r="S359" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="E360" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
@@ -29552,22 +29562,22 @@
       </c>
       <c r="H360" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I360" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="K360" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L360" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M360" t="inlineStr">
@@ -29577,7 +29587,7 @@
       </c>
       <c r="N360" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O360" t="inlineStr">
@@ -29592,19 +29602,24 @@
       </c>
       <c r="S360" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="E361" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">Hek caspex</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H361" t="inlineStr">
@@ -29617,9 +29632,14 @@
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
+      <c r="K361" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
       <c r="L361" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M361" t="inlineStr">
@@ -29629,7 +29649,7 @@
       </c>
       <c r="N361" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O361" t="inlineStr">
@@ -29644,14 +29664,14 @@
       </c>
       <c r="S361" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="E362" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="G362" t="inlineStr">
@@ -29671,7 +29691,7 @@
       </c>
       <c r="L362" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M362" t="inlineStr">
@@ -29696,7 +29716,7 @@
       </c>
       <c r="S362" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
@@ -29748,7 +29768,7 @@
       </c>
       <c r="S363" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
@@ -29800,57 +29820,109 @@
       </c>
       <c r="S364" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="E365" t="inlineStr">
         <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L365" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M365" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N365" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O365" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R365" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S365" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="E366" t="inlineStr">
+        <is>
           <t xml:space="preserve">khk</t>
         </is>
       </c>
-      <c r="G365" t="inlineStr">
+      <c r="G366" t="inlineStr">
         <is>
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H365" t="inlineStr">
+      <c r="H366" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
-      <c r="I365" t="inlineStr">
+      <c r="I366" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
-      <c r="L365" t="inlineStr">
+      <c r="L366" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M365" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="N365" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="O365" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="R365" t="inlineStr">
+      <c r="M366" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N366" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O366" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R366" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
-      <c r="S365" t="inlineStr">
+      <c r="S366" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mtt5ckqo-0</t>
         </is>
@@ -34264,30 +34336,30 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">kkk</t>
         </is>
       </c>
       <c r="E143">
+        <v>1</v>
+      </c>
+      <c r="F143">
         <v>0</v>
       </c>
-      <c r="F143">
+      <c r="G143">
         <v>1</v>
-      </c>
-      <c r="G143">
-        <v>0</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
       <c r="E144">
         <v>0</v>
       </c>
       <c r="F144">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G144">
         <v>0</v>
@@ -34296,14 +34368,14 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="E145">
         <v>0</v>
       </c>
       <c r="F145">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G145">
         <v>0</v>
@@ -34312,7 +34384,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="E146">
@@ -34322,6 +34394,22 @@
         <v>1</v>
       </c>
       <c r="G146">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">klm ox</t>
+        </is>
+      </c>
+      <c r="E147">
+        <v>0</v>
+      </c>
+      <c r="F147">
+        <v>1</v>
+      </c>
+      <c r="G147">
         <v>0</v>
       </c>
     </row>
@@ -36173,10 +36261,10 @@
         <v>81</v>
       </c>
       <c r="I6">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J6">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Add 1 × deneme from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -29111,34 +29111,44 @@
       </c>
     </row>
     <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unnamed box</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B3</t>
+        </is>
+      </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
-        </is>
-      </c>
-      <c r="F353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">deneme</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H353" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
       <c r="I353" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="K353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
       <c r="L353" t="inlineStr">
@@ -29158,24 +29168,24 @@
       </c>
       <c r="O353" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R353" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">stored</t>
         </is>
       </c>
       <c r="S353" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
+          <t xml:space="preserve">v-mtu5lgdc-0</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="E354" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F354" t="inlineStr">
@@ -29205,7 +29215,7 @@
       </c>
       <c r="L354" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M354" t="inlineStr">
@@ -29220,7 +29230,7 @@
       </c>
       <c r="O354" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R354" t="inlineStr">
@@ -29230,14 +29240,14 @@
       </c>
       <c r="S354" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="E355" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F355" t="inlineStr">
@@ -29267,7 +29277,7 @@
       </c>
       <c r="L355" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M355" t="inlineStr">
@@ -29292,19 +29302,19 @@
       </c>
       <c r="S355" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="E356" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
@@ -29329,7 +29339,7 @@
       </c>
       <c r="L356" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M356" t="inlineStr">
@@ -29354,19 +29364,19 @@
       </c>
       <c r="S356" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="E357" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
@@ -29386,12 +29396,12 @@
       </c>
       <c r="K357" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L357" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M357" t="inlineStr">
@@ -29406,7 +29416,7 @@
       </c>
       <c r="O357" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R357" t="inlineStr">
@@ -29416,19 +29426,19 @@
       </c>
       <c r="S357" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="E358" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
@@ -29453,7 +29463,7 @@
       </c>
       <c r="L358" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M358" t="inlineStr">
@@ -29468,7 +29478,7 @@
       </c>
       <c r="O358" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R358" t="inlineStr">
@@ -29478,19 +29488,19 @@
       </c>
       <c r="S358" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="E359" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
@@ -29515,7 +29525,7 @@
       </c>
       <c r="L359" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M359" t="inlineStr">
@@ -29540,19 +29550,19 @@
       </c>
       <c r="S359" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="E360" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
@@ -29577,7 +29587,7 @@
       </c>
       <c r="L360" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M360" t="inlineStr">
@@ -29602,19 +29612,19 @@
       </c>
       <c r="S360" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="E361" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F361" t="inlineStr">
         <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
@@ -29624,22 +29634,22 @@
       </c>
       <c r="H361" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I361" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="K361" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L361" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M361" t="inlineStr">
@@ -29649,7 +29659,7 @@
       </c>
       <c r="N361" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O361" t="inlineStr">
@@ -29664,19 +29674,24 @@
       </c>
       <c r="S361" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="E362" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">Hek caspex</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G362" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H362" t="inlineStr">
@@ -29689,9 +29704,14 @@
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
+      <c r="K362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
       <c r="L362" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M362" t="inlineStr">
@@ -29701,7 +29721,7 @@
       </c>
       <c r="N362" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O362" t="inlineStr">
@@ -29716,14 +29736,14 @@
       </c>
       <c r="S362" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="E363" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
@@ -29743,7 +29763,7 @@
       </c>
       <c r="L363" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M363" t="inlineStr">
@@ -29768,7 +29788,7 @@
       </c>
       <c r="S363" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
@@ -29820,7 +29840,7 @@
       </c>
       <c r="S364" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
@@ -29872,14 +29892,14 @@
       </c>
       <c r="S365" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="E366" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G366" t="inlineStr">
@@ -29924,14 +29944,14 @@
       </c>
       <c r="S366" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt5ckqo-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="E367" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="G367" t="inlineStr">
@@ -29941,12 +29961,12 @@
       </c>
       <c r="H367" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I367" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L367" t="inlineStr">
@@ -29976,7 +29996,7 @@
       </c>
       <c r="S367" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmypa-0</t>
+          <t xml:space="preserve">v-mtt5ckqo-0</t>
         </is>
       </c>
     </row>
@@ -30027,6 +30047,58 @@
         </is>
       </c>
       <c r="S368" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmmypa-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="E369" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L369" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M369" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N369" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O369" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R369" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S369" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mttmn045-0</t>
         </is>
@@ -34440,24 +34512,14 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">deneme</t>
         </is>
       </c>
       <c r="E143">
         <v>1</v>
       </c>
       <c r="F143">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G143">
         <v>1</v>
@@ -34466,30 +34528,40 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E144">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F144">
+        <v>2</v>
+      </c>
+      <c r="G144">
         <v>1</v>
-      </c>
-      <c r="G144">
-        <v>0</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
       <c r="E145">
         <v>0</v>
       </c>
       <c r="F145">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G145">
         <v>0</v>
@@ -34498,14 +34570,14 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="E146">
         <v>0</v>
       </c>
       <c r="F146">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G146">
         <v>0</v>
@@ -34514,7 +34586,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="E147">
@@ -34524,6 +34596,22 @@
         <v>1</v>
       </c>
       <c r="G147">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">klm ox</t>
+        </is>
+      </c>
+      <c r="E148">
+        <v>0</v>
+      </c>
+      <c r="F148">
+        <v>1</v>
+      </c>
+      <c r="G148">
         <v>0</v>
       </c>
     </row>
@@ -36506,10 +36594,10 @@
         <v>81</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Take out deneme from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -29111,44 +29111,34 @@
       </c>
     </row>
     <row r="353">
-      <c r="A353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Freezer 1</t>
-        </is>
-      </c>
-      <c r="B353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rack 1</t>
-        </is>
-      </c>
-      <c r="C353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Unnamed box</t>
-        </is>
-      </c>
-      <c r="D353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">B3</t>
-        </is>
-      </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">HEK gNT</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H353" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I353" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L353" t="inlineStr">
@@ -29168,24 +29158,24 @@
       </c>
       <c r="O353" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R353" t="inlineStr">
         <is>
-          <t xml:space="preserve">stored</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="S353" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtu5lgdc-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="E354" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F354" t="inlineStr">
@@ -29215,7 +29205,7 @@
       </c>
       <c r="L354" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M354" t="inlineStr">
@@ -29230,7 +29220,7 @@
       </c>
       <c r="O354" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R354" t="inlineStr">
@@ -29240,14 +29230,14 @@
       </c>
       <c r="S354" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="E355" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F355" t="inlineStr">
@@ -29277,7 +29267,7 @@
       </c>
       <c r="L355" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M355" t="inlineStr">
@@ -29302,19 +29292,19 @@
       </c>
       <c r="S355" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="E356" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
@@ -29339,7 +29329,7 @@
       </c>
       <c r="L356" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M356" t="inlineStr">
@@ -29364,19 +29354,19 @@
       </c>
       <c r="S356" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="E357" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
@@ -29396,12 +29386,12 @@
       </c>
       <c r="K357" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L357" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M357" t="inlineStr">
@@ -29416,7 +29406,7 @@
       </c>
       <c r="O357" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R357" t="inlineStr">
@@ -29426,19 +29416,19 @@
       </c>
       <c r="S357" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="E358" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
@@ -29463,7 +29453,7 @@
       </c>
       <c r="L358" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M358" t="inlineStr">
@@ -29478,7 +29468,7 @@
       </c>
       <c r="O358" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="R358" t="inlineStr">
@@ -29488,19 +29478,19 @@
       </c>
       <c r="S358" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="E359" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
@@ -29525,7 +29515,7 @@
       </c>
       <c r="L359" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M359" t="inlineStr">
@@ -29550,19 +29540,19 @@
       </c>
       <c r="S359" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="E360" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
@@ -29587,7 +29577,7 @@
       </c>
       <c r="L360" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M360" t="inlineStr">
@@ -29612,19 +29602,19 @@
       </c>
       <c r="S360" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="E361" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
       <c r="F361" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
@@ -29634,22 +29624,22 @@
       </c>
       <c r="H361" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I361" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="K361" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L361" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M361" t="inlineStr">
@@ -29659,7 +29649,7 @@
       </c>
       <c r="N361" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O361" t="inlineStr">
@@ -29674,24 +29664,19 @@
       </c>
       <c r="S361" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="E362" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
-        </is>
-      </c>
-      <c r="F362" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="G362" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H362" t="inlineStr">
@@ -29704,14 +29689,9 @@
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
-      <c r="K362" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
       <c r="L362" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M362" t="inlineStr">
@@ -29721,7 +29701,7 @@
       </c>
       <c r="N362" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O362" t="inlineStr">
@@ -29736,14 +29716,14 @@
       </c>
       <c r="S362" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="E363" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
@@ -29763,7 +29743,7 @@
       </c>
       <c r="L363" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M363" t="inlineStr">
@@ -29788,7 +29768,7 @@
       </c>
       <c r="S363" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
@@ -29840,7 +29820,7 @@
       </c>
       <c r="S364" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
@@ -29892,14 +29872,14 @@
       </c>
       <c r="S365" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="E366" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="G366" t="inlineStr">
@@ -29944,14 +29924,14 @@
       </c>
       <c r="S366" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtt5ckqo-0</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="E367" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">kkk</t>
         </is>
       </c>
       <c r="G367" t="inlineStr">
@@ -29961,12 +29941,12 @@
       </c>
       <c r="H367" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
       <c r="I367" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
       <c r="L367" t="inlineStr">
@@ -29996,7 +29976,7 @@
       </c>
       <c r="S367" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt5ckqo-0</t>
+          <t xml:space="preserve">v-mttmmypa-0</t>
         </is>
       </c>
     </row>
@@ -30048,14 +30028,14 @@
       </c>
       <c r="S368" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmypa-0</t>
+          <t xml:space="preserve">v-mttmn045-0</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="E369" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">deneme</t>
         </is>
       </c>
       <c r="G369" t="inlineStr">
@@ -30100,7 +30080,7 @@
       </c>
       <c r="S369" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmn045-0</t>
+          <t xml:space="preserve">v-mtu5lgdc-0</t>
         </is>
       </c>
     </row>
@@ -34512,14 +34492,24 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E143">
         <v>1</v>
       </c>
       <c r="F143">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G143">
         <v>1</v>
@@ -34528,33 +34518,23 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
       <c r="E144">
+        <v>0</v>
+      </c>
+      <c r="F144">
         <v>1</v>
       </c>
-      <c r="F144">
-        <v>2</v>
-      </c>
       <c r="G144">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">deneme</t>
         </is>
       </c>
       <c r="E145">
@@ -34959,12 +34939,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">deneme</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -34979,12 +34959,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">DUZENLE</t>
+          <t xml:space="preserve">Unnamed box</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">I8</t>
+          <t xml:space="preserve">B3</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -34999,7 +34979,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtu5lgdc-0</t>
         </is>
       </c>
     </row>
@@ -35011,7 +34991,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -35026,12 +35006,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">UMUT CELLS -4-</t>
+          <t xml:space="preserve">DUZENLE</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">I8</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -35046,7 +35026,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
@@ -35058,7 +35038,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -35078,7 +35058,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">A6</t>
+          <t xml:space="preserve">A4</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -35093,7 +35073,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
@@ -35105,7 +35085,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -35125,7 +35105,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">A8</t>
+          <t xml:space="preserve">A6</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -35140,7 +35120,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
@@ -35152,7 +35132,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -35167,12 +35147,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">DUZENLE</t>
+          <t xml:space="preserve">UMUT CELLS -4-</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">E6</t>
+          <t xml:space="preserve">A8</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -35187,7 +35167,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
@@ -35199,7 +35179,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -35219,7 +35199,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">E8</t>
+          <t xml:space="preserve">E6</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -35234,7 +35214,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
@@ -35246,7 +35226,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -35261,12 +35241,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">UMUT CELLS -4-</t>
+          <t xml:space="preserve">DUZENLE</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">B8</t>
+          <t xml:space="preserve">E8</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -35281,7 +35261,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
@@ -35293,7 +35273,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -35313,7 +35293,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">D5</t>
+          <t xml:space="preserve">B8</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -35328,7 +35308,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
@@ -35340,7 +35320,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -35360,7 +35340,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">D3</t>
+          <t xml:space="preserve">D5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -35375,7 +35355,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
@@ -35387,7 +35367,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -35402,12 +35382,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">UMUT CELLS -4-</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">D4</t>
+          <t xml:space="preserve">D3</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -35422,7 +35402,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt5ckqo-0</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
@@ -35434,7 +35414,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -35454,7 +35434,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">D4</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -35469,7 +35449,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtt5ckqo-0</t>
         </is>
       </c>
     </row>
@@ -35481,7 +35461,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -35501,7 +35481,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">A1</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -35516,7 +35496,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
@@ -35548,7 +35528,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">A2</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -35563,7 +35543,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
@@ -35595,7 +35575,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">A3</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -35610,7 +35590,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
@@ -35622,7 +35602,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -35642,7 +35622,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">A4</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -35657,7 +35637,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
       </c>
     </row>
@@ -35669,7 +35649,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -35689,7 +35669,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">A1</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -35704,7 +35684,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
@@ -35716,7 +35696,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -35736,7 +35716,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">A2</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -35751,7 +35731,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
@@ -35763,7 +35743,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -35783,7 +35763,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">A1</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -35798,7 +35778,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
@@ -35830,7 +35810,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">A2</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -35845,7 +35825,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
@@ -35877,7 +35857,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">A3</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -35892,7 +35872,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
@@ -35971,7 +35951,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">A4</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -35986,7 +35966,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
       </c>
     </row>
@@ -36018,7 +35998,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">A3</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -36033,7 +36013,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
@@ -36045,7 +36025,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -36065,7 +36045,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">A2</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -36080,7 +36060,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
@@ -36092,7 +36072,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -36112,7 +36092,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">A1</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -36127,7 +36107,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
@@ -36159,7 +36139,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">A4</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -36174,7 +36154,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
       </c>
     </row>
@@ -36206,7 +36186,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">A3</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -36221,7 +36201,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
@@ -36253,7 +36233,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">A4</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -36268,7 +36248,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
       </c>
     </row>
@@ -36300,20 +36280,67 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
+          <t xml:space="preserve">A3</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown device</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unnamed box</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
           <t xml:space="preserve">A4</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t xml:space="preserve">unknown device</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t xml:space="preserve">thaw</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="J37" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
@@ -36594,10 +36621,10 @@
         <v>81</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Edit Common Box #1
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -34677,7 +34677,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -34724,7 +34724,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -34771,7 +34771,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -34818,7 +34818,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -34959,7 +34959,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -35429,7 +35429,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -35476,7 +35476,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -35523,7 +35523,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -35570,7 +35570,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -35617,7 +35617,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -35664,7 +35664,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -35711,7 +35711,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -35758,7 +35758,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -35805,7 +35805,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -35852,7 +35852,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -35899,7 +35899,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -35946,7 +35946,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -35993,7 +35993,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -36040,7 +36040,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -36087,7 +36087,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -36134,7 +36134,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -36181,7 +36181,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -36228,7 +36228,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -36275,7 +36275,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -36322,7 +36322,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -36603,7 +36603,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unnamed box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">

</xml_diff>